<commit_message>
Add symptom CSV file and update master_table
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\tool-fcost\example\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\ExcelAutoTool\masters\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4045" uniqueCount="2126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4177" uniqueCount="2179">
   <si>
     <t>DSGY-F704JBKZ</t>
   </si>
@@ -6096,7 +6096,451 @@
     <t>*</t>
   </si>
   <si>
-    <t>garis / line</t>
+    <t>BLANK</t>
+  </si>
+  <si>
+    <t>X ADA GAMBAR</t>
+  </si>
+  <si>
+    <t>MATI</t>
+  </si>
+  <si>
+    <t>HANYA SUARA SAJA</t>
+  </si>
+  <si>
+    <t>TIDAK BISA HIDUP</t>
+  </si>
+  <si>
+    <t>TIDAK BS HIDUP</t>
+  </si>
+  <si>
+    <t>LOGO</t>
+  </si>
+  <si>
+    <t>HDMI</t>
+  </si>
+  <si>
+    <t>SIARAN</t>
+  </si>
+  <si>
+    <t>CHANNEL</t>
+  </si>
+  <si>
+    <t>Diff Month</t>
+  </si>
+  <si>
+    <t>0-12</t>
+  </si>
+  <si>
+    <t>&lt; 1 Year</t>
+  </si>
+  <si>
+    <t>13-24</t>
+  </si>
+  <si>
+    <t>1 - 2 Years</t>
+  </si>
+  <si>
+    <t>25-36</t>
+  </si>
+  <si>
+    <t>2 - 3 Years</t>
+  </si>
+  <si>
+    <t>=&gt;37</t>
+  </si>
+  <si>
+    <t>&gt; 3 Years</t>
+  </si>
+  <si>
+    <t>Panel Usage</t>
+  </si>
+  <si>
+    <t>init</t>
+  </si>
+  <si>
+    <t>branch</t>
+  </si>
+  <si>
+    <t>CIDENG</t>
+  </si>
+  <si>
+    <t>JAKARTA</t>
+  </si>
+  <si>
+    <t>PULOGADUNG</t>
+  </si>
+  <si>
+    <t>JAKARTA SELATAN</t>
+  </si>
+  <si>
+    <t>action</t>
+  </si>
+  <si>
+    <t>replace_power_unit</t>
+  </si>
+  <si>
+    <t>replace_panel</t>
+  </si>
+  <si>
+    <t>replace_main_unit</t>
+  </si>
+  <si>
+    <t>Remote Control</t>
+  </si>
+  <si>
+    <t>replace_remote_control</t>
+  </si>
+  <si>
+    <t>repair_comment</t>
+  </si>
+  <si>
+    <t>*bawa</t>
+  </si>
+  <si>
+    <t>ZY</t>
+  </si>
+  <si>
+    <t>*ext</t>
+  </si>
+  <si>
+    <t>external</t>
+  </si>
+  <si>
+    <t>UPGRADE</t>
+  </si>
+  <si>
+    <t>upgrade</t>
+  </si>
+  <si>
+    <t>*factor</t>
+  </si>
+  <si>
+    <t>factory_reset</t>
+  </si>
+  <si>
+    <t>JELAS</t>
+  </si>
+  <si>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>BATAL</t>
+  </si>
+  <si>
+    <t>cancel</t>
+  </si>
+  <si>
+    <t>Repair Action</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Defect</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Repair LVDS</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Reinsert Speaker</t>
+  </si>
+  <si>
+    <t>Subtitusi</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Replace Panel - Before Change</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>Non Defect</t>
+  </si>
+  <si>
+    <t>Setting</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
+    <t>Signal</t>
+  </si>
+  <si>
+    <t>Replace Panel</t>
+  </si>
+  <si>
+    <t>Panel</t>
+  </si>
+  <si>
+    <t>Repair Panel</t>
+  </si>
+  <si>
+    <t>Replace Main Unit</t>
+  </si>
+  <si>
+    <t>Main Unit</t>
+  </si>
+  <si>
+    <t>Repair Main Unit</t>
+  </si>
+  <si>
+    <t>Replace Power Unit</t>
+  </si>
+  <si>
+    <t>Power Unit</t>
+  </si>
+  <si>
+    <t>Replace TCON</t>
+  </si>
+  <si>
+    <t>Repair Power Unit</t>
+  </si>
+  <si>
+    <t>Factory Reset</t>
+  </si>
+  <si>
+    <t>Software</t>
+  </si>
+  <si>
+    <t>Upgrade</t>
+  </si>
+  <si>
+    <t>Reinsert LVDS</t>
+  </si>
+  <si>
+    <t>Repair IR Unit</t>
+  </si>
+  <si>
+    <t>Repair LED BAR</t>
+  </si>
+  <si>
+    <t>Repair Speaker</t>
+  </si>
+  <si>
+    <t>Replace Speaker</t>
+  </si>
+  <si>
+    <t>Replace Led Bar</t>
+  </si>
+  <si>
+    <t>Replace LVDS</t>
+  </si>
+  <si>
+    <t>Replace IR Unit</t>
+  </si>
+  <si>
+    <t>Replace Wifi Unit</t>
+  </si>
+  <si>
+    <t>Repair TCON</t>
+  </si>
+  <si>
+    <t>Repair Wifi Unit</t>
+  </si>
+  <si>
+    <t>Reinsert Wifi Unit</t>
+  </si>
+  <si>
+    <t>Reinsert Cabinet</t>
+  </si>
+  <si>
+    <t>Reinsert Socket</t>
+  </si>
+  <si>
+    <t>Replace Remote</t>
+  </si>
+  <si>
+    <t>Repair Remote</t>
+  </si>
+  <si>
+    <t>Replace Tape</t>
+  </si>
+  <si>
+    <t>Verified OK</t>
+  </si>
+  <si>
+    <t>Cancel</t>
+  </si>
+  <si>
+    <t>External</t>
+  </si>
+  <si>
+    <t>Before Improve - Remote</t>
+  </si>
+  <si>
+    <t>Before Improve</t>
+  </si>
+  <si>
+    <t>TOTAL_OFF</t>
+  </si>
+  <si>
+    <t>LINE</t>
+  </si>
+  <si>
+    <t>STANDBY</t>
+  </si>
+  <si>
+    <t>LOGO_FREEZE</t>
+  </si>
+  <si>
+    <t>HDMI_NG</t>
+  </si>
+  <si>
+    <t>NO_CHANNEL</t>
+  </si>
+  <si>
+    <t>*garis*</t>
+  </si>
+  <si>
+    <t>*line*</t>
+  </si>
+  <si>
+    <t>*GOYANG*</t>
+  </si>
+  <si>
+    <t>DISPLAY NG</t>
+  </si>
+  <si>
+    <t>*BAYANG*</t>
+  </si>
+  <si>
+    <t>BLUR</t>
+  </si>
+  <si>
+    <t>DOT</t>
+  </si>
+  <si>
+    <t>*DOT*</t>
+  </si>
+  <si>
+    <t>*BERGERAK*</t>
+  </si>
+  <si>
+    <t>*SETENGAH*</t>
+  </si>
+  <si>
+    <t>HALF</t>
+  </si>
+  <si>
+    <t>*RUSAK PANEL*</t>
+  </si>
+  <si>
+    <t>BROKEN</t>
+  </si>
+  <si>
+    <t>*BURAM*</t>
+  </si>
+  <si>
+    <t>MURA</t>
+  </si>
+  <si>
+    <t>*PIXEL*</t>
+  </si>
+  <si>
+    <t>*GAMBAR TDK KELUAR*</t>
+  </si>
+  <si>
+    <t>*BLANK*</t>
+  </si>
+  <si>
+    <t>NO_PICTURE</t>
+  </si>
+  <si>
+    <t>TDK ADA GAMABAR</t>
+  </si>
+  <si>
+    <t>TIDAK AD AGAMBAR</t>
+  </si>
+  <si>
+    <t>TIDAK AD GAMBAR</t>
+  </si>
+  <si>
+    <t>*TIDAK BISA HIDUP*</t>
+  </si>
+  <si>
+    <t>*STANDBY*</t>
+  </si>
+  <si>
+    <t>*STAND BY*</t>
+  </si>
+  <si>
+    <t>*STANBY*</t>
+  </si>
+  <si>
+    <t>*MATOT*</t>
+  </si>
+  <si>
+    <t>*MATOL*</t>
+  </si>
+  <si>
+    <t>LAYAR BLANK</t>
+  </si>
+  <si>
+    <t>*TDK ADA GAMBAR*</t>
+  </si>
+  <si>
+    <t>*TIDAK ADA GAMBAR*</t>
+  </si>
+  <si>
+    <t>ERROR</t>
+  </si>
+  <si>
+    <t>*NETFLIX*</t>
+  </si>
+  <si>
+    <t>*MATI*</t>
+  </si>
+  <si>
+    <t>SIGNAL</t>
+  </si>
+  <si>
+    <t>SINYAL</t>
+  </si>
+  <si>
+    <t>INDIKATOR</t>
+  </si>
+  <si>
+    <t>PROTECT</t>
+  </si>
+  <si>
+    <t>REMOT</t>
+  </si>
+  <si>
+    <t>SENSOR_NG</t>
+  </si>
+  <si>
+    <t>REMOTE</t>
+  </si>
+  <si>
+    <t>SENSOR</t>
+  </si>
+  <si>
+    <t>TIDAK ADA SUARA</t>
+  </si>
+  <si>
+    <t>CHANEL</t>
+  </si>
+  <si>
+    <t>SOUND_NG</t>
+  </si>
+  <si>
+    <t>TOMBOL</t>
+  </si>
+  <si>
+    <t>BUTTON_NG</t>
+  </si>
+  <si>
+    <t>EROR</t>
   </si>
   <si>
     <t>TIDAK ADA GAMBAR</t>
@@ -6105,313 +6549,28 @@
     <t>TDK ADA GAMBAR</t>
   </si>
   <si>
-    <t>BLANK</t>
-  </si>
-  <si>
-    <t>X ADA GAMBAR</t>
-  </si>
-  <si>
-    <t>MATI</t>
-  </si>
-  <si>
-    <t>HANYA SUARA SAJA</t>
-  </si>
-  <si>
-    <t>TIDAK BISA HIDUP</t>
-  </si>
-  <si>
-    <t>TIDAK BS HIDUP</t>
-  </si>
-  <si>
-    <t>STANDBY / STAND BY</t>
-  </si>
-  <si>
-    <t>LOGO</t>
-  </si>
-  <si>
-    <t>HDMI</t>
-  </si>
-  <si>
-    <t>SIARAN</t>
-  </si>
-  <si>
-    <t>SIGNAL / SINYAL</t>
-  </si>
-  <si>
-    <t>CHANNEL</t>
-  </si>
-  <si>
-    <t>Diff Month</t>
-  </si>
-  <si>
-    <t>0-12</t>
-  </si>
-  <si>
-    <t>&lt; 1 Year</t>
-  </si>
-  <si>
-    <t>13-24</t>
-  </si>
-  <si>
-    <t>1 - 2 Years</t>
-  </si>
-  <si>
-    <t>25-36</t>
-  </si>
-  <si>
-    <t>2 - 3 Years</t>
-  </si>
-  <si>
-    <t>=&gt;37</t>
-  </si>
-  <si>
-    <t>&gt; 3 Years</t>
-  </si>
-  <si>
-    <t>Panel Usage</t>
-  </si>
-  <si>
-    <t>init</t>
-  </si>
-  <si>
-    <t>branch</t>
-  </si>
-  <si>
-    <t>CIDENG</t>
-  </si>
-  <si>
-    <t>JAKARTA</t>
-  </si>
-  <si>
-    <t>PULOGADUNG</t>
-  </si>
-  <si>
-    <t>JAKARTA SELATAN</t>
-  </si>
-  <si>
-    <t>action</t>
-  </si>
-  <si>
-    <t>replace_power_unit</t>
-  </si>
-  <si>
-    <t>replace_panel</t>
-  </si>
-  <si>
-    <t>replace_main_unit</t>
-  </si>
-  <si>
-    <t>Remote Control</t>
-  </si>
-  <si>
-    <t>replace_remote_control</t>
-  </si>
-  <si>
-    <t>repair_comment</t>
-  </si>
-  <si>
-    <t>*bawa</t>
-  </si>
-  <si>
-    <t>ZY</t>
-  </si>
-  <si>
-    <t>*ext</t>
-  </si>
-  <si>
-    <t>external</t>
-  </si>
-  <si>
-    <t>UPGRADE</t>
-  </si>
-  <si>
-    <t>upgrade</t>
-  </si>
-  <si>
-    <t>*factor</t>
-  </si>
-  <si>
-    <t>factory_reset</t>
-  </si>
-  <si>
-    <t>JELAS</t>
-  </si>
-  <si>
-    <t>explanation</t>
-  </si>
-  <si>
-    <t>BATAL</t>
-  </si>
-  <si>
-    <t>cancel</t>
-  </si>
-  <si>
-    <t>Repair Action</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Defect</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Repair LVDS</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>Reinsert Speaker</t>
-  </si>
-  <si>
-    <t>Subtitusi</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Replace Panel - Before Change</t>
-  </si>
-  <si>
-    <t>User</t>
-  </si>
-  <si>
-    <t>Non Defect</t>
-  </si>
-  <si>
-    <t>Setting</t>
-  </si>
-  <si>
-    <t>Explanation</t>
-  </si>
-  <si>
-    <t>Signal</t>
-  </si>
-  <si>
-    <t>Replace Panel</t>
-  </si>
-  <si>
-    <t>Panel</t>
-  </si>
-  <si>
-    <t>Repair Panel</t>
-  </si>
-  <si>
-    <t>Replace Main Unit</t>
-  </si>
-  <si>
-    <t>Main Unit</t>
-  </si>
-  <si>
-    <t>Repair Main Unit</t>
-  </si>
-  <si>
-    <t>Replace Power Unit</t>
-  </si>
-  <si>
-    <t>Power Unit</t>
-  </si>
-  <si>
-    <t>Replace TCON</t>
-  </si>
-  <si>
-    <t>Repair Power Unit</t>
-  </si>
-  <si>
-    <t>Factory Reset</t>
-  </si>
-  <si>
-    <t>Software</t>
-  </si>
-  <si>
-    <t>Upgrade</t>
-  </si>
-  <si>
-    <t>Reinsert LVDS</t>
-  </si>
-  <si>
-    <t>Repair IR Unit</t>
-  </si>
-  <si>
-    <t>Repair LED BAR</t>
-  </si>
-  <si>
-    <t>Repair Speaker</t>
-  </si>
-  <si>
-    <t>Replace Speaker</t>
-  </si>
-  <si>
-    <t>Replace Led Bar</t>
-  </si>
-  <si>
-    <t>Replace LVDS</t>
-  </si>
-  <si>
-    <t>Replace IR Unit</t>
-  </si>
-  <si>
-    <t>Replace Wifi Unit</t>
-  </si>
-  <si>
-    <t>Repair TCON</t>
-  </si>
-  <si>
-    <t>Repair Wifi Unit</t>
-  </si>
-  <si>
-    <t>Reinsert Wifi Unit</t>
-  </si>
-  <si>
-    <t>Reinsert Cabinet</t>
-  </si>
-  <si>
-    <t>Reinsert Socket</t>
-  </si>
-  <si>
-    <t>Replace Remote</t>
-  </si>
-  <si>
-    <t>Repair Remote</t>
-  </si>
-  <si>
-    <t>Replace Tape</t>
-  </si>
-  <si>
-    <t>Verified OK</t>
-  </si>
-  <si>
-    <t>Cancel</t>
-  </si>
-  <si>
-    <t>External</t>
-  </si>
-  <si>
-    <t>Before Improve - Remote</t>
-  </si>
-  <si>
-    <t>Before Improve</t>
-  </si>
-  <si>
-    <t>TOTAL_OFF</t>
-  </si>
-  <si>
-    <t>LINE</t>
-  </si>
-  <si>
-    <t>STANDBY</t>
-  </si>
-  <si>
-    <t>LOGO_FREEZE</t>
-  </si>
-  <si>
-    <t>HDMI_NG</t>
-  </si>
-  <si>
-    <t>NO_CHANNEL</t>
+    <t>TIDAK ADA SIARAN</t>
+  </si>
+  <si>
+    <t>DOMINAN</t>
+  </si>
+  <si>
+    <t>MERAH</t>
+  </si>
+  <si>
+    <t>PUTIH</t>
+  </si>
+  <si>
+    <t>SEBELAH</t>
+  </si>
+  <si>
+    <t>NO DISPLAY</t>
+  </si>
+  <si>
+    <t>PECAH</t>
+  </si>
+  <si>
+    <t>RC_NG</t>
   </si>
 </sst>
 </file>
@@ -6421,7 +6580,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="###,###,###,###"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6520,6 +6679,10 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -6609,7 +6772,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -6706,6 +6869,8 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -29923,12 +30088,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="49.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -29950,7 +30116,7 @@
         <v>2019</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>2120</v>
+        <v>2115</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -29958,10 +30124,10 @@
         <v>1853</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>2020</v>
+        <v>2121</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>2121</v>
+        <v>2116</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -29969,10 +30135,10 @@
         <v>1853</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>2021</v>
+        <v>2122</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>2023</v>
+        <v>2116</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -29980,21 +30146,21 @@
         <v>1853</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>2022</v>
+        <v>2140</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>2023</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="23" t="s">
         <v>1853</v>
       </c>
-      <c r="B6" s="23" t="s">
-        <v>2023</v>
+      <c r="B6" t="s">
+        <v>2170</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>2023</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -30002,10 +30168,10 @@
         <v>1853</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>2024</v>
+        <v>2141</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>2023</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -30013,10 +30179,10 @@
         <v>1853</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>2025</v>
+        <v>2142</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>2023</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -30024,113 +30190,598 @@
         <v>1853</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>2026</v>
+        <v>2169</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>2023</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>2029</v>
+        <v>2171</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>2122</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>2120</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>2027</v>
+        <v>2021</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>2120</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>2028</v>
+        <v>2176</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>2120</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>2030</v>
+        <v>2022</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>2123</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>2031</v>
+        <v>2023</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>2124</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>2032</v>
+        <v>2123</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>2125</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>2033</v>
+        <v>2172</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>2125</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="23" t="s">
-        <v>1871</v>
+        <v>1853</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>2034</v>
+        <v>2173</v>
       </c>
       <c r="C18" s="23" t="s">
+        <v>2124</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>2174</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>2124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B20" s="23" t="s">
         <v>2125</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>2126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2126</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>2126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B22" s="23" t="s">
+        <v>2128</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B23" s="23" t="s">
+        <v>2136</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>2143</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>2129</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>2124</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>2130</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>2175</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>2132</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>2133</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B29" s="23" t="s">
+        <v>2177</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>2133</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>2134</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>2135</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="23" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B32" s="23" t="s">
+        <v>2144</v>
+      </c>
+      <c r="C32" s="23" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B33" s="23" t="s">
+        <v>2146</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B34" s="23" t="s">
+        <v>2145</v>
+      </c>
+      <c r="C34" s="23" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B35" s="23" t="s">
+        <v>2154</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B36" s="23" t="s">
+        <v>2147</v>
+      </c>
+      <c r="C36" s="23" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B37" s="23" t="s">
+        <v>2148</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B38" s="23" t="s">
+        <v>2149</v>
+      </c>
+      <c r="C38" s="23" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B39" s="23" t="s">
+        <v>2024</v>
+      </c>
+      <c r="C39" s="23" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B40" s="23" t="s">
+        <v>2025</v>
+      </c>
+      <c r="C40" s="23" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B41" s="23" t="s">
+        <v>2026</v>
+      </c>
+      <c r="C41" s="23" t="s">
+        <v>2118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B42" s="23" t="s">
+        <v>2027</v>
+      </c>
+      <c r="C42" s="23" t="s">
+        <v>2119</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B43" s="23" t="s">
+        <v>2028</v>
+      </c>
+      <c r="C43" s="23" t="s">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B44" s="23" t="s">
+        <v>2156</v>
+      </c>
+      <c r="C44" s="23" t="s">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C45" s="23" t="s">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B46" s="23" t="s">
+        <v>2029</v>
+      </c>
+      <c r="C46" s="23" t="s">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B47" t="s">
+        <v>2164</v>
+      </c>
+      <c r="C47" s="23" t="s">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B48" s="23" t="s">
+        <v>2150</v>
+      </c>
+      <c r="C48" s="42" t="s">
+        <v>2139</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B49" s="23" t="s">
+        <v>2151</v>
+      </c>
+      <c r="C49" s="42" t="s">
+        <v>2139</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B50" s="23" t="s">
+        <v>2138</v>
+      </c>
+      <c r="C50" s="42" t="s">
+        <v>2139</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B51" s="23" t="s">
+        <v>2153</v>
+      </c>
+      <c r="C51" s="42" t="s">
+        <v>2152</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B52" s="23" t="s">
+        <v>2168</v>
+      </c>
+      <c r="C52" s="42" t="s">
+        <v>2152</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B53" s="23" t="s">
+        <v>2152</v>
+      </c>
+      <c r="C53" s="42" t="s">
+        <v>2152</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B54" s="23" t="s">
+        <v>2157</v>
+      </c>
+      <c r="C54" s="42" t="s">
+        <v>2158</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B55" s="23" t="s">
+        <v>2159</v>
+      </c>
+      <c r="C55" s="42" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B56" s="23" t="s">
+        <v>2161</v>
+      </c>
+      <c r="C56" s="42" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B57" s="23" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C57" s="42" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B58" s="23" t="s">
+        <v>2163</v>
+      </c>
+      <c r="C58" s="42" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B59" s="23" t="s">
+        <v>2166</v>
+      </c>
+      <c r="C59" s="42" t="s">
+        <v>2167</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="43" t="s">
+        <v>1870</v>
+      </c>
+      <c r="B60" s="23" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C60" s="42" t="s">
+        <v>2178</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="43" t="s">
+        <v>1870</v>
+      </c>
+      <c r="B61" s="23" t="s">
+        <v>2161</v>
+      </c>
+      <c r="C61" s="42" t="s">
+        <v>2178</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="23" t="s">
+        <v>1878</v>
+      </c>
+      <c r="B62" s="23" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C62" s="23" t="s">
+        <v>2139</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -30144,42 +30795,42 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="25" t="s">
-        <v>2035</v>
+        <v>2030</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>2044</v>
+        <v>2039</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="26" t="s">
-        <v>2036</v>
+        <v>2031</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>2037</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="26" t="s">
-        <v>2038</v>
+        <v>2033</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>2039</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="26" t="s">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>2041</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="27" t="s">
-        <v>2042</v>
+        <v>2037</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>2043</v>
+        <v>2038</v>
       </c>
     </row>
   </sheetData>
@@ -30198,34 +30849,34 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="25" t="s">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>2046</v>
+        <v>2041</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="26" t="s">
-        <v>2047</v>
+        <v>2042</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>2048</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="26" t="s">
-        <v>2049</v>
+        <v>2044</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>2048</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="26" t="s">
-        <v>2050</v>
+        <v>2045</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>2048</v>
+        <v>2043</v>
       </c>
     </row>
   </sheetData>
@@ -30249,28 +30900,28 @@
         <v>1841</v>
       </c>
       <c r="B1" s="28" t="s">
-        <v>2057</v>
+        <v>2052</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>2051</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="31" customFormat="1">
       <c r="A2" s="36"/>
       <c r="B2" s="29" t="s">
-        <v>2060</v>
+        <v>2055</v>
       </c>
       <c r="C2" s="33" t="s">
-        <v>2061</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="31" customFormat="1">
       <c r="A3" s="36"/>
       <c r="B3" s="32" t="s">
-        <v>2068</v>
+        <v>2063</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>2069</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -30281,7 +30932,7 @@
         <v>2019</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>2052</v>
+        <v>2047</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -30292,7 +30943,7 @@
         <v>2019</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>2053</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -30303,63 +30954,63 @@
         <v>2019</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>2054</v>
+        <v>2049</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="32" t="s">
-        <v>2055</v>
+        <v>2050</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>2019</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>2056</v>
+        <v>2051</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="32"/>
       <c r="B8" s="32" t="s">
-        <v>2058</v>
+        <v>2053</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>2059</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="32"/>
       <c r="B9" s="32" t="s">
-        <v>2059</v>
+        <v>2054</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>2059</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="32"/>
       <c r="B10" s="32" t="s">
-        <v>2062</v>
+        <v>2057</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>2063</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="32"/>
       <c r="B11" s="32" t="s">
-        <v>2064</v>
+        <v>2059</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>2065</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="32"/>
       <c r="B12" s="32" t="s">
-        <v>2066</v>
+        <v>2061</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>2067</v>
+        <v>2062</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -30388,27 +31039,27 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="37" t="s">
-        <v>2070</v>
+        <v>2065</v>
       </c>
       <c r="B1" s="37" t="s">
-        <v>2071</v>
+        <v>2066</v>
       </c>
       <c r="C1" s="37" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="D1" s="37" t="s">
-        <v>2073</v>
+        <v>2068</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="39" t="s">
-        <v>2074</v>
+        <v>2069</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C2" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D2" s="40">
         <v>0</v>
@@ -30416,13 +31067,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="39" t="s">
-        <v>2076</v>
+        <v>2071</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C3" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D3" s="40">
         <v>0</v>
@@ -30430,13 +31081,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="41" t="s">
-        <v>2077</v>
+        <v>2072</v>
       </c>
       <c r="B4" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C4" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D4" s="40">
         <v>0</v>
@@ -30444,13 +31095,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="41" t="s">
-        <v>2079</v>
+        <v>2074</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D5" s="40">
         <v>0</v>
@@ -30458,13 +31109,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="39" t="s">
-        <v>2059</v>
+        <v>2054</v>
       </c>
       <c r="B6" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D6" s="40">
         <v>0</v>
@@ -30472,13 +31123,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="41" t="s">
-        <v>2079</v>
+        <v>2074</v>
       </c>
       <c r="B7" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D7" s="40">
         <v>0</v>
@@ -30486,13 +31137,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="39" t="s">
-        <v>2059</v>
+        <v>2054</v>
       </c>
       <c r="B8" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D8" s="40">
         <v>0</v>
@@ -30500,13 +31151,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="40" t="s">
-        <v>2080</v>
+        <v>2075</v>
       </c>
       <c r="B9" s="39" t="s">
-        <v>2081</v>
+        <v>2076</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>2080</v>
+        <v>2075</v>
       </c>
       <c r="D9" s="40">
         <v>11</v>
@@ -30514,13 +31165,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="40" t="s">
-        <v>2082</v>
+        <v>2077</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>2081</v>
+        <v>2076</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>2082</v>
+        <v>2077</v>
       </c>
       <c r="D10" s="40">
         <v>12</v>
@@ -30528,13 +31179,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="40" t="s">
-        <v>2083</v>
+        <v>2078</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>2081</v>
+        <v>2076</v>
       </c>
       <c r="C11" s="40" t="s">
-        <v>2083</v>
+        <v>2078</v>
       </c>
       <c r="D11" s="40">
         <v>13</v>
@@ -30542,13 +31193,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="40" t="s">
-        <v>2084</v>
+        <v>2079</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>2081</v>
+        <v>2076</v>
       </c>
       <c r="C12" s="40" t="s">
-        <v>2084</v>
+        <v>2079</v>
       </c>
       <c r="D12" s="40">
         <v>14</v>
@@ -30556,13 +31207,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="39" t="s">
-        <v>2085</v>
+        <v>2080</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>2086</v>
+        <v>2081</v>
       </c>
       <c r="D13" s="40">
         <v>20</v>
@@ -30570,13 +31221,13 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="39" t="s">
-        <v>2087</v>
+        <v>2082</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C14" s="40" t="s">
-        <v>2086</v>
+        <v>2081</v>
       </c>
       <c r="D14" s="40">
         <v>21</v>
@@ -30584,13 +31235,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="39" t="s">
-        <v>2088</v>
+        <v>2083</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>2089</v>
+        <v>2084</v>
       </c>
       <c r="D15" s="40">
         <v>30</v>
@@ -30598,13 +31249,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="39" t="s">
-        <v>2090</v>
+        <v>2085</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C16" s="40" t="s">
-        <v>2089</v>
+        <v>2084</v>
       </c>
       <c r="D16" s="40">
         <v>31</v>
@@ -30612,13 +31263,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="41" t="s">
-        <v>2091</v>
+        <v>2086</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>2092</v>
+        <v>2087</v>
       </c>
       <c r="D17" s="40">
         <v>40</v>
@@ -30626,13 +31277,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="40" t="s">
-        <v>2093</v>
+        <v>2088</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C18" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D18" s="40">
         <v>42</v>
@@ -30640,13 +31291,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="41" t="s">
-        <v>2094</v>
+        <v>2089</v>
       </c>
       <c r="B19" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C19" s="40" t="s">
-        <v>2092</v>
+        <v>2087</v>
       </c>
       <c r="D19" s="40">
         <v>41</v>
@@ -30654,13 +31305,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="39" t="s">
-        <v>2095</v>
+        <v>2090</v>
       </c>
       <c r="B20" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C20" s="39" t="s">
-        <v>2096</v>
+        <v>2091</v>
       </c>
       <c r="D20" s="40">
         <v>50</v>
@@ -30668,13 +31319,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="39" t="s">
-        <v>2097</v>
+        <v>2092</v>
       </c>
       <c r="B21" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C21" s="39" t="s">
-        <v>2096</v>
+        <v>2091</v>
       </c>
       <c r="D21" s="40">
         <v>51</v>
@@ -30682,13 +31333,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="41" t="s">
-        <v>2098</v>
+        <v>2093</v>
       </c>
       <c r="B22" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D22" s="40">
         <v>60</v>
@@ -30696,13 +31347,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="40" t="s">
-        <v>2099</v>
+        <v>2094</v>
       </c>
       <c r="B23" s="40" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D23" s="40">
         <v>61</v>
@@ -30710,13 +31361,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="39" t="s">
-        <v>2100</v>
+        <v>2095</v>
       </c>
       <c r="B24" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D24" s="40">
         <v>62</v>
@@ -30724,13 +31375,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="41" t="s">
-        <v>2101</v>
+        <v>2096</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C25" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D25" s="40">
         <v>63</v>
@@ -30738,13 +31389,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="40" t="s">
-        <v>2102</v>
+        <v>2097</v>
       </c>
       <c r="B26" s="40" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C26" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D26" s="40">
         <v>66</v>
@@ -30752,13 +31403,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="40" t="s">
-        <v>2103</v>
+        <v>2098</v>
       </c>
       <c r="B27" s="40" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C27" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D27" s="40">
         <v>67</v>
@@ -30766,13 +31417,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="39" t="s">
-        <v>2104</v>
+        <v>2099</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D28" s="40">
         <v>68</v>
@@ -30780,13 +31431,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="39" t="s">
-        <v>2105</v>
+        <v>2100</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C29" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D29" s="40">
         <v>69</v>
@@ -30794,13 +31445,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="40" t="s">
-        <v>2106</v>
+        <v>2101</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C30" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D30" s="40">
         <v>70</v>
@@ -30808,13 +31459,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="40" t="s">
-        <v>2107</v>
+        <v>2102</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C31" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D31" s="40">
         <v>71</v>
@@ -30822,13 +31473,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="40" t="s">
-        <v>2108</v>
+        <v>2103</v>
       </c>
       <c r="B32" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C32" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D32" s="40">
         <v>72</v>
@@ -30836,13 +31487,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="40" t="s">
-        <v>2109</v>
+        <v>2104</v>
       </c>
       <c r="B33" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C33" s="40" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D33" s="40">
         <v>73</v>
@@ -30850,13 +31501,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="39" t="s">
-        <v>2110</v>
+        <v>2105</v>
       </c>
       <c r="B34" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C34" s="39" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D34" s="40">
         <v>74</v>
@@ -30864,13 +31515,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="39" t="s">
-        <v>2111</v>
+        <v>2106</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C35" s="39" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D35" s="40">
         <v>76</v>
@@ -30878,13 +31529,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="39" t="s">
-        <v>2112</v>
+        <v>2107</v>
       </c>
       <c r="B36" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C36" s="39" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D36" s="40">
         <v>75</v>
@@ -30892,13 +31543,13 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="39" t="s">
-        <v>2113</v>
+        <v>2108</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C37" s="39" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D37" s="40">
         <v>77</v>
@@ -30906,13 +31557,13 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="39" t="s">
-        <v>2114</v>
+        <v>2109</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="C38" s="39" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="D38" s="40">
         <v>78</v>
@@ -30920,72 +31571,72 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="39" t="s">
-        <v>2115</v>
+        <v>2110</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C39" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D39" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="39" t="s">
-        <v>2116</v>
+        <v>2111</v>
       </c>
       <c r="B40" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C40" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D40" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="39" t="s">
-        <v>2117</v>
+        <v>2112</v>
       </c>
       <c r="B41" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C41" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D41" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="40" t="s">
-        <v>2118</v>
+        <v>2113</v>
       </c>
       <c r="B42" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C42" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D42" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="40" t="s">
-        <v>2119</v>
+        <v>2114</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="C43" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D43" s="40" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: capture current workspace changes
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\ExcelAuto\ExcelAutoTool_1.1\masters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\tool-fcost\masters\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4407" uniqueCount="2276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4412" uniqueCount="2262">
   <si>
     <t>part_used</t>
   </si>
@@ -6753,109 +6753,67 @@
     <t>DEFECT</t>
   </si>
   <si>
-    <t>REINSERT SPEAKER</t>
-  </si>
-  <si>
     <t>SUBTITUSI</t>
   </si>
   <si>
-    <t>REPLACE PANEL - BEFORE CHANGE</t>
-  </si>
-  <si>
-    <t>NON DEFECT</t>
-  </si>
-  <si>
     <t>SIGNAL</t>
   </si>
   <si>
-    <t>REPLACE PANEL</t>
-  </si>
-  <si>
-    <t>REPAIR PANEL</t>
-  </si>
-  <si>
-    <t>REPLACE MAIN UNIT</t>
-  </si>
-  <si>
-    <t>MAIN UNIT</t>
-  </si>
-  <si>
-    <t>REPAIR MAIN UNIT</t>
-  </si>
-  <si>
-    <t>REPLACE POWER UNIT</t>
-  </si>
-  <si>
-    <t>POWER UNIT</t>
-  </si>
-  <si>
-    <t>REPLACE TCON</t>
-  </si>
-  <si>
-    <t>REPAIR POWER UNIT</t>
-  </si>
-  <si>
-    <t>FACTORY RESET</t>
-  </si>
-  <si>
-    <t>REINSERT LVDS</t>
-  </si>
-  <si>
-    <t>REPAIR IR UNIT</t>
-  </si>
-  <si>
-    <t>REPAIR LED BAR</t>
-  </si>
-  <si>
-    <t>REPAIR SPEAKER</t>
-  </si>
-  <si>
-    <t>REPLACE SPEAKER</t>
-  </si>
-  <si>
-    <t>REPLACE LED BAR</t>
-  </si>
-  <si>
-    <t>REPLACE LVDS</t>
-  </si>
-  <si>
-    <t>REPLACE IR UNIT</t>
-  </si>
-  <si>
-    <t>REPLACE WIFI UNIT</t>
-  </si>
-  <si>
-    <t>REPAIR TCON</t>
-  </si>
-  <si>
-    <t>REPAIR WIFI UNIT</t>
-  </si>
-  <si>
-    <t>REINSERT WIFI UNIT</t>
-  </si>
-  <si>
-    <t>REINSERT CABINET</t>
-  </si>
-  <si>
-    <t>REINSERT SOCKET</t>
-  </si>
-  <si>
-    <t>REPLACE REMOTE</t>
-  </si>
-  <si>
-    <t>REPLACE TAPE</t>
-  </si>
-  <si>
-    <t>VERIFIED OK</t>
-  </si>
-  <si>
-    <t>BEFORE IMPROVE - REMOTE</t>
-  </si>
-  <si>
-    <t>BEFORE IMPROVE</t>
-  </si>
-  <si>
     <t>SOFWARE</t>
+  </si>
+  <si>
+    <t>BEFORE_IMPROVE</t>
+  </si>
+  <si>
+    <t>NON_DEFECT</t>
+  </si>
+  <si>
+    <t>REINSERT_SOCKET</t>
+  </si>
+  <si>
+    <t>REINSERT_SPEAKER</t>
+  </si>
+  <si>
+    <t>REINSERT_WIFI_UNIT</t>
+  </si>
+  <si>
+    <t>REPAIR_IR_UNIT</t>
+  </si>
+  <si>
+    <t>REPAIR_LED_BAR</t>
+  </si>
+  <si>
+    <t>REPAIR_LVDS</t>
+  </si>
+  <si>
+    <t>REPAIR_PANEL</t>
+  </si>
+  <si>
+    <t>REPAIR_SPEAKER</t>
+  </si>
+  <si>
+    <t>REPAIR_TCON</t>
+  </si>
+  <si>
+    <t>REPAIR_WIFI_UNIT</t>
+  </si>
+  <si>
+    <t>REPLACE_TAPE</t>
+  </si>
+  <si>
+    <t>REPLACE_WIFI_UNIT</t>
+  </si>
+  <si>
+    <t>VERIFIED_OK</t>
+  </si>
+  <si>
+    <t>BEFORE_IMPROVE_REMOTE</t>
+  </si>
+  <si>
+    <t>REPLACE_PANEL_BEFORE_CHANGE</t>
+  </si>
+  <si>
+    <t>CEK NORMAL</t>
   </si>
 </sst>
 </file>
@@ -31459,7 +31417,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" style="27" bestFit="1" customWidth="1"/>
@@ -31499,62 +31457,62 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="26" t="s">
-        <v>1428</v>
-      </c>
+      <c r="A4" s="31"/>
       <c r="B4" s="26" t="s">
-        <v>2110</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>2149</v>
+        <v>2261</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>2169</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="26" t="s">
-        <v>989</v>
+        <v>1428</v>
       </c>
       <c r="B5" s="26" t="s">
         <v>2110</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>2150</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="26" t="s">
-        <v>459</v>
+        <v>989</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>2110</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>2151</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="26" t="s">
-        <v>1659</v>
+        <v>459</v>
       </c>
       <c r="B7" s="26" t="s">
         <v>2110</v>
       </c>
-      <c r="C7" s="38" t="s">
+      <c r="C7" s="26" t="s">
+        <v>2151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="26" t="s">
+        <v>1659</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>2110</v>
+      </c>
+      <c r="C8" s="38" t="s">
         <v>2165</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="26"/>
-      <c r="B8" s="26" t="s">
-        <v>2152</v>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>2111</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="26"/>
       <c r="B9" s="26" t="s">
-        <v>2111</v>
+        <v>2152</v>
       </c>
       <c r="C9" s="26" t="s">
         <v>2111</v>
@@ -31563,166 +31521,166 @@
     <row r="10" spans="1:3">
       <c r="A10" s="26"/>
       <c r="B10" s="26" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="26"/>
       <c r="B11" s="26" t="s">
-        <v>2153</v>
+        <v>2112</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>2154</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="26"/>
       <c r="B12" s="26" t="s">
-        <v>2113</v>
+        <v>2153</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>2155</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="26"/>
       <c r="B13" s="26" t="s">
-        <v>2156</v>
-      </c>
-      <c r="C13" s="38" t="s">
-        <v>2157</v>
+        <v>2113</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>2155</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="26"/>
       <c r="B14" s="26" t="s">
+        <v>2156</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>2157</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="26"/>
+      <c r="B15" s="26" t="s">
         <v>2158</v>
       </c>
-      <c r="C14" s="38" t="s">
+      <c r="C15" s="38" t="s">
         <v>2147</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="26" t="s">
+    <row r="16" spans="1:3">
+      <c r="A16" s="26" t="s">
         <v>1397</v>
-      </c>
-      <c r="B15" s="38" t="s">
-        <v>2110</v>
-      </c>
-      <c r="C15" s="38" t="s">
-        <v>2159</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="39" t="s">
-        <v>214</v>
       </c>
       <c r="B16" s="38" t="s">
         <v>2110</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>2160</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="39" t="s">
-        <v>109</v>
+        <v>214</v>
       </c>
       <c r="B17" s="38" t="s">
         <v>2110</v>
       </c>
       <c r="C17" s="38" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="38" t="s">
+        <v>2110</v>
+      </c>
+      <c r="C18" s="38" t="s">
         <v>2161</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26" t="s">
-        <v>2162</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>2112</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="26"/>
       <c r="B19" s="26" t="s">
-        <v>2163</v>
+        <v>2162</v>
       </c>
       <c r="C19" s="38" t="s">
-        <v>2164</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="26"/>
       <c r="B20" s="26" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
       <c r="C20" s="38" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="26"/>
       <c r="B21" s="26" t="s">
-        <v>2167</v>
+        <v>2166</v>
       </c>
       <c r="C21" s="38" t="s">
-        <v>2111</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="26"/>
       <c r="B22" s="26" t="s">
-        <v>2168</v>
+        <v>2167</v>
       </c>
       <c r="C22" s="38" t="s">
-        <v>2169</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="26"/>
       <c r="B23" s="26" t="s">
-        <v>2170</v>
+        <v>2168</v>
       </c>
       <c r="C23" s="38" t="s">
-        <v>2147</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="26"/>
       <c r="B24" s="26" t="s">
-        <v>2171</v>
+        <v>2170</v>
       </c>
       <c r="C24" s="38" t="s">
-        <v>2161</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="26"/>
-      <c r="B25" s="40" t="s">
-        <v>2157</v>
+      <c r="B25" s="26" t="s">
+        <v>2171</v>
       </c>
       <c r="C25" s="38" t="s">
-        <v>2157</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="26"/>
-      <c r="B26" s="41" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C26" s="26" t="s">
-        <v>2111</v>
+      <c r="B26" s="40" t="s">
+        <v>2157</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>2157</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="26"/>
-      <c r="B27" s="40" t="s">
-        <v>2111</v>
+      <c r="B27" s="41" t="s">
+        <v>2172</v>
       </c>
       <c r="C27" s="26" t="s">
         <v>2111</v>
@@ -31731,7 +31689,7 @@
     <row r="28" spans="1:3">
       <c r="A28" s="26"/>
       <c r="B28" s="40" t="s">
-        <v>2173</v>
+        <v>2111</v>
       </c>
       <c r="C28" s="26" t="s">
         <v>2111</v>
@@ -31740,25 +31698,25 @@
     <row r="29" spans="1:3">
       <c r="A29" s="26"/>
       <c r="B29" s="40" t="s">
-        <v>2174</v>
-      </c>
-      <c r="C29" s="38" t="s">
+        <v>2173</v>
+      </c>
+      <c r="C29" s="26" t="s">
         <v>2111</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="26"/>
       <c r="B30" s="40" t="s">
-        <v>2112</v>
-      </c>
-      <c r="C30" s="26" t="s">
-        <v>2112</v>
+        <v>2174</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>2111</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="26"/>
-      <c r="B31" s="41" t="s">
-        <v>2162</v>
+      <c r="B31" s="40" t="s">
+        <v>2112</v>
       </c>
       <c r="C31" s="26" t="s">
         <v>2112</v>
@@ -31766,71 +31724,71 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="26"/>
-      <c r="B32" s="40" t="s">
-        <v>2175</v>
+      <c r="B32" s="41" t="s">
+        <v>2162</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>2154</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="26"/>
       <c r="B33" s="40" t="s">
-        <v>2113</v>
+        <v>2175</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>2155</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="26"/>
       <c r="B34" s="40" t="s">
-        <v>2166</v>
-      </c>
-      <c r="C34" s="38" t="s">
-        <v>2159</v>
+        <v>2113</v>
+      </c>
+      <c r="C34" s="26" t="s">
+        <v>2155</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="26"/>
       <c r="B35" s="40" t="s">
-        <v>2176</v>
+        <v>2166</v>
       </c>
       <c r="C35" s="38" t="s">
-        <v>2169</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="26"/>
       <c r="B36" s="40" t="s">
-        <v>2177</v>
+        <v>2176</v>
       </c>
       <c r="C36" s="38" t="s">
-        <v>2161</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="26"/>
       <c r="B37" s="40" t="s">
-        <v>2156</v>
+        <v>2177</v>
       </c>
       <c r="C37" s="38" t="s">
-        <v>2157</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="26"/>
       <c r="B38" s="40" t="s">
-        <v>2178</v>
+        <v>2156</v>
       </c>
       <c r="C38" s="38" t="s">
-        <v>2169</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="26"/>
       <c r="B39" s="40" t="s">
-        <v>2168</v>
+        <v>2178</v>
       </c>
       <c r="C39" s="38" t="s">
         <v>2169</v>
@@ -31839,43 +31797,43 @@
     <row r="40" spans="1:3">
       <c r="A40" s="26"/>
       <c r="B40" s="40" t="s">
-        <v>2179</v>
+        <v>2168</v>
       </c>
       <c r="C40" s="38" t="s">
-        <v>2148</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="26"/>
       <c r="B41" s="40" t="s">
-        <v>2180</v>
+        <v>2179</v>
       </c>
       <c r="C41" s="38" t="s">
-        <v>2161</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="26"/>
       <c r="B42" s="40" t="s">
-        <v>2181</v>
+        <v>2180</v>
       </c>
       <c r="C42" s="38" t="s">
-        <v>2159</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="26"/>
       <c r="B43" s="40" t="s">
-        <v>2182</v>
+        <v>2181</v>
       </c>
       <c r="C43" s="38" t="s">
-        <v>2161</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="26"/>
       <c r="B44" s="40" t="s">
-        <v>2183</v>
+        <v>2182</v>
       </c>
       <c r="C44" s="38" t="s">
         <v>2161</v>
@@ -31884,34 +31842,34 @@
     <row r="45" spans="1:3">
       <c r="A45" s="26"/>
       <c r="B45" s="40" t="s">
-        <v>2166</v>
+        <v>2183</v>
       </c>
       <c r="C45" s="38" t="s">
-        <v>2159</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="26"/>
       <c r="B46" s="40" t="s">
-        <v>2184</v>
+        <v>2166</v>
       </c>
       <c r="C46" s="38" t="s">
-        <v>2169</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="26"/>
       <c r="B47" s="40" t="s">
-        <v>2185</v>
+        <v>2184</v>
       </c>
       <c r="C47" s="38" t="s">
-        <v>2161</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="26"/>
-      <c r="B48" s="27" t="s">
-        <v>2186</v>
+      <c r="B48" s="40" t="s">
+        <v>2185</v>
       </c>
       <c r="C48" s="38" t="s">
         <v>2161</v>
@@ -31919,26 +31877,26 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="26"/>
-      <c r="B49" s="40" t="s">
-        <v>2187</v>
+      <c r="B49" s="27" t="s">
+        <v>2186</v>
       </c>
       <c r="C49" s="38" t="s">
-        <v>2169</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="26"/>
       <c r="B50" s="40" t="s">
-        <v>2188</v>
+        <v>2187</v>
       </c>
       <c r="C50" s="38" t="s">
-        <v>2157</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="26"/>
       <c r="B51" s="40" t="s">
-        <v>2189</v>
+        <v>2188</v>
       </c>
       <c r="C51" s="38" t="s">
         <v>2157</v>
@@ -31947,16 +31905,16 @@
     <row r="52" spans="1:3">
       <c r="A52" s="26"/>
       <c r="B52" s="40" t="s">
-        <v>2190</v>
+        <v>2189</v>
       </c>
       <c r="C52" s="38" t="s">
-        <v>2159</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="26"/>
       <c r="B53" s="40" t="s">
-        <v>2191</v>
+        <v>2190</v>
       </c>
       <c r="C53" s="38" t="s">
         <v>2159</v>
@@ -31965,61 +31923,61 @@
     <row r="54" spans="1:3">
       <c r="A54" s="26"/>
       <c r="B54" s="40" t="s">
-        <v>2192</v>
+        <v>2191</v>
       </c>
       <c r="C54" s="38" t="s">
-        <v>2147</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="26"/>
       <c r="B55" s="40" t="s">
-        <v>2193</v>
+        <v>2192</v>
       </c>
       <c r="C55" s="38" t="s">
-        <v>2161</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="26"/>
       <c r="B56" s="40" t="s">
-        <v>2194</v>
+        <v>2193</v>
       </c>
       <c r="C56" s="38" t="s">
-        <v>2154</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="26"/>
       <c r="B57" s="40" t="s">
-        <v>2195</v>
+        <v>2194</v>
       </c>
       <c r="C57" s="38" t="s">
-        <v>2159</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="26"/>
       <c r="B58" s="40" t="s">
-        <v>2196</v>
+        <v>2195</v>
       </c>
       <c r="C58" s="38" t="s">
-        <v>2161</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="26"/>
       <c r="B59" s="40" t="s">
-        <v>2197</v>
+        <v>2196</v>
       </c>
       <c r="C59" s="38" t="s">
-        <v>2147</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="26"/>
-      <c r="B60" s="41" t="s">
-        <v>2170</v>
+      <c r="B60" s="40" t="s">
+        <v>2197</v>
       </c>
       <c r="C60" s="38" t="s">
         <v>2147</v>
@@ -32027,62 +31985,62 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="26"/>
-      <c r="B61" s="40" t="s">
-        <v>2198</v>
+      <c r="B61" s="41" t="s">
+        <v>2170</v>
       </c>
       <c r="C61" s="38" t="s">
-        <v>2157</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="26"/>
       <c r="B62" s="40" t="s">
-        <v>2199</v>
+        <v>2198</v>
       </c>
       <c r="C62" s="38" t="s">
-        <v>2161</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="26"/>
-      <c r="B63" s="41" t="s">
-        <v>2200</v>
+      <c r="B63" s="40" t="s">
+        <v>2199</v>
       </c>
       <c r="C63" s="38" t="s">
-        <v>2159</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="26"/>
-      <c r="B64" s="40" t="s">
-        <v>2201</v>
+      <c r="B64" s="41" t="s">
+        <v>2200</v>
       </c>
       <c r="C64" s="38" t="s">
-        <v>2157</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="26"/>
       <c r="B65" s="40" t="s">
-        <v>2202</v>
+        <v>2201</v>
       </c>
       <c r="C65" s="38" t="s">
-        <v>2169</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="26"/>
       <c r="B66" s="40" t="s">
-        <v>2203</v>
+        <v>2202</v>
       </c>
       <c r="C66" s="38" t="s">
-        <v>2161</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="26"/>
-      <c r="B67" s="42" t="s">
-        <v>2204</v>
+      <c r="B67" s="40" t="s">
+        <v>2203</v>
       </c>
       <c r="C67" s="38" t="s">
         <v>2161</v>
@@ -32091,252 +32049,252 @@
     <row r="68" spans="1:3">
       <c r="A68" s="26"/>
       <c r="B68" s="42" t="s">
-        <v>2205</v>
+        <v>2204</v>
       </c>
       <c r="C68" s="38" t="s">
-        <v>2159</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="26"/>
       <c r="B69" s="42" t="s">
-        <v>2206</v>
+        <v>2205</v>
       </c>
       <c r="C69" s="38" t="s">
-        <v>2164</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="26"/>
-      <c r="B70" s="40" t="s">
-        <v>2207</v>
+      <c r="B70" s="42" t="s">
+        <v>2206</v>
       </c>
       <c r="C70" s="38" t="s">
-        <v>2157</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="26"/>
       <c r="B71" s="40" t="s">
-        <v>2208</v>
+        <v>2207</v>
       </c>
       <c r="C71" s="38" t="s">
-        <v>2148</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" s="26"/>
       <c r="B72" s="40" t="s">
-        <v>2209</v>
+        <v>2208</v>
       </c>
       <c r="C72" s="38" t="s">
-        <v>2157</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" s="26"/>
       <c r="B73" s="40" t="s">
-        <v>2210</v>
+        <v>2209</v>
       </c>
       <c r="C73" s="38" t="s">
         <v>2157</v>
       </c>
     </row>
     <row r="74" spans="1:3">
-      <c r="A74" s="39" t="s">
+      <c r="A74" s="26"/>
+      <c r="B74" s="40" t="s">
+        <v>2210</v>
+      </c>
+      <c r="C74" s="38" t="s">
+        <v>2157</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="39" t="s">
         <v>345</v>
       </c>
-      <c r="B74" s="38" t="s">
+      <c r="B75" s="38" t="s">
         <v>2110</v>
       </c>
-      <c r="C74" s="38" t="s">
+      <c r="C75" s="38" t="s">
         <v>2211</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" s="38" t="s">
-        <v>3</v>
-      </c>
-      <c r="B75" s="26"/>
-      <c r="C75" s="38" t="s">
-        <v>2212</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" s="38" t="s">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="B76" s="26"/>
       <c r="C76" s="38" t="s">
-        <v>2213</v>
+        <v>2212</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" s="38" t="s">
-        <v>128</v>
+        <v>90</v>
       </c>
       <c r="B77" s="26"/>
       <c r="C77" s="38" t="s">
-        <v>2214</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="38" t="s">
-        <v>1731</v>
+        <v>128</v>
       </c>
       <c r="B78" s="26"/>
       <c r="C78" s="38" t="s">
-        <v>2215</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" s="38" t="s">
-        <v>1825</v>
+        <v>1731</v>
       </c>
       <c r="B79" s="26"/>
       <c r="C79" s="38" t="s">
+        <v>2215</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" s="38" t="s">
+        <v>1825</v>
+      </c>
+      <c r="B80" s="26"/>
+      <c r="C80" s="38" t="s">
         <v>2216</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3">
-      <c r="A80" s="26"/>
-      <c r="B80" s="26" t="s">
-        <v>2217</v>
-      </c>
-      <c r="C80" s="38" t="s">
-        <v>2150</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" s="26"/>
       <c r="B81" s="26" t="s">
-        <v>2218</v>
+        <v>2217</v>
       </c>
       <c r="C81" s="38" t="s">
-        <v>2169</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" s="26"/>
       <c r="B82" s="26" t="s">
-        <v>2219</v>
+        <v>2218</v>
       </c>
       <c r="C82" s="38" t="s">
-        <v>2161</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" s="26"/>
       <c r="B83" s="26" t="s">
-        <v>2220</v>
+        <v>2219</v>
       </c>
       <c r="C83" s="38" t="s">
-        <v>2221</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" s="26"/>
       <c r="B84" s="26" t="s">
-        <v>2222</v>
+        <v>2220</v>
       </c>
       <c r="C84" s="38" t="s">
-        <v>2150</v>
+        <v>2221</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="26"/>
       <c r="B85" s="26" t="s">
-        <v>2223</v>
+        <v>2222</v>
       </c>
       <c r="C85" s="38" t="s">
-        <v>2224</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" s="26"/>
       <c r="B86" s="26" t="s">
-        <v>2225</v>
+        <v>2223</v>
       </c>
       <c r="C86" s="38" t="s">
-        <v>2148</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" s="26"/>
       <c r="B87" s="26" t="s">
-        <v>2226</v>
+        <v>2225</v>
       </c>
       <c r="C87" s="38" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" s="26"/>
       <c r="B88" s="26" t="s">
-        <v>2227</v>
+        <v>2226</v>
       </c>
       <c r="C88" s="38" t="s">
-        <v>2159</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" s="26"/>
       <c r="B89" s="26" t="s">
-        <v>2228</v>
+        <v>2227</v>
       </c>
       <c r="C89" s="38" t="s">
-        <v>2112</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" s="26"/>
       <c r="B90" s="26" t="s">
-        <v>2229</v>
+        <v>2228</v>
       </c>
       <c r="C90" s="38" t="s">
-        <v>2147</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" s="26"/>
       <c r="B91" s="26" t="s">
-        <v>2230</v>
+        <v>2229</v>
       </c>
       <c r="C91" s="38" t="s">
-        <v>2169</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" s="26"/>
       <c r="B92" s="26" t="s">
-        <v>2231</v>
+        <v>2230</v>
       </c>
       <c r="C92" s="38" t="s">
-        <v>2147</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" s="26"/>
       <c r="B93" s="26" t="s">
-        <v>2232</v>
+        <v>2231</v>
       </c>
       <c r="C93" s="38" t="s">
-        <v>2224</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" s="26"/>
       <c r="B94" s="26" t="s">
-        <v>2233</v>
+        <v>2232</v>
       </c>
       <c r="C94" s="38" t="s">
-        <v>2148</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" s="26"/>
       <c r="B95" s="26" t="s">
-        <v>2234</v>
+        <v>2233</v>
       </c>
       <c r="C95" s="38" t="s">
         <v>2148</v>
@@ -32345,63 +32303,72 @@
     <row r="96" spans="1:3">
       <c r="A96" s="26"/>
       <c r="B96" s="26" t="s">
-        <v>1888</v>
+        <v>2234</v>
       </c>
       <c r="C96" s="38" t="s">
-        <v>2161</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" s="26"/>
       <c r="B97" s="26" t="s">
+        <v>1888</v>
+      </c>
+      <c r="C97" s="38" t="s">
+        <v>2161</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" s="26"/>
+      <c r="B98" s="26" t="s">
         <v>2235</v>
       </c>
-      <c r="C97" s="38" t="s">
+      <c r="C98" s="38" t="s">
         <v>2111</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
-      <c r="A98" s="39"/>
-      <c r="B98" s="26" t="s">
+    <row r="99" spans="1:3">
+      <c r="A99" s="39"/>
+      <c r="B99" s="26" t="s">
         <v>2236</v>
       </c>
-      <c r="C98" s="38" t="s">
+      <c r="C99" s="38" t="s">
         <v>2148</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3">
-      <c r="A99" s="26"/>
-      <c r="B99" s="26" t="s">
-        <v>2237</v>
-      </c>
-      <c r="C99" s="38" t="s">
-        <v>2111</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" s="26"/>
       <c r="B100" s="26" t="s">
-        <v>2238</v>
+        <v>2237</v>
       </c>
       <c r="C100" s="38" t="s">
-        <v>2159</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" s="26"/>
-      <c r="B101" s="38" t="s">
-        <v>2275</v>
+      <c r="B101" s="26" t="s">
+        <v>2238</v>
       </c>
       <c r="C101" s="38" t="s">
-        <v>2112</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" s="26"/>
-      <c r="B102" s="26" t="s">
+      <c r="B102" s="38" t="s">
+        <v>2243</v>
+      </c>
+      <c r="C102" s="38" t="s">
+        <v>2112</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3">
+      <c r="A103" s="26"/>
+      <c r="B103" s="26" t="s">
         <v>2239</v>
       </c>
-      <c r="C102" s="38" t="s">
+      <c r="C103" s="38" t="s">
         <v>2112</v>
       </c>
     </row>
@@ -32412,7 +32379,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="33.85546875" style="33" customWidth="1"/>
@@ -32438,7 +32405,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="35" t="s">
-        <v>2274</v>
+        <v>2244</v>
       </c>
       <c r="B2" s="34" t="s">
         <v>2118</v>
@@ -32452,7 +32419,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="35" t="s">
-        <v>2273</v>
+        <v>2259</v>
       </c>
       <c r="B3" s="34" t="s">
         <v>2118</v>
@@ -32483,7 +32450,7 @@
         <v>2155</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>2244</v>
+        <v>2245</v>
       </c>
       <c r="C5" s="35" t="s">
         <v>2155</v>
@@ -32508,7 +32475,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="34" t="s">
-        <v>2255</v>
+        <v>2154</v>
       </c>
       <c r="B7" s="34" t="s">
         <v>2240</v>
@@ -32522,7 +32489,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="34" t="s">
-        <v>2268</v>
+        <v>2221</v>
       </c>
       <c r="B8" s="34" t="s">
         <v>2240</v>
@@ -32536,7 +32503,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="36" t="s">
-        <v>2256</v>
+        <v>2224</v>
       </c>
       <c r="B9" s="34" t="s">
         <v>2240</v>
@@ -32550,7 +32517,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="34" t="s">
-        <v>2269</v>
+        <v>2246</v>
       </c>
       <c r="B10" s="34" t="s">
         <v>2240</v>
@@ -32564,7 +32531,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="34" t="s">
-        <v>2241</v>
+        <v>2247</v>
       </c>
       <c r="B11" s="34" t="s">
         <v>2240</v>
@@ -32578,7 +32545,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="35" t="s">
-        <v>2267</v>
+        <v>2248</v>
       </c>
       <c r="B12" s="34" t="s">
         <v>2240</v>
@@ -32592,7 +32559,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="35" t="s">
-        <v>2257</v>
+        <v>2249</v>
       </c>
       <c r="B13" s="35" t="s">
         <v>2240</v>
@@ -32606,7 +32573,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="34" t="s">
-        <v>2258</v>
+        <v>2250</v>
       </c>
       <c r="B14" s="34" t="s">
         <v>2240</v>
@@ -32620,7 +32587,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="34" t="s">
-        <v>2232</v>
+        <v>2251</v>
       </c>
       <c r="B15" s="34" t="s">
         <v>2240</v>
@@ -32634,13 +32601,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="34" t="s">
-        <v>2250</v>
+        <v>2161</v>
       </c>
       <c r="B16" s="34" t="s">
         <v>2240</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>2249</v>
+        <v>459</v>
       </c>
       <c r="D16" s="43">
         <v>31</v>
@@ -32648,7 +32615,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="34" t="s">
-        <v>2247</v>
+        <v>2252</v>
       </c>
       <c r="B17" s="34" t="s">
         <v>2240</v>
@@ -32662,13 +32629,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="36" t="s">
-        <v>2254</v>
+        <v>2159</v>
       </c>
       <c r="B18" s="34" t="s">
         <v>2240</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>2252</v>
+        <v>1428</v>
       </c>
       <c r="D18" s="43">
         <v>41</v>
@@ -32676,7 +32643,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="34" t="s">
-        <v>2206</v>
+        <v>2164</v>
       </c>
       <c r="B19" s="34" t="s">
         <v>2240</v>
@@ -32690,7 +32657,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="36" t="s">
-        <v>2259</v>
+        <v>2253</v>
       </c>
       <c r="B20" s="34" t="s">
         <v>2240</v>
@@ -32704,7 +32671,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="35" t="s">
-        <v>2265</v>
+        <v>2254</v>
       </c>
       <c r="B21" s="34" t="s">
         <v>2240</v>
@@ -32718,7 +32685,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="35" t="s">
-        <v>2266</v>
+        <v>2255</v>
       </c>
       <c r="B22" s="34" t="s">
         <v>2240</v>
@@ -32732,7 +32699,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="34" t="s">
-        <v>2263</v>
+        <v>2214</v>
       </c>
       <c r="B23" s="34" t="s">
         <v>2240</v>
@@ -32746,7 +32713,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="35" t="s">
-        <v>2261</v>
+        <v>2160</v>
       </c>
       <c r="B24" s="35" t="s">
         <v>2240</v>
@@ -32760,7 +32727,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="34" t="s">
-        <v>2262</v>
+        <v>2211</v>
       </c>
       <c r="B25" s="34" t="s">
         <v>2240</v>
@@ -32774,13 +32741,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="34" t="s">
-        <v>2248</v>
+        <v>2151</v>
       </c>
       <c r="B26" s="34" t="s">
         <v>2240</v>
       </c>
       <c r="C26" s="35" t="s">
-        <v>2249</v>
+        <v>459</v>
       </c>
       <c r="D26" s="43">
         <v>30</v>
@@ -32788,7 +32755,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="34" t="s">
-        <v>2246</v>
+        <v>2150</v>
       </c>
       <c r="B27" s="34" t="s">
         <v>2240</v>
@@ -32802,7 +32769,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="36" t="s">
-        <v>2243</v>
+        <v>2260</v>
       </c>
       <c r="B28" s="34" t="s">
         <v>2118</v>
@@ -32816,13 +32783,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="36" t="s">
-        <v>2251</v>
+        <v>2149</v>
       </c>
       <c r="B29" s="35" t="s">
         <v>2240</v>
       </c>
       <c r="C29" s="35" t="s">
-        <v>2252</v>
+        <v>1428</v>
       </c>
       <c r="D29" s="43">
         <v>40</v>
@@ -32830,7 +32797,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="34" t="s">
-        <v>2270</v>
+        <v>2165</v>
       </c>
       <c r="B30" s="34" t="s">
         <v>2240</v>
@@ -32844,7 +32811,7 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="35" t="s">
-        <v>2260</v>
+        <v>2215</v>
       </c>
       <c r="B31" s="35" t="s">
         <v>2240</v>
@@ -32858,7 +32825,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="34" t="s">
-        <v>2271</v>
+        <v>2256</v>
       </c>
       <c r="B32" s="34" t="s">
         <v>2240</v>
@@ -32872,7 +32839,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="35" t="s">
-        <v>2253</v>
+        <v>2216</v>
       </c>
       <c r="B33" s="35" t="s">
         <v>2240</v>
@@ -32886,7 +32853,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="35" t="s">
-        <v>2264</v>
+        <v>2257</v>
       </c>
       <c r="B34" s="34" t="s">
         <v>2240</v>
@@ -32903,7 +32870,7 @@
         <v>2157</v>
       </c>
       <c r="B35" s="34" t="s">
-        <v>2244</v>
+        <v>2245</v>
       </c>
       <c r="C35" s="35" t="s">
         <v>2157</v>
@@ -32914,13 +32881,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="35" t="s">
+        <v>2242</v>
+      </c>
+      <c r="B36" s="34" t="s">
         <v>2245</v>
       </c>
-      <c r="B36" s="34" t="s">
-        <v>2244</v>
-      </c>
       <c r="C36" s="35" t="s">
-        <v>2245</v>
+        <v>2242</v>
       </c>
       <c r="D36" s="43">
         <v>14</v>
@@ -32928,7 +32895,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="36" t="s">
-        <v>2242</v>
+        <v>2241</v>
       </c>
       <c r="B37" s="35" t="s">
         <v>2118</v>
@@ -32959,7 +32926,7 @@
         <v>2169</v>
       </c>
       <c r="B39" s="34" t="s">
-        <v>2244</v>
+        <v>2245</v>
       </c>
       <c r="C39" s="35" t="s">
         <v>2169</v>
@@ -32970,7 +32937,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="34" t="s">
-        <v>2272</v>
+        <v>2258</v>
       </c>
       <c r="B40" s="34" t="s">
         <v>2118</v>
@@ -32997,18 +32964,28 @@
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="34" t="s">
-        <v>2111</v>
-      </c>
-      <c r="B42" s="34" t="s">
-        <v>2118</v>
+      <c r="A42" s="35" t="s">
+        <v>2212</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>2240</v>
       </c>
       <c r="C42" s="35" t="s">
-        <v>2118</v>
-      </c>
-      <c r="D42" s="43">
-        <v>0</v>
-      </c>
+        <v>964</v>
+      </c>
+      <c r="D42" s="35"/>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="35" t="s">
+        <v>2213</v>
+      </c>
+      <c r="B43" s="35" t="s">
+        <v>2240</v>
+      </c>
+      <c r="C43" s="35" t="s">
+        <v>964</v>
+      </c>
+      <c r="D43" s="35"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1">

</xml_diff>

<commit_message>
feat: add scoped comment synonym lookups
Support filtering shared comment synonym masters by scope so symptom and repair normalization can use a unified alias table.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Koding\tool-fcost\masters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\tool-fcost\masters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD67A39-8DAE-4496-B444-D5DAA856388E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -26,12 +25,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">action!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">defect_category!$A$1:$D$1</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4653" uniqueCount="2385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4724" uniqueCount="2385">
   <si>
     <t>part_used</t>
   </si>
@@ -6792,18 +6791,6 @@
     <t>VERIFIED_OK</t>
   </si>
   <si>
-    <t>symptom_alias</t>
-  </si>
-  <si>
-    <t>symptom_canonical</t>
-  </si>
-  <si>
-    <t>repair_alias</t>
-  </si>
-  <si>
-    <t>repair_canonical</t>
-  </si>
-  <si>
     <t>EXS|EXTRNAL|EXTERNAL</t>
   </si>
   <si>
@@ -7186,12 +7173,24 @@
   </si>
   <si>
     <t>9TAHN7000CE002</t>
+  </si>
+  <si>
+    <t>alias</t>
+  </si>
+  <si>
+    <t>canonical</t>
+  </si>
+  <si>
+    <t>scope</t>
+  </si>
+  <si>
+    <t>both</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="###,###,###,###"/>
   </numFmts>
@@ -7463,16 +7462,16 @@
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10 3 14" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 13 2 2 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal 133 2 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 195" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 2 2" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Normal 315" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Normal 80" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 10 3 14" xfId="7"/>
+    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3"/>
+    <cellStyle name="Normal 13 2 2 2" xfId="4"/>
+    <cellStyle name="Normal 133 2 2" xfId="6"/>
+    <cellStyle name="Normal 195" xfId="8"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2 2" xfId="10"/>
+    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5"/>
+    <cellStyle name="Normal 315" xfId="9"/>
+    <cellStyle name="Normal 80" xfId="1"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -7760,7 +7759,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T1834"/>
   <sheetFormatPr defaultColWidth="10.28515625" defaultRowHeight="12.75"/>
   <cols>
@@ -16304,7 +16303,7 @@
     </row>
     <row r="1066" spans="1:2">
       <c r="A1066" s="4" t="s">
-        <v>2384</v>
+        <v>2380</v>
       </c>
       <c r="B1066" s="3" t="s">
         <v>989</v>
@@ -22474,7 +22473,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T1971"/>
   <sheetFormatPr defaultColWidth="10.28515625" defaultRowHeight="12.75"/>
   <cols>
@@ -30675,7 +30674,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -31636,7 +31635,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -31689,7 +31688,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -31735,7 +31734,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -32112,10 +32111,10 @@
       </c>
       <c r="D19"/>
       <c r="E19" t="s">
-        <v>2363</v>
+        <v>2359</v>
       </c>
       <c r="F19" t="s">
-        <v>2364</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -32130,7 +32129,7 @@
       </c>
       <c r="D20"/>
       <c r="E20" t="s">
-        <v>2363</v>
+        <v>2359</v>
       </c>
       <c r="F20" t="s">
         <v>2155</v>
@@ -32147,7 +32146,7 @@
         <v>2137</v>
       </c>
       <c r="E21" s="32" t="s">
-        <v>2375</v>
+        <v>2371</v>
       </c>
       <c r="F21" t="s">
         <v>2158</v>
@@ -32413,7 +32412,7 @@
         <v>2137</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>2380</v>
+        <v>2376</v>
       </c>
       <c r="F37" t="s">
         <v>2151</v>
@@ -32430,7 +32429,7 @@
         <v>2137</v>
       </c>
       <c r="E38" s="33" t="s">
-        <v>2373</v>
+        <v>2369</v>
       </c>
       <c r="F38" t="s">
         <v>2151</v>
@@ -32447,7 +32446,7 @@
         <v>2137</v>
       </c>
       <c r="E39" s="33" t="s">
-        <v>2379</v>
+        <v>2375</v>
       </c>
       <c r="F39" t="s">
         <v>2151</v>
@@ -32583,7 +32582,7 @@
         <v>2137</v>
       </c>
       <c r="E47" s="33" t="s">
-        <v>2374</v>
+        <v>2370</v>
       </c>
       <c r="F47" t="s">
         <v>2149</v>
@@ -32702,7 +32701,7 @@
         <v>2137</v>
       </c>
       <c r="E54" s="32" t="s">
-        <v>2383</v>
+        <v>2379</v>
       </c>
       <c r="F54" t="s">
         <v>2149</v>
@@ -32804,7 +32803,7 @@
         <v>2137</v>
       </c>
       <c r="E60" t="s">
-        <v>2382</v>
+        <v>2378</v>
       </c>
       <c r="F60" t="s">
         <v>2196</v>
@@ -32855,7 +32854,7 @@
         <v>2137</v>
       </c>
       <c r="E63" s="33" t="s">
-        <v>2381</v>
+        <v>2377</v>
       </c>
       <c r="F63" t="s">
         <v>2142</v>
@@ -32991,7 +32990,7 @@
         <v>2137</v>
       </c>
       <c r="E71" s="32" t="s">
-        <v>2371</v>
+        <v>2367</v>
       </c>
       <c r="F71" t="s">
         <v>2144</v>
@@ -33042,7 +33041,7 @@
         <v>2137</v>
       </c>
       <c r="E74" t="s">
-        <v>2368</v>
+        <v>2364</v>
       </c>
       <c r="F74" t="s">
         <v>2166</v>
@@ -33423,13 +33422,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -34039,8 +34038,8 @@
       <c r="D43" s="29"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{00000000-0009-0000-0000-000006000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D43">
+  <autoFilter ref="A1:D1">
+    <sortState ref="A2:D43">
       <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
@@ -34049,582 +34048,831 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:D56"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="89.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="84.140625" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="104.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>2253</v>
+        <v>2381</v>
       </c>
       <c r="B1" t="s">
-        <v>2254</v>
+        <v>2382</v>
       </c>
       <c r="C1" t="s">
-        <v>2255</v>
+        <v>2383</v>
       </c>
       <c r="D1" t="s">
-        <v>2256</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>2261</v>
+        <v>2257</v>
       </c>
       <c r="B2" t="s">
         <v>2067</v>
       </c>
       <c r="C2" t="s">
-        <v>2378</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2258</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>2337</v>
+        <v>2333</v>
       </c>
       <c r="B3" t="s">
-        <v>2260</v>
+        <v>2256</v>
       </c>
       <c r="C3" t="s">
-        <v>2324</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2259</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>2359</v>
+        <v>2355</v>
       </c>
       <c r="B4" t="s">
-        <v>2330</v>
+        <v>2326</v>
       </c>
       <c r="C4" t="s">
-        <v>2337</v>
-      </c>
-      <c r="D4" t="s">
-        <v>2260</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>2269</v>
+        <v>2265</v>
       </c>
       <c r="B5" t="s">
         <v>2028</v>
       </c>
       <c r="C5" t="s">
-        <v>2257</v>
-      </c>
-      <c r="D5" t="s">
-        <v>2361</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>2270</v>
+        <v>2266</v>
       </c>
       <c r="B6" t="s">
-        <v>2271</v>
+        <v>2267</v>
       </c>
       <c r="C6" t="s">
-        <v>2340</v>
-      </c>
-      <c r="D6" t="s">
-        <v>2262</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>2276</v>
+        <v>2272</v>
       </c>
       <c r="B7" t="s">
-        <v>2277</v>
+        <v>2273</v>
       </c>
       <c r="C7" t="s">
-        <v>2369</v>
-      </c>
-      <c r="D7" t="s">
-        <v>2263</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>2341</v>
+        <v>2337</v>
       </c>
       <c r="B8" t="s">
-        <v>2342</v>
+        <v>2338</v>
       </c>
       <c r="C8" t="s">
-        <v>2264</v>
-      </c>
-      <c r="D8" t="s">
-        <v>2265</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>2343</v>
+        <v>2339</v>
       </c>
       <c r="B9" t="s">
-        <v>2277</v>
+        <v>2273</v>
       </c>
       <c r="C9" t="s">
-        <v>2266</v>
-      </c>
-      <c r="D9" t="s">
-        <v>2273</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>2270</v>
+        <v>2266</v>
       </c>
       <c r="B10" t="s">
-        <v>2271</v>
+        <v>2267</v>
       </c>
       <c r="C10" t="s">
-        <v>2307</v>
-      </c>
-      <c r="D10" t="s">
-        <v>2267</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>2336</v>
+        <v>2332</v>
       </c>
       <c r="B11" t="s">
-        <v>2335</v>
+        <v>2331</v>
       </c>
       <c r="C11" t="s">
-        <v>2268</v>
-      </c>
-      <c r="D11" t="s">
-        <v>2028</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>2344</v>
+        <v>2340</v>
       </c>
       <c r="B12" t="s">
-        <v>2345</v>
+        <v>2341</v>
       </c>
       <c r="C12" t="s">
-        <v>2270</v>
-      </c>
-      <c r="D12" t="s">
-        <v>2271</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="31" t="s">
-        <v>2346</v>
+        <v>2342</v>
       </c>
       <c r="B13" t="s">
         <v>2089</v>
       </c>
       <c r="C13" t="s">
-        <v>2365</v>
-      </c>
-      <c r="D13" t="s">
-        <v>2236</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>2347</v>
+        <v>2343</v>
       </c>
       <c r="B14" t="s">
-        <v>2348</v>
+        <v>2344</v>
       </c>
       <c r="C14" t="s">
-        <v>2272</v>
-      </c>
-      <c r="D14" t="s">
-        <v>989</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>2349</v>
+        <v>2345</v>
       </c>
       <c r="B15" t="s">
-        <v>2350</v>
+        <v>2346</v>
       </c>
       <c r="C15" t="s">
-        <v>2274</v>
-      </c>
-      <c r="D15" t="s">
-        <v>2263</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="31" t="s">
+        <v>2347</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>2348</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>2349</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2350</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
         <v>2351</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B18" t="s">
         <v>2352</v>
       </c>
-      <c r="C16" t="s">
-        <v>2275</v>
-      </c>
-      <c r="D16" t="s">
-        <v>2262</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="C18" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>2354</v>
+      </c>
+      <c r="B19" t="s">
         <v>2353</v>
       </c>
-      <c r="B17" t="s">
-        <v>2354</v>
-      </c>
-      <c r="C17" t="s">
-        <v>2276</v>
-      </c>
-      <c r="D17" t="s">
-        <v>2277</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>2355</v>
-      </c>
-      <c r="B18" t="s">
-        <v>2356</v>
-      </c>
-      <c r="C18" t="s">
-        <v>2278</v>
-      </c>
-      <c r="D18" t="s">
-        <v>2279</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>2358</v>
-      </c>
-      <c r="B19" t="s">
-        <v>2357</v>
-      </c>
       <c r="C19" t="s">
-        <v>2280</v>
-      </c>
-      <c r="D19" t="s">
-        <v>2281</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>2250</v>
       </c>
       <c r="B20" t="s">
+        <v>2358</v>
+      </c>
+      <c r="C20" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>2374</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2254</v>
+      </c>
+      <c r="C21" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>2320</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2255</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>2253</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2357</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>2336</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2258</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>2365</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C25" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>2260</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2261</v>
+      </c>
+      <c r="C26" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>2262</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2269</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>2303</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2263</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>2264</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2028</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>2266</v>
+      </c>
+      <c r="B30" t="s">
+        <v>2267</v>
+      </c>
+      <c r="C30" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>2361</v>
+      </c>
+      <c r="B31" t="s">
+        <v>2236</v>
+      </c>
+      <c r="C31" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>2268</v>
+      </c>
+      <c r="B32" t="s">
+        <v>989</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>2270</v>
+      </c>
+      <c r="B33" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C33" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>2271</v>
+      </c>
+      <c r="B34" t="s">
+        <v>2258</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>2272</v>
+      </c>
+      <c r="B35" t="s">
+        <v>2273</v>
+      </c>
+      <c r="C35" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>2274</v>
+      </c>
+      <c r="B36" t="s">
+        <v>2275</v>
+      </c>
+      <c r="C36" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>2276</v>
+      </c>
+      <c r="B37" t="s">
+        <v>2277</v>
+      </c>
+      <c r="C37" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>2278</v>
+      </c>
+      <c r="B38" t="s">
+        <v>2279</v>
+      </c>
+      <c r="C38" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>2280</v>
+      </c>
+      <c r="B39" t="s">
+        <v>2279</v>
+      </c>
+      <c r="C39" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>2281</v>
+      </c>
+      <c r="B40" t="s">
+        <v>2282</v>
+      </c>
+      <c r="C40" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>2283</v>
+      </c>
+      <c r="B41" t="s">
+        <v>2279</v>
+      </c>
+      <c r="C41" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>2302</v>
+      </c>
+      <c r="B42" t="s">
+        <v>2284</v>
+      </c>
+      <c r="C42" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>2285</v>
+      </c>
+      <c r="B43" t="s">
+        <v>2286</v>
+      </c>
+      <c r="C43" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>2287</v>
+      </c>
+      <c r="B44" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C44" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>2288</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2289</v>
+      </c>
+      <c r="C45" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>2290</v>
+      </c>
+      <c r="B46" t="s">
+        <v>2291</v>
+      </c>
+      <c r="C46" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>2292</v>
+      </c>
+      <c r="B47" t="s">
+        <v>2279</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>2293</v>
+      </c>
+      <c r="B48" t="s">
+        <v>2294</v>
+      </c>
+      <c r="C48" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>2368</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1888</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>2295</v>
+      </c>
+      <c r="B50" t="s">
+        <v>2296</v>
+      </c>
+      <c r="C50" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>2301</v>
+      </c>
+      <c r="B51" t="s">
+        <v>2297</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>2298</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2282</v>
+      </c>
+      <c r="C52" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>2299</v>
+      </c>
+      <c r="B53" t="s">
+        <v>2300</v>
+      </c>
+      <c r="C53" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>2305</v>
+      </c>
+      <c r="B54" t="s">
+        <v>2304</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>2334</v>
+      </c>
+      <c r="B55" t="s">
+        <v>2166</v>
+      </c>
+      <c r="C55" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>2306</v>
+      </c>
+      <c r="B56" t="s">
+        <v>2307</v>
+      </c>
+      <c r="C56" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>2308</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2309</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>2310</v>
+      </c>
+      <c r="B58" t="s">
+        <v>2311</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>2312</v>
+      </c>
+      <c r="B59" t="s">
+        <v>2313</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>2356</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2314</v>
+      </c>
+      <c r="C60" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>2315</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2316</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>2317</v>
+      </c>
+      <c r="B62" t="s">
+        <v>2318</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>2328</v>
+      </c>
+      <c r="B63" t="s">
+        <v>2319</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>2321</v>
+      </c>
+      <c r="B64" t="s">
+        <v>2029</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>2322</v>
+      </c>
+      <c r="B65" t="s">
+        <v>2323</v>
+      </c>
+      <c r="C65" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>2324</v>
+      </c>
+      <c r="B66" t="s">
+        <v>2067</v>
+      </c>
+      <c r="C66" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>2325</v>
+      </c>
+      <c r="B67" t="s">
+        <v>2326</v>
+      </c>
+      <c r="C67" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>2327</v>
+      </c>
+      <c r="B68" t="s">
+        <v>2279</v>
+      </c>
+      <c r="C68" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>2329</v>
+      </c>
+      <c r="B69" t="s">
+        <v>2330</v>
+      </c>
+      <c r="C69" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
+        <v>2332</v>
+      </c>
+      <c r="B70" t="s">
+        <v>2331</v>
+      </c>
+      <c r="C70" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>2335</v>
+      </c>
+      <c r="B71" t="s">
+        <v>2160</v>
+      </c>
+      <c r="C71" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
         <v>2362</v>
       </c>
-      <c r="C20" t="s">
-        <v>2282</v>
-      </c>
-      <c r="D20" t="s">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="C21" t="s">
-        <v>2284</v>
-      </c>
-      <c r="D21" t="s">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="C22" t="s">
-        <v>2285</v>
-      </c>
-      <c r="D22" t="s">
-        <v>2286</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="C23" t="s">
-        <v>2287</v>
-      </c>
-      <c r="D23" t="s">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="C24" t="s">
-        <v>2306</v>
-      </c>
-      <c r="D24" t="s">
-        <v>2288</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="C25" t="s">
-        <v>2289</v>
-      </c>
-      <c r="D25" t="s">
-        <v>2290</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="C26" t="s">
-        <v>2291</v>
-      </c>
-      <c r="D26" t="s">
-        <v>2263</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="C27" t="s">
-        <v>2292</v>
-      </c>
-      <c r="D27" t="s">
-        <v>2293</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="C28" t="s">
-        <v>2294</v>
-      </c>
-      <c r="D28" t="s">
-        <v>2295</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="C29" t="s">
-        <v>2296</v>
-      </c>
-      <c r="D29" t="s">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="C30" t="s">
-        <v>2297</v>
-      </c>
-      <c r="D30" t="s">
-        <v>2298</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="C31" t="s">
+      <c r="B72" t="s">
+        <v>2363</v>
+      </c>
+      <c r="C72" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>2366</v>
+      </c>
+      <c r="B73" t="s">
+        <v>2279</v>
+      </c>
+      <c r="C73" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
         <v>2372</v>
       </c>
-      <c r="D31" t="s">
-        <v>1888</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="C32" t="s">
-        <v>2299</v>
-      </c>
-      <c r="D32" t="s">
-        <v>2300</v>
-      </c>
-    </row>
-    <row r="33" spans="3:4">
-      <c r="C33" t="s">
-        <v>2305</v>
-      </c>
-      <c r="D33" t="s">
-        <v>2301</v>
-      </c>
-    </row>
-    <row r="34" spans="3:4">
-      <c r="C34" t="s">
-        <v>2302</v>
-      </c>
-      <c r="D34" t="s">
-        <v>2286</v>
-      </c>
-    </row>
-    <row r="35" spans="3:4">
-      <c r="C35" t="s">
-        <v>2303</v>
-      </c>
-      <c r="D35" t="s">
-        <v>2304</v>
-      </c>
-    </row>
-    <row r="36" spans="3:4">
-      <c r="C36" t="s">
-        <v>2309</v>
-      </c>
-      <c r="D36" t="s">
-        <v>2308</v>
-      </c>
-    </row>
-    <row r="37" spans="3:4">
-      <c r="C37" t="s">
-        <v>2338</v>
-      </c>
-      <c r="D37" t="s">
-        <v>2166</v>
-      </c>
-    </row>
-    <row r="38" spans="3:4">
-      <c r="C38" t="s">
-        <v>2310</v>
-      </c>
-      <c r="D38" t="s">
-        <v>2311</v>
-      </c>
-    </row>
-    <row r="39" spans="3:4">
-      <c r="C39" t="s">
-        <v>2312</v>
-      </c>
-      <c r="D39" t="s">
-        <v>2313</v>
-      </c>
-    </row>
-    <row r="40" spans="3:4">
-      <c r="C40" t="s">
-        <v>2314</v>
-      </c>
-      <c r="D40" t="s">
-        <v>2315</v>
-      </c>
-    </row>
-    <row r="41" spans="3:4">
-      <c r="C41" t="s">
-        <v>2316</v>
-      </c>
-      <c r="D41" t="s">
-        <v>2317</v>
-      </c>
-    </row>
-    <row r="42" spans="3:4">
-      <c r="C42" t="s">
-        <v>2360</v>
-      </c>
-      <c r="D42" t="s">
-        <v>2318</v>
-      </c>
-    </row>
-    <row r="43" spans="3:4">
-      <c r="C43" t="s">
-        <v>2319</v>
-      </c>
-      <c r="D43" t="s">
-        <v>2320</v>
-      </c>
-    </row>
-    <row r="44" spans="3:4">
-      <c r="C44" t="s">
-        <v>2321</v>
-      </c>
-      <c r="D44" t="s">
-        <v>2322</v>
-      </c>
-    </row>
-    <row r="45" spans="3:4">
-      <c r="C45" t="s">
-        <v>2332</v>
-      </c>
-      <c r="D45" t="s">
-        <v>2323</v>
-      </c>
-    </row>
-    <row r="46" spans="3:4">
-      <c r="C46" t="s">
-        <v>2325</v>
-      </c>
-      <c r="D46" t="s">
-        <v>2029</v>
-      </c>
-    </row>
-    <row r="47" spans="3:4">
-      <c r="C47" t="s">
-        <v>2326</v>
-      </c>
-      <c r="D47" t="s">
-        <v>2327</v>
-      </c>
-    </row>
-    <row r="48" spans="3:4">
-      <c r="C48" t="s">
-        <v>2328</v>
-      </c>
-      <c r="D48" t="s">
-        <v>2067</v>
-      </c>
-    </row>
-    <row r="49" spans="3:4">
-      <c r="C49" t="s">
-        <v>2329</v>
-      </c>
-      <c r="D49" t="s">
-        <v>2330</v>
-      </c>
-    </row>
-    <row r="50" spans="3:4">
-      <c r="C50" t="s">
-        <v>2331</v>
-      </c>
-      <c r="D50" t="s">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="51" spans="3:4">
-      <c r="C51" t="s">
-        <v>2333</v>
-      </c>
-      <c r="D51" t="s">
-        <v>2334</v>
-      </c>
-    </row>
-    <row r="52" spans="3:4">
-      <c r="C52" t="s">
-        <v>2336</v>
-      </c>
-      <c r="D52" t="s">
-        <v>2335</v>
-      </c>
-    </row>
-    <row r="53" spans="3:4">
-      <c r="C53" t="s">
-        <v>2339</v>
-      </c>
-      <c r="D53" t="s">
-        <v>2160</v>
-      </c>
-    </row>
-    <row r="54" spans="3:4">
-      <c r="C54" t="s">
-        <v>2366</v>
-      </c>
-      <c r="D54" t="s">
-        <v>2367</v>
-      </c>
-    </row>
-    <row r="55" spans="3:4">
-      <c r="C55" t="s">
-        <v>2370</v>
-      </c>
-      <c r="D55" t="s">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="56" spans="3:4">
-      <c r="C56" t="s">
-        <v>2376</v>
-      </c>
-      <c r="D56" t="s">
-        <v>2377</v>
+      <c r="B74" t="s">
+        <v>2373</v>
+      </c>
+      <c r="C74" t="s">
+        <v>2384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove obsolete symptom definitions from symptom.csv to streamline the symptom matching process.
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4724" uniqueCount="2385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4731" uniqueCount="2386">
   <si>
     <t>part_used</t>
   </si>
@@ -6134,9 +6134,6 @@
     <t>migrated from plain contains; source=X ADA GAMBAR</t>
   </si>
   <si>
-    <t>NO DISPLAY|STANDBY|GAMBAR GELAP|GAMBAR TDK KELUAR</t>
-  </si>
-  <si>
     <t>migrated from plain contains; source=NO DISPLAY</t>
   </si>
   <si>
@@ -6146,9 +6143,6 @@
     <t>migrated from plain contains; source=MATI</t>
   </si>
   <si>
-    <t>HANYA SUARA</t>
-  </si>
-  <si>
     <t>migrated from plain contains; source=HANYA SUARA SAJA</t>
   </si>
   <si>
@@ -6197,9 +6191,6 @@
     <t>migrated from wildcard contains; source=*TIDAK BISA HIDUP*</t>
   </si>
   <si>
-    <t>BERGERAK</t>
-  </si>
-  <si>
     <t>migrated from wildcard contains; source=*BERGERAK*</t>
   </si>
   <si>
@@ -6995,9 +6986,6 @@
     <t>GT|GNT|GNTI</t>
   </si>
   <si>
-    <t>BLAND</t>
-  </si>
-  <si>
     <t>DITAR IK</t>
   </si>
   <si>
@@ -7031,9 +7019,6 @@
     <t>CHANEL|CHENEL</t>
   </si>
   <si>
-    <t>X ADA GAMBAR|TIDAK ADA GAMBAR|TDK ADA GAMBAR|TIDAK AD AGAMBAR|TIDAK AD GAMBAR|TDK ADA GMBR</t>
-  </si>
-  <si>
     <t>SETING|STEL</t>
   </si>
   <si>
@@ -7043,9 +7028,6 @@
     <t>UNIL|UNTIT</t>
   </si>
   <si>
-    <t>0AMBAR</t>
-  </si>
-  <si>
     <t>GAMBAR</t>
   </si>
   <si>
@@ -7185,6 +7167,27 @@
   </si>
   <si>
     <t>both</t>
+  </si>
+  <si>
+    <t>BLAND|BLAN</t>
+  </si>
+  <si>
+    <t>0AMBAR|GAMABAR|</t>
+  </si>
+  <si>
+    <t>HANYA SUARA|SUARA SAJA</t>
+  </si>
+  <si>
+    <t>SUARA SAJA</t>
+  </si>
+  <si>
+    <t>BERGERAK|LAYAR BEREMBUN|LAYAR BERGERAK</t>
+  </si>
+  <si>
+    <t>X ADA GAMBAR|TIDAK ADA GAMBAR|TDK ADA GAMBAR|TIDAK AD AGAMBAR|TIDAK AD GAMBAR|TDK ADA GMBR|GAMBAR TIDAK KELUAR|TIDAK AD AGMBR|LCD-PIC-C01-GAMBAR TIDAK KELUAR</t>
+  </si>
+  <si>
+    <t>NO DISPLAY|STANDBY|GAMBAR GELAP|GAMBAR TDK KELUAR|GELAP|GAMBAR TIDAK KELUAR</t>
   </si>
 </sst>
 </file>
@@ -16303,7 +16306,7 @@
     </row>
     <row r="1066" spans="1:2">
       <c r="A1066" s="4" t="s">
-        <v>2380</v>
+        <v>2374</v>
       </c>
       <c r="B1066" s="3" t="s">
         <v>989</v>
@@ -30675,7 +30678,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -30857,13 +30860,13 @@
         <v>2020</v>
       </c>
       <c r="D9" t="s">
-        <v>2034</v>
+        <v>2385</v>
       </c>
       <c r="E9" t="s">
         <v>2029</v>
       </c>
       <c r="F9" t="s">
-        <v>2035</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -30877,13 +30880,13 @@
         <v>2027</v>
       </c>
       <c r="D10" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
       <c r="E10" t="s">
         <v>2029</v>
       </c>
       <c r="F10" t="s">
-        <v>2037</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -30897,13 +30900,13 @@
         <v>2020</v>
       </c>
       <c r="D11" t="s">
-        <v>2038</v>
+        <v>2382</v>
       </c>
       <c r="E11" t="s">
         <v>2029</v>
       </c>
       <c r="F11" t="s">
-        <v>2039</v>
+        <v>2037</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -30917,13 +30920,13 @@
         <v>2020</v>
       </c>
       <c r="D12" t="s">
+        <v>2038</v>
+      </c>
+      <c r="E12" t="s">
+        <v>2039</v>
+      </c>
+      <c r="F12" t="s">
         <v>2040</v>
-      </c>
-      <c r="E12" t="s">
-        <v>2041</v>
-      </c>
-      <c r="F12" t="s">
-        <v>2042</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -30937,13 +30940,13 @@
         <v>2020</v>
       </c>
       <c r="D13" t="s">
-        <v>2043</v>
+        <v>2041</v>
       </c>
       <c r="E13" t="s">
-        <v>2041</v>
+        <v>2039</v>
       </c>
       <c r="F13" t="s">
-        <v>2044</v>
+        <v>2042</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -30957,13 +30960,13 @@
         <v>2027</v>
       </c>
       <c r="D14" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E14" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F14" t="s">
         <v>2045</v>
-      </c>
-      <c r="E14" t="s">
-        <v>2046</v>
-      </c>
-      <c r="F14" t="s">
-        <v>2047</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -30977,13 +30980,13 @@
         <v>2027</v>
       </c>
       <c r="D15" t="s">
+        <v>2044</v>
+      </c>
+      <c r="E15" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F15" t="s">
         <v>2046</v>
-      </c>
-      <c r="E15" t="s">
-        <v>2046</v>
-      </c>
-      <c r="F15" t="s">
-        <v>2048</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -30997,13 +31000,13 @@
         <v>2027</v>
       </c>
       <c r="D16" t="s">
-        <v>2049</v>
+        <v>2047</v>
       </c>
       <c r="E16" t="s">
-        <v>2049</v>
+        <v>2047</v>
       </c>
       <c r="F16" t="s">
-        <v>2050</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -31017,13 +31020,13 @@
         <v>2027</v>
       </c>
       <c r="D17" t="s">
-        <v>2051</v>
+        <v>2049</v>
       </c>
       <c r="E17" t="s">
-        <v>2049</v>
+        <v>2047</v>
       </c>
       <c r="F17" t="s">
-        <v>2052</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -31037,13 +31040,13 @@
         <v>2027</v>
       </c>
       <c r="D18" t="s">
-        <v>2053</v>
+        <v>2051</v>
       </c>
       <c r="E18" t="s">
         <v>2022</v>
       </c>
       <c r="F18" t="s">
-        <v>2054</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -31054,16 +31057,16 @@
         <v>989</v>
       </c>
       <c r="C19" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D19" t="s">
-        <v>2055</v>
+        <v>2383</v>
       </c>
       <c r="E19" t="s">
-        <v>2041</v>
+        <v>2039</v>
       </c>
       <c r="F19" t="s">
-        <v>2056</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -31077,13 +31080,13 @@
         <v>2020</v>
       </c>
       <c r="D20" t="s">
-        <v>2057</v>
+        <v>2054</v>
       </c>
       <c r="E20" t="s">
-        <v>2058</v>
+        <v>2055</v>
       </c>
       <c r="F20" t="s">
-        <v>2059</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -31097,13 +31100,10 @@
         <v>2020</v>
       </c>
       <c r="D21" t="s">
-        <v>2060</v>
+        <v>2111</v>
       </c>
       <c r="E21" t="s">
-        <v>2061</v>
-      </c>
-      <c r="F21" t="s">
-        <v>2062</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -31114,16 +31114,16 @@
         <v>989</v>
       </c>
       <c r="C22" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D22" t="s">
-        <v>2063</v>
+        <v>2057</v>
       </c>
       <c r="E22" t="s">
-        <v>2064</v>
+        <v>2058</v>
       </c>
       <c r="F22" t="s">
-        <v>2065</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -31131,19 +31131,19 @@
         <v>220</v>
       </c>
       <c r="B23" t="s">
-        <v>459</v>
+        <v>989</v>
       </c>
       <c r="C23" t="s">
-        <v>2020</v>
+        <v>2027</v>
       </c>
       <c r="D23" t="s">
-        <v>2066</v>
+        <v>2060</v>
       </c>
       <c r="E23" t="s">
-        <v>2067</v>
+        <v>2061</v>
       </c>
       <c r="F23" t="s">
-        <v>2068</v>
+        <v>2062</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -31157,13 +31157,13 @@
         <v>2020</v>
       </c>
       <c r="D24" t="s">
-        <v>2069</v>
+        <v>2063</v>
       </c>
       <c r="E24" t="s">
-        <v>2022</v>
+        <v>2064</v>
       </c>
       <c r="F24" t="s">
-        <v>2070</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -31177,13 +31177,13 @@
         <v>2020</v>
       </c>
       <c r="D25" t="s">
-        <v>2071</v>
+        <v>2066</v>
       </c>
       <c r="E25" t="s">
         <v>2022</v>
       </c>
       <c r="F25" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -31197,13 +31197,13 @@
         <v>2020</v>
       </c>
       <c r="D26" t="s">
-        <v>2073</v>
+        <v>2068</v>
       </c>
       <c r="E26" t="s">
-        <v>2074</v>
+        <v>2022</v>
       </c>
       <c r="F26" t="s">
-        <v>2075</v>
+        <v>2069</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -31217,13 +31217,13 @@
         <v>2020</v>
       </c>
       <c r="D27" t="s">
-        <v>2076</v>
+        <v>2070</v>
       </c>
       <c r="E27" t="s">
-        <v>2077</v>
+        <v>2071</v>
       </c>
       <c r="F27" t="s">
-        <v>2078</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -31234,16 +31234,16 @@
         <v>459</v>
       </c>
       <c r="C28" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D28" t="s">
-        <v>2079</v>
+        <v>2073</v>
       </c>
       <c r="E28" t="s">
-        <v>2080</v>
+        <v>2074</v>
       </c>
       <c r="F28" t="s">
-        <v>2081</v>
+        <v>2075</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -31254,16 +31254,16 @@
         <v>459</v>
       </c>
       <c r="C29" t="s">
-        <v>2020</v>
+        <v>2027</v>
       </c>
       <c r="D29" t="s">
-        <v>2082</v>
+        <v>2076</v>
       </c>
       <c r="E29" t="s">
-        <v>2083</v>
+        <v>2077</v>
       </c>
       <c r="F29" t="s">
-        <v>2084</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -31277,13 +31277,13 @@
         <v>2020</v>
       </c>
       <c r="D30" t="s">
-        <v>2085</v>
+        <v>2079</v>
       </c>
       <c r="E30" t="s">
-        <v>2086</v>
+        <v>2080</v>
       </c>
       <c r="F30" t="s">
-        <v>2087</v>
+        <v>2081</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -31294,16 +31294,16 @@
         <v>459</v>
       </c>
       <c r="C31" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D31" t="s">
-        <v>2088</v>
+        <v>2082</v>
       </c>
       <c r="E31" t="s">
-        <v>2089</v>
+        <v>2083</v>
       </c>
       <c r="F31" t="s">
-        <v>2090</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -31314,16 +31314,16 @@
         <v>459</v>
       </c>
       <c r="C32" t="s">
-        <v>2020</v>
+        <v>2027</v>
       </c>
       <c r="D32" t="s">
-        <v>2091</v>
+        <v>2085</v>
       </c>
       <c r="E32" t="s">
-        <v>2089</v>
+        <v>2086</v>
       </c>
       <c r="F32" t="s">
-        <v>2092</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -31334,16 +31334,16 @@
         <v>459</v>
       </c>
       <c r="C33" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D33" t="s">
-        <v>2093</v>
+        <v>2088</v>
       </c>
       <c r="E33" t="s">
-        <v>2094</v>
+        <v>2086</v>
       </c>
       <c r="F33" t="s">
-        <v>2095</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -31354,16 +31354,16 @@
         <v>459</v>
       </c>
       <c r="C34" t="s">
-        <v>2020</v>
+        <v>2027</v>
       </c>
       <c r="D34" t="s">
-        <v>2096</v>
+        <v>2090</v>
       </c>
       <c r="E34" t="s">
-        <v>2097</v>
+        <v>2091</v>
       </c>
       <c r="F34" t="s">
-        <v>2098</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -31374,16 +31374,16 @@
         <v>459</v>
       </c>
       <c r="C35" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D35" t="s">
-        <v>2099</v>
+        <v>2093</v>
       </c>
       <c r="E35" t="s">
-        <v>2100</v>
+        <v>2094</v>
       </c>
       <c r="F35" t="s">
-        <v>2101</v>
+        <v>2095</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -31397,13 +31397,13 @@
         <v>2027</v>
       </c>
       <c r="D36" t="s">
-        <v>2102</v>
+        <v>2096</v>
       </c>
       <c r="E36" t="s">
-        <v>2103</v>
+        <v>2097</v>
       </c>
       <c r="F36" t="s">
-        <v>2104</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -31411,19 +31411,19 @@
         <v>360</v>
       </c>
       <c r="B37" t="s">
-        <v>1659</v>
+        <v>459</v>
       </c>
       <c r="C37" t="s">
-        <v>2020</v>
+        <v>2027</v>
       </c>
       <c r="D37" t="s">
-        <v>2105</v>
+        <v>2099</v>
       </c>
       <c r="E37" t="s">
-        <v>2106</v>
+        <v>2100</v>
       </c>
       <c r="F37" t="s">
-        <v>2107</v>
+        <v>2101</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -31431,19 +31431,19 @@
         <v>370</v>
       </c>
       <c r="B38" t="s">
-        <v>989</v>
+        <v>1659</v>
       </c>
       <c r="C38" t="s">
         <v>2020</v>
       </c>
       <c r="D38" t="s">
-        <v>2108</v>
+        <v>2102</v>
       </c>
       <c r="E38" t="s">
-        <v>2029</v>
+        <v>2103</v>
       </c>
       <c r="F38" t="s">
-        <v>2109</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -31451,36 +31451,36 @@
         <v>380</v>
       </c>
       <c r="B39" t="s">
-        <v>1731</v>
+        <v>989</v>
       </c>
       <c r="C39" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D39" t="s">
-        <v>2110</v>
+        <v>2105</v>
       </c>
       <c r="E39" t="s">
-        <v>2100</v>
+        <v>2029</v>
+      </c>
+      <c r="F39" t="s">
+        <v>2106</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40">
         <v>390</v>
       </c>
-      <c r="B40" s="31" t="s">
-        <v>214</v>
+      <c r="B40" t="s">
+        <v>1731</v>
       </c>
       <c r="C40" t="s">
-        <v>2020</v>
+        <v>2027</v>
       </c>
       <c r="D40" t="s">
-        <v>2111</v>
+        <v>2107</v>
       </c>
       <c r="E40" t="s">
-        <v>2067</v>
-      </c>
-      <c r="F40" t="s">
-        <v>2068</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -31494,30 +31494,33 @@
         <v>2020</v>
       </c>
       <c r="D41" t="s">
-        <v>2069</v>
+        <v>2108</v>
       </c>
       <c r="E41" t="s">
-        <v>2022</v>
+        <v>2064</v>
       </c>
       <c r="F41" t="s">
-        <v>2070</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42">
         <v>410</v>
       </c>
-      <c r="B42" t="s">
-        <v>459</v>
+      <c r="B42" s="31" t="s">
+        <v>214</v>
       </c>
       <c r="C42" t="s">
         <v>2020</v>
       </c>
-      <c r="D42" s="31" t="s">
-        <v>2112</v>
+      <c r="D42" t="s">
+        <v>2066</v>
       </c>
       <c r="E42" t="s">
-        <v>2074</v>
+        <v>2022</v>
+      </c>
+      <c r="F42" t="s">
+        <v>2067</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -31525,16 +31528,16 @@
         <v>420</v>
       </c>
       <c r="B43" t="s">
-        <v>345</v>
+        <v>459</v>
       </c>
       <c r="C43" t="s">
         <v>2020</v>
       </c>
       <c r="D43" s="31" t="s">
-        <v>2113</v>
+        <v>2109</v>
       </c>
       <c r="E43" t="s">
-        <v>2086</v>
+        <v>2071</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -31545,33 +31548,30 @@
         <v>345</v>
       </c>
       <c r="C44" t="s">
-        <v>2027</v>
+        <v>2020</v>
       </c>
       <c r="D44" s="31" t="s">
-        <v>2114</v>
+        <v>2110</v>
       </c>
       <c r="E44" t="s">
-        <v>2115</v>
+        <v>2083</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45">
         <v>440</v>
       </c>
-      <c r="B45" s="31" t="s">
-        <v>214</v>
+      <c r="B45" t="s">
+        <v>345</v>
       </c>
       <c r="C45" t="s">
-        <v>2020</v>
-      </c>
-      <c r="D45" t="s">
-        <v>2032</v>
+        <v>2027</v>
+      </c>
+      <c r="D45" s="31" t="s">
+        <v>2111</v>
       </c>
       <c r="E45" t="s">
-        <v>2029</v>
-      </c>
-      <c r="F45" t="s">
-        <v>2033</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -31582,13 +31582,16 @@
         <v>214</v>
       </c>
       <c r="C46" t="s">
-        <v>2027</v>
-      </c>
-      <c r="D46" s="31" t="s">
-        <v>2116</v>
+        <v>2020</v>
+      </c>
+      <c r="D46" t="s">
+        <v>2032</v>
       </c>
       <c r="E46" t="s">
-        <v>2115</v>
+        <v>2029</v>
+      </c>
+      <c r="F46" t="s">
+        <v>2033</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -31596,19 +31599,16 @@
         <v>460</v>
       </c>
       <c r="B47" s="31" t="s">
-        <v>1815</v>
+        <v>214</v>
       </c>
       <c r="C47" t="s">
-        <v>2020</v>
-      </c>
-      <c r="D47" t="s">
-        <v>2024</v>
+        <v>2027</v>
+      </c>
+      <c r="D47" s="31" t="s">
+        <v>2113</v>
       </c>
       <c r="E47" t="s">
-        <v>2025</v>
-      </c>
-      <c r="F47" t="s">
-        <v>2026</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -31622,10 +31622,30 @@
         <v>2020</v>
       </c>
       <c r="D48" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E48" t="s">
+        <v>2025</v>
+      </c>
+      <c r="F48" t="s">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49">
+        <v>480</v>
+      </c>
+      <c r="B49" s="31" t="s">
+        <v>1815</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2020</v>
+      </c>
+      <c r="D49" t="s">
         <v>2032</v>
       </c>
-      <c r="E48" t="s">
-        <v>2086</v>
+      <c r="E49" t="s">
+        <v>2083</v>
       </c>
     </row>
   </sheetData>
@@ -31644,42 +31664,42 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="22" t="s">
-        <v>2117</v>
+        <v>2114</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>2118</v>
+        <v>2115</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="23" t="s">
-        <v>2119</v>
+        <v>2116</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>2120</v>
+        <v>2117</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="23" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>2122</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="23" t="s">
-        <v>2123</v>
+        <v>2120</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>2124</v>
+        <v>2121</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="24" t="s">
-        <v>2125</v>
+        <v>2122</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>2126</v>
+        <v>2123</v>
       </c>
     </row>
   </sheetData>
@@ -31698,34 +31718,34 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="22" t="s">
-        <v>2127</v>
+        <v>2124</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>2128</v>
+        <v>2125</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="23" t="s">
-        <v>2129</v>
+        <v>2126</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>2130</v>
+        <v>2127</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="23" t="s">
-        <v>2131</v>
+        <v>2128</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>2130</v>
+        <v>2127</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="23" t="s">
-        <v>2132</v>
+        <v>2129</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>2130</v>
+        <v>2127</v>
       </c>
     </row>
   </sheetData>
@@ -31753,19 +31773,19 @@
         <v>2015</v>
       </c>
       <c r="B1" t="s">
-        <v>2133</v>
+        <v>2130</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>2134</v>
+        <v>2131</v>
       </c>
       <c r="E1" t="s">
-        <v>2135</v>
+        <v>2132</v>
       </c>
       <c r="F1" t="s">
-        <v>2136</v>
+        <v>2133</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -31776,13 +31796,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E2" t="s">
-        <v>2138</v>
+        <v>2135</v>
       </c>
       <c r="F2" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -31796,13 +31816,13 @@
         <v>1815</v>
       </c>
       <c r="D3" t="s">
+        <v>2134</v>
+      </c>
+      <c r="E3" t="s">
         <v>2137</v>
       </c>
-      <c r="E3" t="s">
-        <v>2140</v>
-      </c>
       <c r="F3" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -31813,13 +31833,13 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E4" t="s">
-        <v>2141</v>
+        <v>2138</v>
       </c>
       <c r="F4" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -31830,13 +31850,13 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E5" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="F5" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -31850,13 +31870,13 @@
         <v>1428</v>
       </c>
       <c r="D6" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E6" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F6" t="s">
-        <v>2145</v>
+        <v>2142</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -31870,13 +31890,13 @@
         <v>989</v>
       </c>
       <c r="D7" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E7" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F7" t="s">
-        <v>2146</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -31890,13 +31910,13 @@
         <v>459</v>
       </c>
       <c r="D8" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E8" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F8" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -31910,13 +31930,13 @@
         <v>1659</v>
       </c>
       <c r="D9" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E9" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F9" t="s">
-        <v>2148</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -31930,13 +31950,13 @@
         <v>1397</v>
       </c>
       <c r="D10" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E10" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F10" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -31950,13 +31970,13 @@
         <v>214</v>
       </c>
       <c r="D11" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E11" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F11" t="s">
-        <v>2150</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -31970,13 +31990,13 @@
         <v>109</v>
       </c>
       <c r="D12" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E12" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F12" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -31990,13 +32010,13 @@
         <v>345</v>
       </c>
       <c r="D13" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E13" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F13" t="s">
-        <v>2152</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -32010,13 +32030,13 @@
         <v>3</v>
       </c>
       <c r="D14" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E14" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F14" t="s">
-        <v>2153</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -32030,13 +32050,13 @@
         <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E15" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F15" t="s">
-        <v>2154</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -32050,13 +32070,13 @@
         <v>128</v>
       </c>
       <c r="D16" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E16" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F16" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -32070,13 +32090,13 @@
         <v>1731</v>
       </c>
       <c r="D17" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E17" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F17" t="s">
-        <v>2156</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -32090,13 +32110,13 @@
         <v>1825</v>
       </c>
       <c r="D18" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E18" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="F18" t="s">
-        <v>2157</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -32111,10 +32131,10 @@
       </c>
       <c r="D19"/>
       <c r="E19" t="s">
-        <v>2359</v>
+        <v>2353</v>
       </c>
       <c r="F19" t="s">
-        <v>2360</v>
+        <v>2354</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -32129,10 +32149,10 @@
       </c>
       <c r="D20"/>
       <c r="E20" t="s">
-        <v>2359</v>
+        <v>2353</v>
       </c>
       <c r="F20" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -32143,13 +32163,13 @@
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E21" s="32" t="s">
-        <v>2371</v>
+        <v>2365</v>
       </c>
       <c r="F21" t="s">
-        <v>2158</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -32160,13 +32180,13 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E22" t="s">
-        <v>2159</v>
+        <v>2156</v>
       </c>
       <c r="F22" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -32177,13 +32197,13 @@
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E23" t="s">
-        <v>2161</v>
+        <v>2158</v>
       </c>
       <c r="F23" t="s">
-        <v>2162</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -32194,13 +32214,13 @@
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E24" t="s">
-        <v>2163</v>
+        <v>2160</v>
       </c>
       <c r="F24" t="s">
-        <v>2164</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -32211,13 +32231,13 @@
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E25" t="s">
-        <v>2165</v>
+        <v>2162</v>
       </c>
       <c r="F25" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -32228,13 +32248,13 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E26" t="s">
-        <v>2167</v>
+        <v>2164</v>
       </c>
       <c r="F26" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -32245,13 +32265,13 @@
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>2036</v>
+        <v>2035</v>
       </c>
       <c r="E27" t="s">
-        <v>2168</v>
+        <v>2165</v>
       </c>
       <c r="F27" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -32262,13 +32282,13 @@
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>2169</v>
+        <v>2166</v>
       </c>
       <c r="E28" s="25" t="s">
-        <v>2170</v>
+        <v>2167</v>
       </c>
       <c r="F28" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -32279,10 +32299,10 @@
         <v>1</v>
       </c>
       <c r="E29" s="25" t="s">
-        <v>2171</v>
+        <v>2168</v>
       </c>
       <c r="F29" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -32296,10 +32316,10 @@
         <v>2029</v>
       </c>
       <c r="E30" s="25" t="s">
-        <v>2172</v>
+        <v>2169</v>
       </c>
       <c r="F30" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -32310,10 +32330,10 @@
         <v>1</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>2173</v>
+        <v>2170</v>
       </c>
       <c r="F31" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -32324,13 +32344,13 @@
         <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E32" t="s">
-        <v>2174</v>
+        <v>2171</v>
       </c>
       <c r="F32" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -32341,13 +32361,13 @@
         <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E33" t="s">
-        <v>2175</v>
+        <v>2172</v>
       </c>
       <c r="F33" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -32358,13 +32378,13 @@
         <v>1</v>
       </c>
       <c r="D34" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E34" t="s">
-        <v>2176</v>
+        <v>2173</v>
       </c>
       <c r="F34" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -32375,13 +32395,13 @@
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E35" t="s">
-        <v>2177</v>
+        <v>2174</v>
       </c>
       <c r="F35" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -32392,13 +32412,13 @@
         <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E36" t="s">
-        <v>2178</v>
+        <v>2175</v>
       </c>
       <c r="F36" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -32409,13 +32429,13 @@
         <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>2376</v>
+        <v>2370</v>
       </c>
       <c r="F37" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -32426,13 +32446,13 @@
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E38" s="33" t="s">
-        <v>2369</v>
+        <v>2363</v>
       </c>
       <c r="F38" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -32443,13 +32463,13 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E39" s="33" t="s">
-        <v>2375</v>
+        <v>2369</v>
       </c>
       <c r="F39" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -32460,13 +32480,13 @@
         <v>1</v>
       </c>
       <c r="D40" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E40" t="s">
-        <v>2179</v>
+        <v>2176</v>
       </c>
       <c r="F40" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -32477,13 +32497,13 @@
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E41" t="s">
-        <v>2180</v>
+        <v>2177</v>
       </c>
       <c r="F41" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -32494,13 +32514,13 @@
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E42" t="s">
-        <v>2181</v>
+        <v>2178</v>
       </c>
       <c r="F42" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -32511,13 +32531,13 @@
         <v>1</v>
       </c>
       <c r="D43" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E43" t="s">
-        <v>2182</v>
+        <v>2179</v>
       </c>
       <c r="F43" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -32528,13 +32548,13 @@
         <v>1</v>
       </c>
       <c r="D44" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E44" t="s">
-        <v>2183</v>
+        <v>2180</v>
       </c>
       <c r="F44" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -32545,13 +32565,13 @@
         <v>1</v>
       </c>
       <c r="D45" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E45" t="s">
-        <v>2184</v>
+        <v>2181</v>
       </c>
       <c r="F45" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -32562,13 +32582,13 @@
         <v>1</v>
       </c>
       <c r="D46" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E46" t="s">
-        <v>2185</v>
+        <v>2182</v>
       </c>
       <c r="F46" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -32579,13 +32599,13 @@
         <v>1</v>
       </c>
       <c r="D47" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E47" s="33" t="s">
-        <v>2370</v>
+        <v>2364</v>
       </c>
       <c r="F47" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -32596,13 +32616,13 @@
         <v>1</v>
       </c>
       <c r="D48" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E48" t="s">
-        <v>2187</v>
+        <v>2184</v>
       </c>
       <c r="F48" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -32613,13 +32633,13 @@
         <v>1</v>
       </c>
       <c r="D49" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E49" t="s">
-        <v>2188</v>
+        <v>2185</v>
       </c>
       <c r="F49" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -32630,13 +32650,13 @@
         <v>1</v>
       </c>
       <c r="D50" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E50" t="s">
-        <v>2189</v>
+        <v>2186</v>
       </c>
       <c r="F50" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -32647,13 +32667,13 @@
         <v>1</v>
       </c>
       <c r="D51" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E51" t="s">
-        <v>2190</v>
+        <v>2187</v>
       </c>
       <c r="F51" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -32664,13 +32684,13 @@
         <v>1</v>
       </c>
       <c r="D52" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E52" t="s">
-        <v>2191</v>
+        <v>2188</v>
       </c>
       <c r="F52" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -32681,13 +32701,13 @@
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E53" t="s">
-        <v>2192</v>
+        <v>2189</v>
       </c>
       <c r="F53" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -32698,13 +32718,13 @@
         <v>1</v>
       </c>
       <c r="D54" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E54" s="32" t="s">
-        <v>2379</v>
+        <v>2373</v>
       </c>
       <c r="F54" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -32715,13 +32735,13 @@
         <v>1</v>
       </c>
       <c r="D55" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E55" t="s">
-        <v>2193</v>
+        <v>2190</v>
       </c>
       <c r="F55" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -32732,13 +32752,13 @@
         <v>1</v>
       </c>
       <c r="D56" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E56" t="s">
-        <v>2186</v>
+        <v>2183</v>
       </c>
       <c r="F56" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -32749,13 +32769,13 @@
         <v>1</v>
       </c>
       <c r="D57" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E57" t="s">
-        <v>2194</v>
+        <v>2191</v>
       </c>
       <c r="F57" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -32766,13 +32786,13 @@
         <v>1</v>
       </c>
       <c r="D58" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E58" t="s">
-        <v>2195</v>
+        <v>2192</v>
       </c>
       <c r="F58" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -32783,13 +32803,13 @@
         <v>1</v>
       </c>
       <c r="D59" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E59" t="s">
-        <v>2194</v>
+        <v>2191</v>
       </c>
       <c r="F59" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -32800,13 +32820,13 @@
         <v>1</v>
       </c>
       <c r="D60" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E60" t="s">
-        <v>2378</v>
+        <v>2372</v>
       </c>
       <c r="F60" t="s">
-        <v>2196</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -32817,13 +32837,13 @@
         <v>1</v>
       </c>
       <c r="D61" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E61" t="s">
-        <v>2197</v>
+        <v>2194</v>
       </c>
       <c r="F61" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -32834,13 +32854,13 @@
         <v>1</v>
       </c>
       <c r="D62" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E62" t="s">
-        <v>2198</v>
+        <v>2195</v>
       </c>
       <c r="F62" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -32851,13 +32871,13 @@
         <v>1</v>
       </c>
       <c r="D63" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E63" s="33" t="s">
-        <v>2377</v>
+        <v>2371</v>
       </c>
       <c r="F63" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -32868,13 +32888,13 @@
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E64" t="s">
-        <v>2199</v>
+        <v>2196</v>
       </c>
       <c r="F64" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -32885,13 +32905,13 @@
         <v>1</v>
       </c>
       <c r="D65" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E65" t="s">
-        <v>2200</v>
+        <v>2197</v>
       </c>
       <c r="F65" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -32902,13 +32922,13 @@
         <v>1</v>
       </c>
       <c r="D66" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E66" t="s">
-        <v>2201</v>
+        <v>2198</v>
       </c>
       <c r="F66" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -32919,13 +32939,13 @@
         <v>1</v>
       </c>
       <c r="D67" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E67" t="s">
-        <v>2202</v>
+        <v>2199</v>
       </c>
       <c r="F67" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -32936,13 +32956,13 @@
         <v>1</v>
       </c>
       <c r="D68" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E68" t="s">
-        <v>2203</v>
+        <v>2200</v>
       </c>
       <c r="F68" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -32953,13 +32973,13 @@
         <v>1</v>
       </c>
       <c r="D69" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E69" t="s">
-        <v>2204</v>
+        <v>2201</v>
       </c>
       <c r="F69" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -32970,13 +32990,13 @@
         <v>1</v>
       </c>
       <c r="D70" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E70" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="F70" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -32987,13 +33007,13 @@
         <v>1</v>
       </c>
       <c r="D71" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E71" s="32" t="s">
-        <v>2367</v>
+        <v>2361</v>
       </c>
       <c r="F71" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -33004,13 +33024,13 @@
         <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E72" t="s">
-        <v>2205</v>
+        <v>2202</v>
       </c>
       <c r="F72" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -33021,13 +33041,13 @@
         <v>1</v>
       </c>
       <c r="D73" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E73" t="s">
-        <v>2206</v>
+        <v>2203</v>
       </c>
       <c r="F73" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -33038,13 +33058,13 @@
         <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E74" t="s">
-        <v>2364</v>
+        <v>2358</v>
       </c>
       <c r="F74" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -33055,13 +33075,13 @@
         <v>1</v>
       </c>
       <c r="D75" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E75" t="s">
-        <v>2165</v>
+        <v>2162</v>
       </c>
       <c r="F75" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -33072,13 +33092,13 @@
         <v>1</v>
       </c>
       <c r="D76" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E76" t="s">
-        <v>2207</v>
+        <v>2204</v>
       </c>
       <c r="F76" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -33089,13 +33109,13 @@
         <v>1</v>
       </c>
       <c r="D77" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E77" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="F77" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -33106,13 +33126,13 @@
         <v>1</v>
       </c>
       <c r="D78" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E78" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="F78" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -33123,13 +33143,13 @@
         <v>1</v>
       </c>
       <c r="D79" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E79" t="s">
-        <v>2210</v>
+        <v>2207</v>
       </c>
       <c r="F79" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -33140,13 +33160,13 @@
         <v>1</v>
       </c>
       <c r="D80" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E80" t="s">
-        <v>2211</v>
+        <v>2208</v>
       </c>
       <c r="F80" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -33157,13 +33177,13 @@
         <v>1</v>
       </c>
       <c r="D81" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E81" t="s">
-        <v>2212</v>
+        <v>2209</v>
       </c>
       <c r="F81" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -33174,13 +33194,13 @@
         <v>1</v>
       </c>
       <c r="D82" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E82" t="s">
-        <v>2213</v>
+        <v>2210</v>
       </c>
       <c r="F82" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -33191,13 +33211,13 @@
         <v>1</v>
       </c>
       <c r="D83" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E83" t="s">
-        <v>2159</v>
+        <v>2156</v>
       </c>
       <c r="F83" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -33208,13 +33228,13 @@
         <v>1</v>
       </c>
       <c r="D84" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E84" t="s">
-        <v>2214</v>
+        <v>2211</v>
       </c>
       <c r="F84" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -33225,13 +33245,13 @@
         <v>1</v>
       </c>
       <c r="D85" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E85" t="s">
-        <v>2215</v>
+        <v>2212</v>
       </c>
       <c r="F85" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -33242,13 +33262,13 @@
         <v>1</v>
       </c>
       <c r="D86" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E86" t="s">
-        <v>2216</v>
+        <v>2213</v>
       </c>
       <c r="F86" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -33259,13 +33279,13 @@
         <v>1</v>
       </c>
       <c r="D87" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E87" t="s">
-        <v>2214</v>
+        <v>2211</v>
       </c>
       <c r="F87" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -33276,13 +33296,13 @@
         <v>1</v>
       </c>
       <c r="D88" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E88" t="s">
-        <v>2163</v>
+        <v>2160</v>
       </c>
       <c r="F88" t="s">
-        <v>2164</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -33293,13 +33313,13 @@
         <v>1</v>
       </c>
       <c r="D89" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E89" t="s">
-        <v>2217</v>
+        <v>2214</v>
       </c>
       <c r="F89" t="s">
-        <v>2162</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -33310,13 +33330,13 @@
         <v>1</v>
       </c>
       <c r="D90" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E90" t="s">
-        <v>2218</v>
+        <v>2215</v>
       </c>
       <c r="F90" t="s">
-        <v>2162</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -33327,13 +33347,13 @@
         <v>1</v>
       </c>
       <c r="D91" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E91" t="s">
-        <v>2219</v>
+        <v>2216</v>
       </c>
       <c r="F91" t="s">
-        <v>2196</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -33344,13 +33364,13 @@
         <v>1</v>
       </c>
       <c r="D92" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E92" t="s">
-        <v>2220</v>
+        <v>2217</v>
       </c>
       <c r="F92" t="s">
-        <v>2146</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -33361,13 +33381,13 @@
         <v>1</v>
       </c>
       <c r="D93" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E93" t="s">
-        <v>2221</v>
+        <v>2218</v>
       </c>
       <c r="F93" t="s">
-        <v>2146</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -33378,13 +33398,13 @@
         <v>1</v>
       </c>
       <c r="D94" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E94" t="s">
-        <v>2222</v>
+        <v>2219</v>
       </c>
       <c r="F94" t="s">
-        <v>2223</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -33395,13 +33415,13 @@
         <v>1</v>
       </c>
       <c r="D95" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E95" t="s">
-        <v>2224</v>
+        <v>2221</v>
       </c>
       <c r="F95" t="s">
-        <v>2225</v>
+        <v>2222</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -33412,13 +33432,13 @@
         <v>1</v>
       </c>
       <c r="D96" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="E96" t="s">
-        <v>2226</v>
+        <v>2223</v>
       </c>
       <c r="F96" t="s">
-        <v>2225</v>
+        <v>2222</v>
       </c>
     </row>
   </sheetData>
@@ -33441,69 +33461,69 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="26" t="s">
+        <v>2224</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>2225</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D1" s="26" t="s">
         <v>2227</v>
-      </c>
-      <c r="B1" s="26" t="s">
-        <v>2228</v>
-      </c>
-      <c r="C1" s="26" t="s">
-        <v>2229</v>
-      </c>
-      <c r="D1" s="26" t="s">
-        <v>2230</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="29" t="s">
-        <v>2231</v>
+        <v>2228</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D2" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="29" t="s">
-        <v>2233</v>
+        <v>2230</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="28" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="29" t="s">
-        <v>2164</v>
+        <v>2161</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>2234</v>
+        <v>2231</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>2164</v>
+        <v>2161</v>
       </c>
       <c r="D5" s="29">
         <v>13</v>
@@ -33511,27 +33531,27 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="28" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="28" t="s">
-        <v>2162</v>
+        <v>2159</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>2236</v>
+        <v>2233</v>
       </c>
       <c r="D7" s="29">
         <v>50</v>
@@ -33539,10 +33559,10 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="28" t="s">
-        <v>2223</v>
+        <v>2220</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C8" s="28" t="s">
         <v>964</v>
@@ -33553,10 +33573,10 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="30" t="s">
-        <v>2225</v>
+        <v>2222</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>964</v>
@@ -33567,10 +33587,10 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="28" t="s">
-        <v>2237</v>
+        <v>2234</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C10" s="28" t="s">
         <v>964</v>
@@ -33581,10 +33601,10 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="28" t="s">
-        <v>2238</v>
+        <v>2235</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C11" s="29" t="s">
         <v>964</v>
@@ -33595,10 +33615,10 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="29" t="s">
-        <v>2239</v>
+        <v>2236</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>964</v>
@@ -33609,10 +33629,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="29" t="s">
-        <v>2240</v>
+        <v>2237</v>
       </c>
       <c r="B13" s="29" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C13" s="29" t="s">
         <v>964</v>
@@ -33623,10 +33643,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="28" t="s">
-        <v>2241</v>
+        <v>2238</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C14" s="29" t="s">
         <v>964</v>
@@ -33637,10 +33657,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="28" t="s">
-        <v>2242</v>
+        <v>2239</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C15" s="29" t="s">
         <v>964</v>
@@ -33651,10 +33671,10 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="28" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C16" s="29" t="s">
         <v>459</v>
@@ -33665,10 +33685,10 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="28" t="s">
-        <v>2243</v>
+        <v>2240</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>989</v>
@@ -33679,10 +33699,10 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="30" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C18" s="29" t="s">
         <v>1428</v>
@@ -33693,10 +33713,10 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="28" t="s">
-        <v>2196</v>
+        <v>2193</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C19" s="28" t="s">
         <v>964</v>
@@ -33707,10 +33727,10 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="30" t="s">
-        <v>2244</v>
+        <v>2241</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C20" s="29" t="s">
         <v>964</v>
@@ -33721,10 +33741,10 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="29" t="s">
-        <v>2245</v>
+        <v>2242</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C21" s="29" t="s">
         <v>964</v>
@@ -33735,10 +33755,10 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="29" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C22" s="29" t="s">
         <v>964</v>
@@ -33749,10 +33769,10 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="28" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C23" s="29" t="s">
         <v>964</v>
@@ -33763,10 +33783,10 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="29" t="s">
-        <v>2150</v>
+        <v>2147</v>
       </c>
       <c r="B24" s="29" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C24" s="29" t="s">
         <v>964</v>
@@ -33777,10 +33797,10 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="28" t="s">
-        <v>2152</v>
+        <v>2149</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C25" s="29" t="s">
         <v>964</v>
@@ -33791,10 +33811,10 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="28" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C26" s="29" t="s">
         <v>459</v>
@@ -33805,10 +33825,10 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="28" t="s">
-        <v>2146</v>
+        <v>2143</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C27" s="29" t="s">
         <v>989</v>
@@ -33819,13 +33839,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="30" t="s">
-        <v>2247</v>
+        <v>2244</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D28" s="29">
         <v>0</v>
@@ -33833,10 +33853,10 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="30" t="s">
-        <v>2145</v>
+        <v>2142</v>
       </c>
       <c r="B29" s="29" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C29" s="29" t="s">
         <v>1428</v>
@@ -33847,10 +33867,10 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="28" t="s">
-        <v>2148</v>
+        <v>2145</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C30" s="28" t="s">
         <v>964</v>
@@ -33861,10 +33881,10 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="29" t="s">
-        <v>2156</v>
+        <v>2153</v>
       </c>
       <c r="B31" s="29" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C31" s="29" t="s">
         <v>964</v>
@@ -33875,10 +33895,10 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="28" t="s">
-        <v>2248</v>
+        <v>2245</v>
       </c>
       <c r="B32" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C32" s="28" t="s">
         <v>964</v>
@@ -33889,10 +33909,10 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="29" t="s">
-        <v>2157</v>
+        <v>2154</v>
       </c>
       <c r="B33" s="29" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C33" s="29" t="s">
         <v>964</v>
@@ -33903,10 +33923,10 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="29" t="s">
-        <v>2249</v>
+        <v>2246</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C34" s="29" t="s">
         <v>964</v>
@@ -33917,13 +33937,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="29" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
       <c r="B35" s="28" t="s">
-        <v>2234</v>
+        <v>2231</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
       <c r="D35" s="29">
         <v>12</v>
@@ -33931,13 +33951,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="29" t="s">
-        <v>2250</v>
+        <v>2247</v>
       </c>
       <c r="B36" s="28" t="s">
-        <v>2234</v>
+        <v>2231</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>2250</v>
+        <v>2247</v>
       </c>
       <c r="D36" s="29">
         <v>14</v>
@@ -33945,13 +33965,13 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="30" t="s">
-        <v>2251</v>
+        <v>2248</v>
       </c>
       <c r="B37" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D37" s="29">
         <v>0</v>
@@ -33959,13 +33979,13 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="28" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C38" s="28" t="s">
-        <v>2236</v>
+        <v>2233</v>
       </c>
       <c r="D38" s="29">
         <v>51</v>
@@ -33973,13 +33993,13 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="29" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>2234</v>
+        <v>2231</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
       <c r="D39" s="29">
         <v>11</v>
@@ -33987,27 +34007,27 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="28" t="s">
-        <v>2252</v>
+        <v>2249</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C40" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D40" s="29" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="28" t="s">
-        <v>2158</v>
+        <v>2155</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="C41" s="28" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
       <c r="D41" s="29">
         <v>0</v>
@@ -34015,10 +34035,10 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="29" t="s">
-        <v>2153</v>
+        <v>2150</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C42" s="29" t="s">
         <v>964</v>
@@ -34027,10 +34047,10 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="29" t="s">
-        <v>2154</v>
+        <v>2151</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="C43" s="29" t="s">
         <v>964</v>
@@ -34049,24 +34069,24 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="84.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="106.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>2381</v>
+        <v>2375</v>
       </c>
       <c r="B1" t="s">
-        <v>2382</v>
+        <v>2376</v>
       </c>
       <c r="C1" t="s">
-        <v>2383</v>
+        <v>2377</v>
       </c>
       <c r="D1" t="s">
         <v>2019</v>
@@ -34074,805 +34094,816 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>2257</v>
+        <v>2254</v>
       </c>
       <c r="B2" t="s">
-        <v>2067</v>
+        <v>2064</v>
       </c>
       <c r="C2" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>2333</v>
+        <v>2384</v>
       </c>
       <c r="B3" t="s">
-        <v>2256</v>
+        <v>2253</v>
       </c>
       <c r="C3" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>2355</v>
+        <v>2349</v>
       </c>
       <c r="B4" t="s">
-        <v>2326</v>
+        <v>2322</v>
       </c>
       <c r="C4" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>2265</v>
+        <v>2262</v>
       </c>
       <c r="B5" t="s">
         <v>2028</v>
       </c>
       <c r="C5" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>2266</v>
+        <v>2263</v>
       </c>
       <c r="B6" t="s">
-        <v>2267</v>
+        <v>2264</v>
       </c>
       <c r="C6" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>2272</v>
+        <v>2269</v>
       </c>
       <c r="B7" t="s">
-        <v>2273</v>
+        <v>2270</v>
       </c>
       <c r="C7" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>2337</v>
+        <v>2380</v>
       </c>
       <c r="B8" t="s">
-        <v>2338</v>
+        <v>2332</v>
       </c>
       <c r="C8" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>2339</v>
+        <v>2333</v>
       </c>
       <c r="B9" t="s">
-        <v>2273</v>
+        <v>2270</v>
       </c>
       <c r="C9" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>2266</v>
+        <v>2263</v>
       </c>
       <c r="B10" t="s">
-        <v>2267</v>
+        <v>2264</v>
       </c>
       <c r="C10" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>2332</v>
+        <v>2328</v>
       </c>
       <c r="B11" t="s">
-        <v>2331</v>
+        <v>2327</v>
       </c>
       <c r="C11" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>2340</v>
+        <v>2334</v>
       </c>
       <c r="B12" t="s">
-        <v>2341</v>
+        <v>2335</v>
       </c>
       <c r="C12" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="31" t="s">
-        <v>2342</v>
+        <v>2336</v>
       </c>
       <c r="B13" t="s">
-        <v>2089</v>
+        <v>2086</v>
       </c>
       <c r="C13" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>2343</v>
+        <v>2337</v>
       </c>
       <c r="B14" t="s">
-        <v>2344</v>
+        <v>2338</v>
       </c>
       <c r="C14" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>2345</v>
+        <v>2339</v>
       </c>
       <c r="B15" t="s">
-        <v>2346</v>
+        <v>2340</v>
       </c>
       <c r="C15" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="31" t="s">
-        <v>2347</v>
+        <v>2341</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>2348</v>
+        <v>2342</v>
       </c>
       <c r="C16" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>2349</v>
+        <v>2343</v>
       </c>
       <c r="B17" t="s">
-        <v>2350</v>
+        <v>2344</v>
       </c>
       <c r="C17" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>2351</v>
+        <v>2345</v>
       </c>
       <c r="B18" t="s">
-        <v>2352</v>
+        <v>2346</v>
       </c>
       <c r="C18" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>2354</v>
+        <v>2348</v>
       </c>
       <c r="B19" t="s">
-        <v>2353</v>
+        <v>2347</v>
       </c>
       <c r="C19" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>2250</v>
+        <v>2247</v>
       </c>
       <c r="B20" t="s">
-        <v>2358</v>
+        <v>2352</v>
       </c>
       <c r="C20" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>2374</v>
+        <v>2368</v>
       </c>
       <c r="B21" t="s">
-        <v>2254</v>
+        <v>2251</v>
       </c>
       <c r="C21" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>2320</v>
+        <v>2317</v>
       </c>
       <c r="B22" t="s">
-        <v>2255</v>
+        <v>2252</v>
       </c>
       <c r="C22" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>2253</v>
+        <v>2250</v>
       </c>
       <c r="B23" t="s">
-        <v>2357</v>
+        <v>2351</v>
       </c>
       <c r="C23" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>2336</v>
+        <v>2331</v>
       </c>
       <c r="B24" t="s">
-        <v>2258</v>
+        <v>2255</v>
       </c>
       <c r="C24" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>2365</v>
+        <v>2359</v>
       </c>
       <c r="B25" t="s">
-        <v>2259</v>
+        <v>2256</v>
       </c>
       <c r="C25" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>2260</v>
+        <v>2257</v>
       </c>
       <c r="B26" t="s">
-        <v>2261</v>
+        <v>2258</v>
       </c>
       <c r="C26" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>2262</v>
+        <v>2259</v>
       </c>
       <c r="B27" t="s">
-        <v>2269</v>
+        <v>2266</v>
       </c>
       <c r="C27" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>2303</v>
+        <v>2300</v>
       </c>
       <c r="B28" t="s">
-        <v>2263</v>
+        <v>2260</v>
       </c>
       <c r="C28" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>2264</v>
+        <v>2261</v>
       </c>
       <c r="B29" t="s">
         <v>2028</v>
       </c>
       <c r="C29" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>2266</v>
+        <v>2263</v>
       </c>
       <c r="B30" t="s">
-        <v>2267</v>
+        <v>2264</v>
       </c>
       <c r="C30" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>2361</v>
+        <v>2355</v>
       </c>
       <c r="B31" t="s">
-        <v>2236</v>
+        <v>2233</v>
       </c>
       <c r="C31" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>2268</v>
+        <v>2265</v>
       </c>
       <c r="B32" t="s">
         <v>989</v>
       </c>
       <c r="C32" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>2270</v>
+        <v>2267</v>
       </c>
       <c r="B33" t="s">
-        <v>2259</v>
+        <v>2256</v>
       </c>
       <c r="C33" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>2271</v>
+        <v>2268</v>
       </c>
       <c r="B34" t="s">
-        <v>2258</v>
+        <v>2255</v>
       </c>
       <c r="C34" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>2272</v>
+        <v>2269</v>
       </c>
       <c r="B35" t="s">
-        <v>2273</v>
+        <v>2270</v>
       </c>
       <c r="C35" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>2274</v>
+        <v>2271</v>
       </c>
       <c r="B36" t="s">
-        <v>2275</v>
+        <v>2272</v>
       </c>
       <c r="C36" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>2276</v>
+        <v>2273</v>
       </c>
       <c r="B37" t="s">
-        <v>2277</v>
+        <v>2274</v>
       </c>
       <c r="C37" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>2278</v>
+        <v>2275</v>
       </c>
       <c r="B38" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="C38" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>2280</v>
+        <v>2277</v>
       </c>
       <c r="B39" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="C39" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>2281</v>
+        <v>2278</v>
       </c>
       <c r="B40" t="s">
-        <v>2282</v>
+        <v>2279</v>
       </c>
       <c r="C40" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>2283</v>
+        <v>2280</v>
       </c>
       <c r="B41" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="C41" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>2302</v>
+        <v>2299</v>
       </c>
       <c r="B42" t="s">
-        <v>2284</v>
+        <v>2281</v>
       </c>
       <c r="C42" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>2285</v>
+        <v>2282</v>
       </c>
       <c r="B43" t="s">
-        <v>2286</v>
+        <v>2283</v>
       </c>
       <c r="C43" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>2287</v>
+        <v>2284</v>
       </c>
       <c r="B44" t="s">
-        <v>2259</v>
+        <v>2256</v>
       </c>
       <c r="C44" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>2288</v>
+        <v>2285</v>
       </c>
       <c r="B45" t="s">
-        <v>2289</v>
+        <v>2286</v>
       </c>
       <c r="C45" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>2290</v>
+        <v>2287</v>
       </c>
       <c r="B46" t="s">
-        <v>2291</v>
+        <v>2288</v>
       </c>
       <c r="C46" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>2292</v>
+        <v>2289</v>
       </c>
       <c r="B47" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="C47" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>2293</v>
+        <v>2290</v>
       </c>
       <c r="B48" t="s">
-        <v>2294</v>
+        <v>2291</v>
       </c>
       <c r="C48" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>2368</v>
+        <v>2362</v>
       </c>
       <c r="B49" t="s">
         <v>1888</v>
       </c>
       <c r="C49" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>2295</v>
+        <v>2292</v>
       </c>
       <c r="B50" t="s">
-        <v>2296</v>
+        <v>2293</v>
       </c>
       <c r="C50" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>2301</v>
+        <v>2298</v>
       </c>
       <c r="B51" t="s">
-        <v>2297</v>
+        <v>2294</v>
       </c>
       <c r="C51" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>2298</v>
+        <v>2295</v>
       </c>
       <c r="B52" t="s">
-        <v>2282</v>
+        <v>2279</v>
       </c>
       <c r="C52" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>2299</v>
+        <v>2296</v>
       </c>
       <c r="B53" t="s">
-        <v>2300</v>
+        <v>2297</v>
       </c>
       <c r="C53" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>2305</v>
+        <v>2302</v>
       </c>
       <c r="B54" t="s">
-        <v>2304</v>
+        <v>2301</v>
       </c>
       <c r="C54" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>2334</v>
+        <v>2329</v>
       </c>
       <c r="B55" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
       <c r="C55" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>2306</v>
+        <v>2303</v>
       </c>
       <c r="B56" t="s">
-        <v>2307</v>
+        <v>2304</v>
       </c>
       <c r="C56" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>2308</v>
+        <v>2305</v>
       </c>
       <c r="B57" t="s">
-        <v>2309</v>
+        <v>2306</v>
       </c>
       <c r="C57" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>2310</v>
+        <v>2307</v>
       </c>
       <c r="B58" t="s">
-        <v>2311</v>
+        <v>2308</v>
       </c>
       <c r="C58" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>2312</v>
+        <v>2309</v>
       </c>
       <c r="B59" t="s">
-        <v>2313</v>
+        <v>2310</v>
       </c>
       <c r="C59" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>2356</v>
+        <v>2350</v>
       </c>
       <c r="B60" t="s">
-        <v>2314</v>
+        <v>2311</v>
       </c>
       <c r="C60" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>2315</v>
+        <v>2312</v>
       </c>
       <c r="B61" t="s">
-        <v>2316</v>
+        <v>2313</v>
       </c>
       <c r="C61" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>2317</v>
+        <v>2314</v>
       </c>
       <c r="B62" t="s">
-        <v>2318</v>
+        <v>2315</v>
       </c>
       <c r="C62" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>2328</v>
+        <v>2324</v>
       </c>
       <c r="B63" t="s">
-        <v>2319</v>
+        <v>2316</v>
       </c>
       <c r="C63" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>2321</v>
+        <v>2379</v>
       </c>
       <c r="B64" t="s">
         <v>2029</v>
       </c>
       <c r="C64" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>2322</v>
+        <v>2318</v>
       </c>
       <c r="B65" t="s">
-        <v>2323</v>
+        <v>2319</v>
       </c>
       <c r="C65" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>2324</v>
+        <v>2320</v>
       </c>
       <c r="B66" t="s">
-        <v>2067</v>
+        <v>2064</v>
       </c>
       <c r="C66" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>2325</v>
+        <v>2321</v>
       </c>
       <c r="B67" t="s">
-        <v>2326</v>
+        <v>2322</v>
       </c>
       <c r="C67" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>2327</v>
+        <v>2323</v>
       </c>
       <c r="B68" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="C68" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>2329</v>
+        <v>2325</v>
       </c>
       <c r="B69" t="s">
-        <v>2330</v>
+        <v>2326</v>
       </c>
       <c r="C69" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>2332</v>
+        <v>2328</v>
       </c>
       <c r="B70" t="s">
-        <v>2331</v>
+        <v>2327</v>
       </c>
       <c r="C70" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>2335</v>
+        <v>2330</v>
       </c>
       <c r="B71" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
       <c r="C71" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>2362</v>
+        <v>2356</v>
       </c>
       <c r="B72" t="s">
-        <v>2363</v>
+        <v>2357</v>
       </c>
       <c r="C72" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>2366</v>
+        <v>2360</v>
       </c>
       <c r="B73" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="C73" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>2372</v>
+        <v>2366</v>
       </c>
       <c r="B74" t="s">
-        <v>2373</v>
+        <v>2367</v>
       </c>
       <c r="C74" t="s">
-        <v>2384</v>
+        <v>2378</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>2381</v>
+      </c>
+      <c r="B75" t="s">
+        <v>2382</v>
+      </c>
+      <c r="C75" t="s">
+        <v>2378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update master_table.xlsx with revised data
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Koding\tool-fcost\masters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\tool-fcost\masters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1332D24D-101B-4C37-82BC-567689E71700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -32,12 +31,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">part_list!$A$1:$B$1834</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">symptom!$A$1:$F$41</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4769" uniqueCount="2457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4851" uniqueCount="2483">
   <si>
     <t>part_used</t>
   </si>
@@ -6303,9 +6302,6 @@
     <t>action</t>
   </si>
   <si>
-    <t>ext|external|cairan|cleaning|semut|kotor|bersih|bersihkan|kardus rusak</t>
-  </si>
-  <si>
     <t>EXTERNAL</t>
   </si>
   <si>
@@ -6315,9 +6311,6 @@
     <t>CANCEL</t>
   </si>
   <si>
-    <t>cek normal|cek ok|unit cek ok|normal|fungsi ok|test fungsi|cek fungsi ok|cek unit|reposisi antena|antena</t>
-  </si>
-  <si>
     <t>USER</t>
   </si>
   <si>
@@ -6345,9 +6338,6 @@
     <t>FACTORY_RESET</t>
   </si>
   <si>
-    <t>setting|set up data|reset program|reset pabrik|stel ulang program|restart program|program ulang|reset unit|unit reset|reset ulang|riset program|data error-reset</t>
-  </si>
-  <si>
     <t>SETTING</t>
   </si>
   <si>
@@ -7408,12 +7398,99 @@
   </si>
   <si>
     <t>perbaikan remote|repair remote|resolder ulang sensor|remote</t>
+  </si>
+  <si>
+    <t>cek normal|cek ok|unit cek ok|normal|fungsi ok|test fungsi|cek fungsi ok|cek unit|reposisi antena|antena|DITEST OK</t>
+  </si>
+  <si>
+    <t>RESOLDER IC3101|RESOLDER IC7891|IC3101</t>
+  </si>
+  <si>
+    <t>lvds</t>
+  </si>
+  <si>
+    <t>setting|set up data|reset program|reset pabrik|stel ulang program|restart program|program ulang|reset unit|unit reset|reset ulang|riset program|data error-reset|RESTAR PROGRAM|RESET-ULANG|RESET MENU|RESET DATA|INSTALL ULANG</t>
+  </si>
+  <si>
+    <t>GANTI MAINBOARD|TU1102</t>
+  </si>
+  <si>
+    <t>PETIR</t>
+  </si>
+  <si>
+    <t>service power|repair power|repair regulator|repair modul|resolder power|resolder blok power|resolder modul power|resoldering modul|resoldering psu|resoldering|perbaikan power|perbaikan modul power|perbaiki power|ganti d1012|ganti dioda|REPAIR PCB|POWER</t>
+  </si>
+  <si>
+    <t>service main|repair main|repair main unit|repair pwb main|repair pwb|resolder main|resoldering main|resoldering mb|resolder ic7801|resolder ic memory|d7801|resolder blok main|resolder pwb|resolder pcb main|perbaikan main|perbaiki main|solder main|flash eprom|tuner|rusak main|REPAIR-MAIN</t>
+  </si>
+  <si>
+    <t>ext|external|cairan|cleaning|semut|kotor|bersih|bersihkan|kardus rusak|EKSTERNAL</t>
+  </si>
+  <si>
+    <t>RESOLDER R323|RESOLDER DIODA|Q4</t>
+  </si>
+  <si>
+    <t>COVER|FRAME</t>
+  </si>
+  <si>
+    <t>BACKLIGHT|BACK LIGHT|BACKLIG|LAMPU BACKLIG|LED BACKLIGHT|SOCKET BACKLIGHT|PANEL BACKLIGHT</t>
+  </si>
+  <si>
+    <t>LCD-PW|MATI TOTAL|MATI STANDBY|MATI-MATI|MATI$|STANDBY|POWER TIDAK FUNGSI</t>
+  </si>
+  <si>
+    <t>FUSE|DIODA|VARISTOR|CAPACITOR|TRANSISTOR|THERMOSTAT|Q702|Q4|REGULATOR|MODUL INVERTER|POWER|PWB RUSAK|RESOLDER MODUL|REPAIR MODUL</t>
+  </si>
+  <si>
+    <t>MAIN UNIT|MAINBOARD|MAIN-RUSAK|DIODA MAIN|IC MEMORY|COAX|AUDIO OUT|KABEL RCA|MICROPHONE|CONNECTOR AUDIO</t>
+  </si>
+  <si>
+    <t>TCON|TIKON</t>
+  </si>
+  <si>
+    <t>REPAIR_TCON_UNIT</t>
+  </si>
+  <si>
+    <t>REMOTE|REMOT|REMOTRE|DIREMOT|SENSOR ERROR|TIDAK RESPON.*REMOT</t>
+  </si>
+  <si>
+    <t>SENSOR IR|IR SENSOR|MODUL IR|SOCKET IR|REPAIR SENSOR IR|RESOLDER MODUL IR</t>
+  </si>
+  <si>
+    <t>KNOP|SWITCH POWE|TOMBOL</t>
+  </si>
+  <si>
+    <t>AC CORD|KABEL POWER</t>
+  </si>
+  <si>
+    <t>LUDS|LVDS|REPOSISI SOKET</t>
+  </si>
+  <si>
+    <t>RESET|SET ULANG|PENGATURAN PABRIK|CARI SIARAN|INSTAL ULANG|INSTALL ULANG|RESTART UNIT|RESTART|NO CHANGEL|CONNECTING ULANG|WIFI|INTERNET</t>
+  </si>
+  <si>
+    <t>FACTOYY|FACTORY</t>
+  </si>
+  <si>
+    <t>SUBT|SUBTITUSI|SUBSTITUSI|TKR|TUKAR|PENARIKAN DAN PENGANTARAN</t>
+  </si>
+  <si>
+    <t>CLAIM|KLAIM|GARANSI|TGG ACC|MAU DISERVICE|MAU TKR|CEK INFORMASI|DIKERJAKN KONS SENDIRI|DIKERJAKAN KONS SENDIRI</t>
+  </si>
+  <si>
+    <t>SEMUT|KENA SEMUT|BAUT KAKI PATAH|KOROSIF|RENGGANG</t>
+  </si>
+  <si>
+    <t>KOROSIF|BERSIHKAN SHEET|KOTOR|RENGGANG|LEPAS-BAUT|BAUT-PATAH|PASANG ULANG|PSNG ULANG</t>
+  </si>
+  <si>
+    <t>CEK FNGSI|CEK UNIT|CEK-UNIT|CEK FUNGSI|TES FUNGSI|OKE|OK</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="10">
     <font>
       <sz val="11"/>
@@ -7470,13 +7547,15 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7486,6 +7565,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -7526,7 +7611,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -7538,19 +7623,23 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10 3 14" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 13 2 2 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal 133 2 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 195" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 2 2" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Normal 315" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Normal 80" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 10 3 14" xfId="7"/>
+    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3"/>
+    <cellStyle name="Normal 13 2 2 2" xfId="4"/>
+    <cellStyle name="Normal 133 2 2" xfId="6"/>
+    <cellStyle name="Normal 195" xfId="8"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2 2" xfId="10"/>
+    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5"/>
+    <cellStyle name="Normal 315" xfId="9"/>
+    <cellStyle name="Normal 80" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -7827,7 +7916,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B1834"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -22508,13 +22597,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1834" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:B1834"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -23091,13 +23180,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B71" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:B71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -23140,13 +23229,13 @@
         <v>2021</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>2358</v>
+        <v>2355</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>2022</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>2359</v>
+        <v>2356</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -23160,13 +23249,13 @@
         <v>2021</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>2358</v>
+        <v>2355</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>2022</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>2359</v>
+        <v>2356</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -23180,13 +23269,13 @@
         <v>2021</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>2358</v>
+        <v>2355</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>2022</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>2359</v>
+        <v>2356</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -23200,13 +23289,13 @@
         <v>2021</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>2358</v>
+        <v>2355</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>2022</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>2359</v>
+        <v>2356</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -23220,13 +23309,13 @@
         <v>2021</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2360</v>
+        <v>2357</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>2023</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>2361</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -23240,13 +23329,13 @@
         <v>2021</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2360</v>
+        <v>2357</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>2023</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>2361</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -23260,13 +23349,13 @@
         <v>2021</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>2360</v>
+        <v>2357</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>2024</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>2361</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -23280,13 +23369,13 @@
         <v>2021</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>2360</v>
+        <v>2357</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>2024</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>2361</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -23300,13 +23389,13 @@
         <v>2021</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>2440</v>
+        <v>2437</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>2023</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>2362</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -23320,13 +23409,13 @@
         <v>2021</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>2436</v>
+        <v>2433</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>2025</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>2363</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -23346,7 +23435,7 @@
         <v>2027</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>2364</v>
+        <v>2361</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -23366,7 +23455,7 @@
         <v>2029</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>2365</v>
+        <v>2362</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -23386,7 +23475,7 @@
         <v>2031</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>2366</v>
+        <v>2363</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -23406,7 +23495,7 @@
         <v>2033</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>2367</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -23420,7 +23509,7 @@
         <v>2021</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>2441</v>
+        <v>2438</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>2034</v>
@@ -23440,13 +23529,13 @@
         <v>2021</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>2368</v>
+        <v>2365</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>2036</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>2369</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -23460,13 +23549,13 @@
         <v>2021</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>2370</v>
+        <v>2367</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>2023</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>2371</v>
+        <v>2368</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -23480,13 +23569,13 @@
         <v>2021</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>2372</v>
+        <v>2369</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>2037</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>2373</v>
+        <v>2370</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -23500,7 +23589,7 @@
         <v>2021</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>2447</v>
+        <v>2444</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>2036</v>
@@ -23526,7 +23615,7 @@
         <v>2040</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>2375</v>
+        <v>2372</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -23560,13 +23649,13 @@
         <v>2021</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>2376</v>
+        <v>2373</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>2044</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>2377</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -23580,13 +23669,13 @@
         <v>2021</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>2448</v>
+        <v>2445</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>2024</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>2378</v>
+        <v>2375</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -23600,7 +23689,7 @@
         <v>2021</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>2446</v>
+        <v>2443</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>2045</v>
@@ -23640,7 +23729,7 @@
         <v>2021</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>2379</v>
+        <v>2376</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>2050</v>
@@ -23700,7 +23789,7 @@
         <v>2021</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>2449</v>
+        <v>2446</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>2058</v>
@@ -23726,7 +23815,7 @@
         <v>2036</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>2380</v>
+        <v>2377</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -23740,7 +23829,7 @@
         <v>2021</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>2381</v>
+        <v>2378</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>2061</v>
@@ -23766,7 +23855,7 @@
         <v>2053</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>2382</v>
+        <v>2379</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -23800,13 +23889,13 @@
         <v>2021</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>2372</v>
+        <v>2369</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>2037</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>2383</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -23820,13 +23909,13 @@
         <v>2021</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>2384</v>
+        <v>2381</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>2058</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>2385</v>
+        <v>2382</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -23840,7 +23929,7 @@
         <v>2021</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>2379</v>
+        <v>2376</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>2050</v>
@@ -23860,13 +23949,13 @@
         <v>2021</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>2386</v>
+        <v>2383</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>2044</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>2387</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -23918,13 +24007,13 @@
         <v>2021</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>2388</v>
+        <v>2385</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>2022</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>2389</v>
+        <v>2386</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -23936,13 +24025,13 @@
         <v>2021</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>2433</v>
+        <v>2430</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>2024</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>2390</v>
+        <v>2387</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -23954,13 +24043,13 @@
         <v>2021</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>2432</v>
+        <v>2429</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>2044</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>2391</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -23972,13 +24061,13 @@
         <v>2021</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>2392</v>
+        <v>2389</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>2033</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>2393</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -23990,13 +24079,13 @@
         <v>2021</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>2394</v>
+        <v>2391</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>2061</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>2395</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -24008,13 +24097,13 @@
         <v>2021</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>2396</v>
+        <v>2393</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>2053</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>2397</v>
+        <v>2394</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -24026,13 +24115,13 @@
         <v>2021</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>2455</v>
+        <v>2452</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>2045</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>2398</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -24044,13 +24133,13 @@
         <v>2021</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>2399</v>
+        <v>2396</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>2037</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>2400</v>
+        <v>2397</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -24062,13 +24151,13 @@
         <v>2021</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>2401</v>
+        <v>2398</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>2025</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>2402</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -24080,13 +24169,13 @@
         <v>2021</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>2403</v>
+        <v>2400</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>2029</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>2404</v>
+        <v>2401</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -24098,13 +24187,13 @@
         <v>2021</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>2405</v>
+        <v>2402</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>2034</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>2406</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -24116,13 +24205,13 @@
         <v>2021</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>2407</v>
+        <v>2404</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>2056</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>2408</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -24134,13 +24223,13 @@
         <v>2021</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>2409</v>
+        <v>2406</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>2036</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>2410</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -24154,13 +24243,13 @@
         <v>2021</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>2411</v>
+        <v>2408</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>2025</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>2412</v>
+        <v>2409</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -24174,13 +24263,13 @@
         <v>2021</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>2413</v>
+        <v>2410</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>2027</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>2414</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -24194,13 +24283,13 @@
         <v>2021</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>2415</v>
+        <v>2412</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>2034</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>2416</v>
+        <v>2413</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -24212,13 +24301,13 @@
         <v>2021</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>2417</v>
+        <v>2414</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>2024</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>2418</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -24230,13 +24319,13 @@
         <v>2021</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>2419</v>
+        <v>2416</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>2025</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>2420</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -24248,13 +24337,13 @@
         <v>2021</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>2421</v>
+        <v>2418</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>2036</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>2422</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -24266,13 +24355,13 @@
         <v>2021</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>2423</v>
+        <v>2420</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>2058</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>2424</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -24284,13 +24373,13 @@
         <v>2021</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>2425</v>
+        <v>2422</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>2044</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>2426</v>
+        <v>2423</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -24304,13 +24393,13 @@
         <v>2021</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>2427</v>
+        <v>2424</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>2036</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>2428</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -24324,13 +24413,13 @@
         <v>2021</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>2429</v>
+        <v>2426</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>2044</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>2430</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -24344,7 +24433,7 @@
         <v>2021</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>2374</v>
+        <v>2371</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>2036</v>
@@ -24364,7 +24453,7 @@
         <v>2021</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>2374</v>
+        <v>2371</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>2036</v>
@@ -24384,7 +24473,7 @@
         <v>2021</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>2374</v>
+        <v>2371</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>2036</v>
@@ -24404,7 +24493,7 @@
         <v>2021</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>2374</v>
+        <v>2371</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>2036</v>
@@ -24447,7 +24536,7 @@
         <v>2060</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>2439</v>
+        <v>2436</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>2038</v>
@@ -24461,7 +24550,7 @@
         <v>2021</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>2374</v>
+        <v>2371</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>2036</v>
@@ -24496,10 +24585,10 @@
         <v>2021</v>
       </c>
       <c r="D72" t="s">
-        <v>2434</v>
+        <v>2431</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>2435</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -24513,10 +24602,10 @@
         <v>2021</v>
       </c>
       <c r="D73" t="s">
-        <v>2437</v>
+        <v>2434</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>2093</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -24528,7 +24617,7 @@
         <v>2021</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>2438</v>
+        <v>2435</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>2058</v>
@@ -24545,13 +24634,13 @@
         <v>2021</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>2444</v>
+        <v>2441</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>2058</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>2383</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -24565,7 +24654,7 @@
         <v>2021</v>
       </c>
       <c r="D76" t="s">
-        <v>2445</v>
+        <v>2442</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>2050</v>
@@ -24582,10 +24671,10 @@
         <v>2021</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>2451</v>
+        <v>2448</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>2452</v>
+        <v>2449</v>
       </c>
       <c r="F77" s="3"/>
     </row>
@@ -24597,20 +24686,20 @@
         <v>2021</v>
       </c>
       <c r="D78" t="s">
-        <v>2453</v>
+        <v>2450</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>2454</v>
+        <v>2451</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F41" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:F41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -24657,13 +24746,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -24704,14 +24793,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B4" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F46"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -24753,10 +24842,10 @@
         <v>2060</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>2462</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>2088</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>2089</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -24771,13 +24860,13 @@
         <v>2060</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>2089</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>2090</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>2091</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+    </row>
+    <row r="4" spans="1:6" ht="30">
       <c r="A4" s="1">
         <v>30</v>
       </c>
@@ -24789,10 +24878,10 @@
         <v>2060</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>2092</v>
+        <v>2454</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>2093</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -24807,10 +24896,10 @@
         <v>2060</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>2094</v>
+        <v>2092</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>2095</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -24825,10 +24914,10 @@
         <v>2060</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>2096</v>
+        <v>2094</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>2097</v>
+        <v>2095</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -24843,10 +24932,10 @@
         <v>2060</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>2098</v>
+        <v>2096</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>2099</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -24861,13 +24950,13 @@
         <v>2060</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>2100</v>
+        <v>2098</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>2101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="30">
+        <v>2099</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="45">
       <c r="A9" s="1">
         <v>80</v>
       </c>
@@ -24879,10 +24968,10 @@
         <v>2060</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>2102</v>
+        <v>2457</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>2103</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -24899,10 +24988,10 @@
         <v>2060</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>2104</v>
+        <v>2101</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>2105</v>
+        <v>2102</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -24919,10 +25008,10 @@
         <v>2060</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>2106</v>
+        <v>2103</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>2107</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -24939,10 +25028,10 @@
         <v>2060</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>2108</v>
+        <v>2105</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>2109</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -24959,10 +25048,10 @@
         <v>2060</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>2110</v>
+        <v>2107</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>2111</v>
+        <v>2108</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -24979,10 +25068,10 @@
         <v>2060</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>2112</v>
+        <v>2109</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>2113</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -24999,10 +25088,10 @@
         <v>2060</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>2114</v>
+        <v>2111</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>2115</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -25019,10 +25108,10 @@
         <v>2060</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>2116</v>
+        <v>2113</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>2117</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -25039,10 +25128,10 @@
         <v>2060</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>2118</v>
+        <v>2115</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>2119</v>
+        <v>2116</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -25059,10 +25148,10 @@
         <v>2060</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>2120</v>
+        <v>2117</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -25079,10 +25168,10 @@
         <v>2060</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>2120</v>
+        <v>2117</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -25099,10 +25188,10 @@
         <v>2060</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>2122</v>
+        <v>2119</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>2123</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -25119,10 +25208,10 @@
         <v>2060</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>2124</v>
+        <v>2121</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>2125</v>
+        <v>2122</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -25139,10 +25228,10 @@
         <v>2060</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>2126</v>
+        <v>2123</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>2127</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="45">
@@ -25159,10 +25248,10 @@
         <v>2060</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>2128</v>
+        <v>2125</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>2129</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="45">
@@ -25179,10 +25268,10 @@
         <v>2060</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>2130</v>
+        <v>2127</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>2131</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -25199,10 +25288,10 @@
         <v>2060</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>2132</v>
+        <v>2129</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>2133</v>
+        <v>2130</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -25219,10 +25308,10 @@
         <v>2060</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>2134</v>
+        <v>2131</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>2135</v>
+        <v>2132</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -25239,10 +25328,10 @@
         <v>2060</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>2136</v>
+        <v>2133</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -25259,10 +25348,10 @@
         <v>2060</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>2136</v>
+        <v>2133</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -25282,7 +25371,7 @@
         <v>2060</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>2107</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -25302,7 +25391,7 @@
         <v>2060</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>2105</v>
+        <v>2102</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -25322,7 +25411,7 @@
         <v>2060</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>2109</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -25342,7 +25431,7 @@
         <v>2060</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>2111</v>
+        <v>2108</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -25362,7 +25451,7 @@
         <v>2060</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>2131</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -25382,7 +25471,7 @@
         <v>2060</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>2113</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -25402,7 +25491,7 @@
         <v>2060</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>2129</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -25422,7 +25511,7 @@
         <v>2060</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>2115</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -25442,7 +25531,7 @@
         <v>2060</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>2119</v>
+        <v>2116</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -25462,7 +25551,7 @@
         <v>2060</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>2117</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -25482,7 +25571,7 @@
         <v>2060</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -25502,7 +25591,7 @@
         <v>2060</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -25522,7 +25611,7 @@
         <v>2060</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>2123</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -25542,7 +25631,7 @@
         <v>2060</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>2125</v>
+        <v>2122</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -25562,7 +25651,7 @@
         <v>2060</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>2127</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -25577,13 +25666,13 @@
         <v>2060</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>2456</v>
+        <v>2453</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>2133</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="45">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="60">
       <c r="A45" s="1">
         <v>440</v>
       </c>
@@ -25595,10 +25684,10 @@
         <v>2060</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>2128</v>
+        <v>2461</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>2129</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="45">
@@ -25613,20 +25702,502 @@
         <v>2060</v>
       </c>
       <c r="E46" s="1" t="s">
+        <v>2460</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>2128</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="1">
+        <v>460</v>
+      </c>
+      <c r="B47" s="1">
+        <v>1</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E47" t="s">
+        <v>2455</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>2126</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="1">
+        <v>470</v>
+      </c>
+      <c r="B48" s="1">
+        <v>1</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>2463</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>2128</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="1">
+        <v>480</v>
+      </c>
+      <c r="B49" s="1">
+        <v>1</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E49" t="s">
+        <v>2458</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>2126</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="1">
+        <v>490</v>
+      </c>
+      <c r="B50" s="1">
+        <v>1</v>
+      </c>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>2456</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>2132</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="1">
+        <v>500</v>
+      </c>
+      <c r="B51" s="1">
+        <v>1</v>
+      </c>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E51" t="s">
+        <v>2464</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>2134</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="1">
+        <v>510</v>
+      </c>
+      <c r="B52" s="1">
+        <v>1</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>2462</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="1">
+        <v>520</v>
+      </c>
+      <c r="B53" s="1">
+        <v>1</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1" t="s">
+        <v>2462</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="1">
+        <v>530</v>
+      </c>
+      <c r="B54" s="1">
+        <v>1</v>
+      </c>
+      <c r="D54" t="s">
+        <v>2459</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="1">
+        <v>540</v>
+      </c>
+      <c r="B55" s="1">
+        <v>1</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E55" t="s">
+        <v>2459</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="1">
+        <v>550</v>
+      </c>
+      <c r="B56" s="1">
+        <v>1</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E56" t="s">
+        <v>2188</v>
+      </c>
+      <c r="F56" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="5">
+        <v>560</v>
+      </c>
+      <c r="B57" s="5">
+        <v>1</v>
+      </c>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>2465</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>2157</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="5">
+        <v>570</v>
+      </c>
+      <c r="B58" s="6">
+        <v>1</v>
+      </c>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6" t="s">
+        <v>2466</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>2128</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="5">
+        <v>580</v>
+      </c>
+      <c r="B59" s="6">
+        <v>1</v>
+      </c>
+      <c r="C59" s="6"/>
+      <c r="D59" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>2467</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>2128</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="5">
+        <v>590</v>
+      </c>
+      <c r="B60" s="6">
+        <v>1</v>
+      </c>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>2468</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>2126</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="5">
+        <v>600</v>
+      </c>
+      <c r="B61" s="6">
+        <v>1</v>
+      </c>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>2469</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>2470</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" s="5">
+        <v>610</v>
+      </c>
+      <c r="B62" s="6">
+        <v>1</v>
+      </c>
+      <c r="C62" s="6"/>
+      <c r="D62" s="6" t="s">
+        <v>2471</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="F62" s="6" t="s">
         <v>2130</v>
       </c>
-      <c r="F46" s="1" t="s">
-        <v>2131</v>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="5">
+        <v>620</v>
+      </c>
+      <c r="B63" s="6">
+        <v>1</v>
+      </c>
+      <c r="C63" s="6"/>
+      <c r="D63" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="5">
+        <v>630</v>
+      </c>
+      <c r="B64" s="6">
+        <v>1</v>
+      </c>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>2473</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>2124</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="5">
+        <v>640</v>
+      </c>
+      <c r="B65" s="6">
+        <v>1</v>
+      </c>
+      <c r="C65" s="6"/>
+      <c r="D65" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>2474</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>2091</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" s="5">
+        <v>650</v>
+      </c>
+      <c r="B66" s="6">
+        <v>1</v>
+      </c>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>2475</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>2132</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" s="5">
+        <v>660</v>
+      </c>
+      <c r="B67" s="6">
+        <v>1</v>
+      </c>
+      <c r="C67" s="6"/>
+      <c r="D67" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>2476</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" s="5">
+        <v>670</v>
+      </c>
+      <c r="B68" s="6">
+        <v>1</v>
+      </c>
+      <c r="C68" s="6"/>
+      <c r="D68" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>2477</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>2099</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" s="5">
+        <v>680</v>
+      </c>
+      <c r="B69" s="6">
+        <v>1</v>
+      </c>
+      <c r="C69" s="6"/>
+      <c r="D69" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>2478</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" s="5">
+        <v>690</v>
+      </c>
+      <c r="B70" s="6">
+        <v>1</v>
+      </c>
+      <c r="C70" s="6"/>
+      <c r="D70" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>2479</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" s="5">
+        <v>700</v>
+      </c>
+      <c r="B71" s="6">
+        <v>1</v>
+      </c>
+      <c r="C71" s="6"/>
+      <c r="D71" s="6" t="s">
+        <v>2480</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="5">
+        <v>710</v>
+      </c>
+      <c r="B72" s="6">
+        <v>1</v>
+      </c>
+      <c r="C72" s="6"/>
+      <c r="D72" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>2481</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="5">
+        <v>720</v>
+      </c>
+      <c r="B73" s="6">
+        <v>1</v>
+      </c>
+      <c r="C73" s="6"/>
+      <c r="D73" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>2482</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>2091</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F43" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:F43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -25638,584 +26209,584 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
+        <v>2135</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2136</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2137</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2138</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>2139</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2140</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2141</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>2091</v>
+        <v>2090</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>2097</v>
+        <v>2095</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>2145</v>
+        <v>2142</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>2097</v>
+        <v>2095</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>2146</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>2089</v>
+        <v>2088</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>2101</v>
+        <v>2099</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>2148</v>
+        <v>2145</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>2150</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>2135</v>
+        <v>2132</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>2152</v>
+        <v>2149</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>2153</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
-        <v>2154</v>
+        <v>2151</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1" t="s">
-        <v>2156</v>
+        <v>2153</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>2157</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1" t="s">
-        <v>2158</v>
+        <v>2155</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>2159</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>2161</v>
+        <v>2158</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1" t="s">
-        <v>2162</v>
+        <v>2159</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1" t="s">
-        <v>2129</v>
+        <v>2126</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>459</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>2163</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1" t="s">
-        <v>2164</v>
+        <v>2161</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>989</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>2165</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="1" t="s">
-        <v>2131</v>
+        <v>2128</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>1429</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1" t="s">
-        <v>2133</v>
+        <v>2130</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>2167</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1" t="s">
-        <v>2168</v>
+        <v>2165</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>2169</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1" t="s">
-        <v>2170</v>
+        <v>2167</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>2171</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1" t="s">
-        <v>2172</v>
+        <v>2169</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>2173</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>2174</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="1" t="s">
-        <v>2113</v>
+        <v>2110</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>2175</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1" t="s">
-        <v>2115</v>
+        <v>2112</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>2176</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="1" t="s">
-        <v>2109</v>
+        <v>2106</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>459</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>2177</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="1" t="s">
-        <v>2105</v>
+        <v>2102</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>989</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>2178</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="30">
       <c r="A28" s="1" t="s">
-        <v>2179</v>
+        <v>2176</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="1" t="s">
-        <v>2107</v>
+        <v>2104</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>1429</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>2180</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="1" t="s">
-        <v>2111</v>
+        <v>2108</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>2181</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1" t="s">
-        <v>2123</v>
+        <v>2120</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>2182</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1" t="s">
-        <v>2183</v>
+        <v>2180</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>2184</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1" t="s">
-        <v>2125</v>
+        <v>2122</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>2185</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1" t="s">
-        <v>2186</v>
+        <v>2183</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>964</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>2187</v>
+        <v>2184</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1" t="s">
-        <v>2103</v>
+        <v>2100</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>2145</v>
+        <v>2142</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>2103</v>
+        <v>2100</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>2188</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1" t="s">
-        <v>2189</v>
+        <v>2186</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>2145</v>
+        <v>2142</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>2189</v>
+        <v>2186</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>2190</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="1" t="s">
-        <v>2191</v>
+        <v>2188</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1" t="s">
-        <v>2099</v>
+        <v>2097</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>2148</v>
+        <v>2145</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>2192</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1" t="s">
-        <v>2093</v>
+        <v>2091</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>2145</v>
+        <v>2142</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>2093</v>
+        <v>2091</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>2193</v>
+        <v>2190</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1" t="s">
-        <v>2194</v>
+        <v>2191</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1" t="s">
-        <v>2095</v>
+        <v>2093</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>2155</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="1" t="s">
-        <v>2119</v>
+        <v>2116</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>964</v>
@@ -26224,10 +26795,10 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1" t="s">
-        <v>2117</v>
+        <v>2114</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>964</v>
@@ -26235,13 +26806,13 @@
       <c r="D43" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D43" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:D43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -26253,13 +26824,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>2195</v>
+        <v>2192</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2196</v>
+        <v>2193</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2197</v>
+        <v>2194</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2020</v>
@@ -26267,7 +26838,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>2198</v>
+        <v>2195</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2037</v>
@@ -26276,110 +26847,110 @@
         <v>2019</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>2199</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45">
       <c r="A3" s="1" t="s">
-        <v>2200</v>
+        <v>2197</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>2201</v>
+        <v>2198</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>2202</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>2431</v>
+        <v>2428</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>2203</v>
+        <v>2200</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>2204</v>
+        <v>2201</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>2205</v>
+        <v>2202</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>2206</v>
+        <v>2203</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>2207</v>
+        <v>2204</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>2210</v>
+        <v>2207</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>2211</v>
+        <v>2208</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>2212</v>
+        <v>2209</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>2213</v>
+        <v>2210</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>2214</v>
+        <v>2211</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>2215</v>
+        <v>2212</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>2216</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>2189</v>
+        <v>2186</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>2217</v>
+        <v>2214</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>2218</v>
+        <v>2215</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>2219</v>
+        <v>2216</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>2045</v>
@@ -26388,68 +26959,68 @@
         <v>2019</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>2220</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
-        <v>2221</v>
+        <v>2218</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>2222</v>
+        <v>2219</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>2223</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1" t="s">
-        <v>2224</v>
+        <v>2221</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>2225</v>
+        <v>2222</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>2226</v>
+        <v>2223</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1" t="s">
-        <v>2227</v>
+        <v>2224</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>2228</v>
+        <v>2225</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>2229</v>
+        <v>2226</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>2230</v>
+        <v>2227</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>2231</v>
+        <v>2228</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>2232</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1" t="s">
-        <v>2233</v>
+        <v>2230</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>2023</v>
@@ -26458,624 +27029,624 @@
         <v>2019</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>2234</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1" t="s">
-        <v>2235</v>
+        <v>2232</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>2236</v>
+        <v>2233</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>2237</v>
+        <v>2234</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1" t="s">
-        <v>2238</v>
+        <v>2235</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>2239</v>
+        <v>2236</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>2240</v>
+        <v>2237</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="1" t="s">
-        <v>2241</v>
+        <v>2238</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>2242</v>
+        <v>2239</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>2019</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>2243</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1" t="s">
+        <v>2241</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>2243</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>2244</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>2245</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>2246</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>2247</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1" t="s">
-        <v>2248</v>
+        <v>2245</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>2249</v>
+        <v>2246</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>2250</v>
+        <v>2247</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1" t="s">
-        <v>2251</v>
+        <v>2248</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>2252</v>
+        <v>2249</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>2253</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1" t="s">
-        <v>2254</v>
+        <v>2251</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>2255</v>
+        <v>2252</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>2256</v>
+        <v>2253</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1" t="s">
-        <v>2257</v>
+        <v>2254</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>2258</v>
+        <v>2255</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>2259</v>
+        <v>2256</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="1" t="s">
-        <v>2260</v>
+        <v>2257</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>2261</v>
+        <v>2258</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>2262</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1" t="s">
-        <v>2263</v>
+        <v>2260</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>2264</v>
+        <v>2261</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>2265</v>
+        <v>2262</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="1" t="s">
-        <v>2266</v>
+        <v>2263</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>2267</v>
+        <v>2264</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>2268</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="1" t="s">
-        <v>2269</v>
+        <v>2266</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>2270</v>
+        <v>2267</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>2271</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="1" t="s">
-        <v>2272</v>
+        <v>2269</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>2148</v>
+        <v>2145</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>2273</v>
+        <v>2270</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="1" t="s">
-        <v>2274</v>
+        <v>2271</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>989</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>2275</v>
+        <v>2272</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="1" t="s">
-        <v>2276</v>
+        <v>2273</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>2258</v>
+        <v>2255</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>2277</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1" t="s">
-        <v>2278</v>
+        <v>2275</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>2280</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1" t="s">
-        <v>2281</v>
+        <v>2278</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>2282</v>
+        <v>2279</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>2283</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="30">
       <c r="A33" s="1" t="s">
-        <v>2284</v>
+        <v>2281</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>2285</v>
+        <v>2282</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>2286</v>
+        <v>2283</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1" t="s">
-        <v>2287</v>
+        <v>2284</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>2288</v>
+        <v>2285</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>2289</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1" t="s">
-        <v>2290</v>
+        <v>2287</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>2291</v>
+        <v>2288</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>2292</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1" t="s">
-        <v>2293</v>
+        <v>2290</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>2294</v>
+        <v>2291</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>2295</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="1" t="s">
-        <v>2296</v>
+        <v>2293</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>2297</v>
+        <v>2294</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>2298</v>
+        <v>2295</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1" t="s">
-        <v>2299</v>
+        <v>2296</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>2300</v>
+        <v>2297</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>2301</v>
+        <v>2298</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1" t="s">
-        <v>2302</v>
+        <v>2299</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>1889</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>2303</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1" t="s">
-        <v>2304</v>
+        <v>2301</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>2305</v>
+        <v>2302</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>2306</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1" t="s">
-        <v>2307</v>
+        <v>2304</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>2308</v>
+        <v>2305</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>2309</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="1" t="s">
-        <v>2310</v>
+        <v>2307</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>2311</v>
+        <v>2308</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>2312</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1" t="s">
-        <v>2313</v>
+        <v>2310</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>2314</v>
+        <v>2311</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>2315</v>
+        <v>2312</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="1" t="s">
-        <v>2316</v>
+        <v>2313</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>2103</v>
+        <v>2100</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>2317</v>
+        <v>2314</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="1" t="s">
-        <v>2318</v>
+        <v>2315</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>2319</v>
+        <v>2316</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>2320</v>
+        <v>2317</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="1" t="s">
-        <v>2321</v>
+        <v>2318</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>2322</v>
+        <v>2319</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>2323</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1" t="s">
-        <v>2324</v>
+        <v>2321</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>2325</v>
+        <v>2322</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>2326</v>
+        <v>2323</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="1" t="s">
-        <v>2327</v>
+        <v>2324</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>2328</v>
+        <v>2325</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>2329</v>
+        <v>2326</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="1" t="s">
-        <v>2330</v>
+        <v>2327</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>2331</v>
+        <v>2328</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>2332</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="1" t="s">
-        <v>2333</v>
+        <v>2330</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>2334</v>
+        <v>2331</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>2335</v>
+        <v>2332</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="1" t="s">
-        <v>2336</v>
+        <v>2333</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>2337</v>
+        <v>2334</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>2338</v>
+        <v>2335</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="1" t="s">
-        <v>2339</v>
+        <v>2336</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>2099</v>
+        <v>2097</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>2340</v>
+        <v>2337</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="1" t="s">
-        <v>2341</v>
+        <v>2338</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>2342</v>
+        <v>2339</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>2343</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="1" t="s">
-        <v>2450</v>
+        <v>2447</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>2344</v>
+        <v>2341</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>2345</v>
+        <v>2342</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="1" t="s">
-        <v>2346</v>
+        <v>2343</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>2347</v>
+        <v>2344</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>2348</v>
+        <v>2345</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="1" t="s">
-        <v>2349</v>
+        <v>2346</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>2350</v>
+        <v>2347</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>2351</v>
+        <v>2348</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="1" t="s">
-        <v>2352</v>
+        <v>2349</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>2353</v>
+        <v>2350</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>2354</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="1" t="s">
-        <v>2355</v>
+        <v>2352</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>2356</v>
+        <v>2353</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>2246</v>
+        <v>2243</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>2357</v>
+        <v>2354</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>2442</v>
+        <v>2439</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>2443</v>
+        <v>2440</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>2019</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D58" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
+  <autoFilter ref="A1:D58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update master_table.xlsx with new data
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4851" uniqueCount="2483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4923" uniqueCount="2521">
   <si>
     <t>part_used</t>
   </si>
@@ -7485,6 +7485,120 @@
   </si>
   <si>
     <t>CEK FNGSI|CEK UNIT|CEK-UNIT|CEK FUNGSI|TES FUNGSI|OKE|OK</t>
+  </si>
+  <si>
+    <t>2TC45AD1X</t>
+  </si>
+  <si>
+    <t>2TC45AE1X</t>
+  </si>
+  <si>
+    <t>4TC50AH1X</t>
+  </si>
+  <si>
+    <t>4TC50DL1X</t>
+  </si>
+  <si>
+    <t>4TC50FJ1X</t>
+  </si>
+  <si>
+    <t>4TC55EJ2X</t>
+  </si>
+  <si>
+    <t>4TC55EK2X</t>
+  </si>
+  <si>
+    <t>4TC55FJ1X</t>
+  </si>
+  <si>
+    <t>4TC55FL1X</t>
+  </si>
+  <si>
+    <t>4TC55GN7000X</t>
+  </si>
+  <si>
+    <t>4TC60AH1X</t>
+  </si>
+  <si>
+    <t>4TC60BK1X</t>
+  </si>
+  <si>
+    <t>4TC60CH1X</t>
+  </si>
+  <si>
+    <t>4TC60CK1X</t>
+  </si>
+  <si>
+    <t>4TC60DK1X</t>
+  </si>
+  <si>
+    <t>4TC60DL1X</t>
+  </si>
+  <si>
+    <t>4TC65CK1X</t>
+  </si>
+  <si>
+    <t>4TC65DK1X</t>
+  </si>
+  <si>
+    <t>4TC65DL1X</t>
+  </si>
+  <si>
+    <t>4TC65FJ1X</t>
+  </si>
+  <si>
+    <t>4TC65FK1X</t>
+  </si>
+  <si>
+    <t>4TC65FL1X</t>
+  </si>
+  <si>
+    <t>4TC65GU8500X</t>
+  </si>
+  <si>
+    <t>4TC70AH1X</t>
+  </si>
+  <si>
+    <t>4TC70AL1X</t>
+  </si>
+  <si>
+    <t>4TC70BK1X</t>
+  </si>
+  <si>
+    <t>4TC70CK3X</t>
+  </si>
+  <si>
+    <t>4TC70DK1X</t>
+  </si>
+  <si>
+    <t>4TC70DL1X</t>
+  </si>
+  <si>
+    <t>4TC75EK2X</t>
+  </si>
+  <si>
+    <t>4TC75FJ1X</t>
+  </si>
+  <si>
+    <t>4TC85HN7000X</t>
+  </si>
+  <si>
+    <t>4TC98HN7000X</t>
+  </si>
+  <si>
+    <t>8TC70DW1X</t>
+  </si>
+  <si>
+    <t>LC32LE375X</t>
+  </si>
+  <si>
+    <t>LC40LE380X</t>
+  </si>
+  <si>
+    <t>SMM</t>
+  </si>
+  <si>
+    <t>AETECH</t>
   </si>
 </sst>
 </file>
@@ -22604,7 +22718,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -23179,8 +23293,295 @@
         <v>2014</v>
       </c>
     </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>2483</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>2484</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>2485</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>2486</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
+        <v>2487</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="s">
+        <v>2488</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>2489</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>2490</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>2491</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>2492</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>2493</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
+        <v>2494</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" t="s">
+        <v>2495</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>2496</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>2497</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
+        <v>2498</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" t="s">
+        <v>2499</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>2500</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>2501</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>2502</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>2503</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>2504</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>2505</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>2506</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>2507</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>2508</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
+        <v>2509</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
+        <v>2510</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>2511</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
+        <v>2512</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" t="s">
+        <v>2513</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" t="s">
+        <v>2514</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>1943</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" t="s">
+        <v>2515</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>1943</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" t="s">
+        <v>2516</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" t="s">
+        <v>2517</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" t="s">
+        <v>2518</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>2519</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: Enhance summary result workbook output
Support configurable summary result formatting and validation so generated workbooks match the updated FCOST output requirements.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\tool-fcost\masters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Koding\tool-fcost\masters\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2DE972C-D48D-422D-92E8-183C47B625F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -7586,9 +7587,6 @@
     <t>TIDAK BISA INTERNET|KERUSAKAN INTERNET</t>
   </si>
   <si>
-    <t>goyang|bergelombang|delay|dominan|merah|putih|blue|warna|kualitas gambar|slow motion|gambar bermasalah|layar bermasalah|bergerak|berembun|BERMASALAH|</t>
-  </si>
-  <si>
     <t>gambar berganti sendiri|gambar blur|gambar klise|layar merah|gambar tidak baik|warna|GAMBAR TIDAK NORMAL|KEDIP|TAMPILAN DELAY|berkedip|GAMBAR BERBAYANG</t>
   </si>
   <si>
@@ -7605,12 +7603,15 @@
   </si>
   <si>
     <t>cek normal|cek ok|unit cek ok|normal|fungsi ok|test fungsi|cek fungsi ok|cek unit|reposisi antena|antena|DITEST OK|TIDAK ADA KERUSAKAN</t>
+  </si>
+  <si>
+    <t>goyang|bergelombang|delay|dominan|merah|putih|blue|warna|kualitas gambar|slow motion|gambar bermasalah|layar bermasalah|bergerak|berembun|BERMASALAH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="10">
     <font>
       <sz val="11"/>
@@ -7731,7 +7732,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -7746,25 +7747,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10 3 14" xfId="7"/>
-    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3"/>
-    <cellStyle name="Normal 13 2 2 2" xfId="4"/>
-    <cellStyle name="Normal 133 2 2" xfId="6"/>
-    <cellStyle name="Normal 195" xfId="8"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 2 2" xfId="10"/>
-    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5"/>
-    <cellStyle name="Normal 315" xfId="9"/>
-    <cellStyle name="Normal 80" xfId="1"/>
+    <cellStyle name="Normal 10 3 14" xfId="7" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Normal 13 2 2 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 133 2 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 195" xfId="8" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Normal 2 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Normal 315" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Normal 80" xfId="1" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -8041,7 +8038,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B1834"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -22722,13 +22719,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1834"/>
+  <autoFilter ref="A1:B1834" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -23598,7 +23595,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -23955,7 +23952,7 @@
         <v>2021</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>2035</v>
@@ -24155,7 +24152,7 @@
         <v>2021</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>2057</v>
@@ -24231,7 +24228,7 @@
         <v>2021</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>2023</v>
@@ -24271,7 +24268,7 @@
         <v>2021</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>2516</v>
+        <v>2522</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>2025</v>
@@ -24291,7 +24288,7 @@
         <v>2021</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>2026</v>
@@ -24957,7 +24954,7 @@
       <c r="A70" s="3">
         <v>520</v>
       </c>
-      <c r="B70" s="9"/>
+      <c r="B70" s="3"/>
       <c r="C70" s="3" t="s">
         <v>2021</v>
       </c>
@@ -25083,7 +25080,6 @@
       <c r="A77" s="3">
         <v>700</v>
       </c>
-      <c r="B77" s="8"/>
       <c r="C77" s="3" t="s">
         <v>2021</v>
       </c>
@@ -25125,8 +25121,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F41">
-    <sortState ref="A2:F79">
+  <autoFilter ref="A1:F41" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F79">
       <sortCondition ref="B1:B41"/>
     </sortState>
   </autoFilter>
@@ -25135,7 +25131,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -25182,13 +25178,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
+  <autoFilter ref="A1:B5" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -25229,13 +25225,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B4"/>
+  <autoFilter ref="A1:B4" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -25580,7 +25576,7 @@
         <v>2059</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>2521</v>
+        <v>2520</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>2124</v>
@@ -26566,7 +26562,7 @@
         <v>2059</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>2522</v>
+        <v>2521</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>2090</v>
@@ -26627,8 +26623,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F43">
-    <sortState ref="A2:F73">
+  <autoFilter ref="A1:F43" xr:uid="{00000000-0009-0000-0000-000005000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F73">
       <sortCondition descending="1" ref="C1:C43"/>
     </sortState>
   </autoFilter>
@@ -26637,7 +26633,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -27246,13 +27242,13 @@
       <c r="D43" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D43"/>
+  <autoFilter ref="A1:D43" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -28086,7 +28082,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D58"/>
+  <autoFilter ref="A1:D58" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: Update master_table.xlsx with new data
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Koding\tool-fcost\masters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\tool-fcost\masters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2DE972C-D48D-422D-92E8-183C47B625F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4927" uniqueCount="2523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4931" uniqueCount="2525">
   <si>
     <t>part_used</t>
   </si>
@@ -7606,13 +7605,19 @@
   </si>
   <si>
     <t>goyang|bergelombang|delay|dominan|merah|putih|blue|warna|kualitas gambar|slow motion|gambar bermasalah|layar bermasalah|bergerak|berembun|BERMASALAH</t>
+  </si>
+  <si>
+    <t>4TC75GU8500X</t>
+  </si>
+  <si>
+    <t>4TC85HU8500X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7675,8 +7680,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7692,6 +7701,11 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -7732,7 +7746,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -7749,19 +7763,20 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10 3 14" xfId="7" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 13 2 2 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 133 2 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal 195" xfId="8" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 2 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="Normal 315" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Normal 80" xfId="1" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Normal 10 3 14" xfId="7"/>
+    <cellStyle name="Normal 13 2 2 10 2 2 5 2 2 2 2" xfId="3"/>
+    <cellStyle name="Normal 13 2 2 2" xfId="4"/>
+    <cellStyle name="Normal 133 2 2" xfId="6"/>
+    <cellStyle name="Normal 195" xfId="8"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2 2" xfId="10"/>
+    <cellStyle name="Normal 2 2 7 2 2 2" xfId="5"/>
+    <cellStyle name="Normal 315" xfId="9"/>
+    <cellStyle name="Normal 80" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -8038,7 +8053,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B1834"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -22719,14 +22734,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1834" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:B1834"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B107"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -23589,13 +23604,29 @@
         <v>2507</v>
       </c>
     </row>
+    <row r="108" spans="1:2">
+      <c r="A108" s="8" t="s">
+        <v>2523</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>2507</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="8" t="s">
+        <v>2524</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>2507</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -25121,8 +25152,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F41" xr:uid="{00000000-0009-0000-0000-000002000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F79">
+  <autoFilter ref="A1:F41">
+    <sortState ref="A2:F79">
       <sortCondition ref="B1:B41"/>
     </sortState>
   </autoFilter>
@@ -25131,7 +25162,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -25178,13 +25209,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -25225,13 +25256,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B4" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -26623,8 +26654,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F43" xr:uid="{00000000-0009-0000-0000-000005000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F73">
+  <autoFilter ref="A1:F43">
+    <sortState ref="A2:F73">
       <sortCondition descending="1" ref="C1:C43"/>
     </sortState>
   </autoFilter>
@@ -26633,7 +26664,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -27242,13 +27273,13 @@
       <c r="D43" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D43" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:D43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -28082,7 +28113,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D58" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
+  <autoFilter ref="A1:D58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Enhance sheet selection logic for workbook processing and add support for any sheet mode
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4931" uniqueCount="2525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4937" uniqueCount="2528">
   <si>
     <t>part_used</t>
   </si>
@@ -7611,6 +7611,15 @@
   </si>
   <si>
     <t>4TC85HU8500X</t>
+  </si>
+  <si>
+    <t>4TC65HN7000I</t>
+  </si>
+  <si>
+    <t>4TC65HU8500I</t>
+  </si>
+  <si>
+    <t>4TC75HN7000I</t>
   </si>
 </sst>
 </file>
@@ -22741,7 +22750,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B109"/>
+  <dimension ref="A1:B112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -23618,6 +23627,30 @@
       </c>
       <c r="B109" s="1" t="s">
         <v>2507</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" t="s">
+        <v>2525</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>1943</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" t="s">
+        <v>2526</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>1943</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" t="s">
+        <v>2527</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>1943</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update part signatures and winners in monthly report recipes for improved accuracy
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -7771,7 +7771,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7781,12 +7781,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -7832,7 +7826,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -7843,11 +7837,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -7856,10 +7846,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -22830,7 +22825,7 @@
       </c>
     </row>
     <row r="1835" spans="1:2">
-      <c r="A1835" s="11" t="s">
+      <c r="A1835" s="9" t="s">
         <v>2548</v>
       </c>
       <c r="B1835" s="1" t="s">
@@ -22838,15 +22833,15 @@
       </c>
     </row>
     <row r="1836" spans="1:2">
-      <c r="A1836" s="11" t="s">
+      <c r="A1836" s="9" t="s">
         <v>2549</v>
       </c>
-      <c r="B1836" s="12" t="s">
+      <c r="B1836" s="10" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="1837" spans="1:2">
-      <c r="A1837" s="11" t="s">
+      <c r="A1837" s="9" t="s">
         <v>2550</v>
       </c>
       <c r="B1837" s="1" t="s">
@@ -23725,7 +23720,7 @@
       </c>
     </row>
     <row r="108" spans="1:2">
-      <c r="A108" s="6" t="s">
+      <c r="A108" s="4" t="s">
         <v>2511</v>
       </c>
       <c r="B108" s="1" t="s">
@@ -23733,7 +23728,7 @@
       </c>
     </row>
     <row r="109" spans="1:2">
-      <c r="A109" s="6" t="s">
+      <c r="A109" s="4" t="s">
         <v>2512</v>
       </c>
       <c r="B109" s="1" t="s">
@@ -24220,7 +24215,7 @@
       <c r="C22" s="3" t="s">
         <v>2021</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="8" t="s">
         <v>2545</v>
       </c>
       <c r="E22" s="3" t="s">
@@ -25250,7 +25245,7 @@
       <c r="A76" s="3">
         <v>690</v>
       </c>
-      <c r="B76" s="7"/>
+      <c r="B76" s="5"/>
       <c r="C76" s="3" t="s">
         <v>2021</v>
       </c>
@@ -25372,7 +25367,7 @@
       <c r="A83" s="3">
         <v>750</v>
       </c>
-      <c r="B83" s="9" t="s">
+      <c r="B83" s="7" t="s">
         <v>322</v>
       </c>
       <c r="C83" s="3" t="s">
@@ -25389,7 +25384,7 @@
       <c r="A84" s="3">
         <v>760</v>
       </c>
-      <c r="B84" s="8" t="s">
+      <c r="B84" s="6" t="s">
         <v>459</v>
       </c>
       <c r="C84" s="3" t="s">
@@ -25547,7 +25542,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -25557,7 +25552,7 @@
     <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" s="2" t="s">
         <v>2016</v>
       </c>
@@ -25577,7 +25572,7 @@
         <v>2085</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:8">
       <c r="A2" s="1">
         <v>10</v>
       </c>
@@ -25595,1383 +25590,1601 @@
         <v>2086</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="1">
+    <row r="3" spans="1:8">
+      <c r="A3" s="11">
         <v>20</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="11">
         <v>1</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1" t="s">
+      <c r="C3" s="11"/>
+      <c r="D3" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="11" t="s">
         <v>2087</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="11" t="s">
         <v>2088</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="30">
-      <c r="A4" s="1">
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" spans="1:8" ht="30">
+      <c r="A4" s="11">
         <v>30</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="11">
         <v>1</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1" t="s">
+      <c r="C4" s="11"/>
+      <c r="D4" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="11" t="s">
         <v>2510</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="11" t="s">
         <v>2089</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="1">
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="11">
         <v>40</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="11">
         <v>1</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1" t="s">
+      <c r="C5" s="11"/>
+      <c r="D5" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="11" t="s">
         <v>2090</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="11" t="s">
         <v>2091</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="1">
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="11">
         <v>50</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="11">
         <v>1</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1" t="s">
+      <c r="C6" s="11"/>
+      <c r="D6" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="11" t="s">
         <v>2092</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="11" t="s">
         <v>2093</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="1">
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="11">
         <v>60</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="11">
         <v>1</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1" t="s">
+      <c r="C7" s="11"/>
+      <c r="D7" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="11" t="s">
         <v>2094</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="11" t="s">
         <v>2095</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="1">
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="11">
         <v>70</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="11">
         <v>1</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1" t="s">
+      <c r="C8" s="11"/>
+      <c r="D8" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="11" t="s">
         <v>2096</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="11" t="s">
         <v>2097</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="45">
-      <c r="A9" s="1">
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+    </row>
+    <row r="9" spans="1:8" ht="45">
+      <c r="A9" s="11">
         <v>80</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="11">
         <v>1</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="11" t="s">
         <v>2437</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="11" t="s">
         <v>2098</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="1">
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="11">
         <v>90</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="11">
         <v>1</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>989</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="C10" s="11" t="s">
+        <v>989</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="11" t="s">
         <v>2099</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="11" t="s">
         <v>2100</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="1">
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="11">
         <v>100</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="11">
         <v>1</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="11" t="s">
         <v>1429</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="11" t="s">
         <v>2101</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="11" t="s">
         <v>2102</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="1">
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="11">
         <v>110</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="11">
         <v>1</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="D12" s="1" t="s">
+      <c r="C12" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="11" t="s">
         <v>2103</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="11" t="s">
         <v>2104</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="1">
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="11">
         <v>111</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="11">
         <v>1</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="C13" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="11" t="s">
         <v>2501</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="11" t="s">
         <v>2086</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="1">
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="11">
         <v>120</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="11">
         <v>1</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="11" t="s">
         <v>1660</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="11" t="s">
         <v>2105</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="11" t="s">
         <v>2106</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="1">
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="11">
         <v>130</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="11">
         <v>1</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="11" t="s">
         <v>2107</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="11" t="s">
         <v>2108</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="1">
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="11">
         <v>140</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="11">
         <v>1</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="11" t="s">
         <v>2109</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="11" t="s">
         <v>2110</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="1">
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="11">
         <v>150</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="11">
         <v>1</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="11" t="s">
         <v>2111</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" s="11" t="s">
         <v>2112</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="1">
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="11">
         <v>160</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="11">
         <v>1</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="11" t="s">
         <v>2113</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="11" t="s">
         <v>2114</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="1">
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="11">
         <v>170</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="11">
         <v>1</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="11" t="s">
         <v>2115</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="11" t="s">
         <v>2116</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="1">
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="11">
         <v>180</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="11">
         <v>1</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="11" t="s">
         <v>2115</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" s="11" t="s">
         <v>2116</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="1">
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="11">
         <v>190</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="11">
         <v>1</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="11" t="s">
         <v>1732</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="11" t="s">
         <v>2117</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="11" t="s">
         <v>2118</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="1">
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="11">
         <v>200</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="11">
         <v>1</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="11" t="s">
         <v>1826</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="11" t="s">
         <v>2119</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F22" s="11" t="s">
         <v>2120</v>
       </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="1">
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="11">
         <v>210</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="11">
         <v>1</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="11" t="s">
         <v>1811</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="11" t="s">
         <v>2121</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F23" s="11" t="s">
         <v>2122</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="60">
-      <c r="A24" s="1">
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="1:8" ht="60">
+      <c r="A24" s="11">
         <v>220</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="11">
         <v>1</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="D24" s="1" t="s">
+      <c r="C24" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="11" t="s">
         <v>2509</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F24" s="11" t="s">
         <v>2123</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="45">
-      <c r="A25" s="1">
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="1:8" ht="45">
+      <c r="A25" s="11">
         <v>230</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="11">
         <v>1</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="11" t="s">
         <v>1429</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="11" t="s">
         <v>2124</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" s="11" t="s">
         <v>2125</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="1">
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="11">
         <v>240</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="11">
         <v>1</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="11" t="s">
         <v>1660</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="11" t="s">
         <v>2126</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="11" t="s">
         <v>2127</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="1">
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="11">
         <v>250</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="11">
         <v>1</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="11" t="s">
         <v>2128</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" s="11" t="s">
         <v>2129</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="1">
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" s="11">
         <v>260</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="11">
         <v>1</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" s="11" t="s">
         <v>2130</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" s="11" t="s">
         <v>2131</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="1">
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="11">
         <v>270</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="11">
         <v>1</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E29" s="11" t="s">
         <v>2130</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="F29" s="11" t="s">
         <v>2131</v>
       </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" s="1">
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="11">
         <v>280</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="11">
         <v>1</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="11" t="s">
         <v>1429</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F30" s="11" t="s">
         <v>2102</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="1">
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="11">
         <v>290</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="11">
         <v>1</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>989</v>
-      </c>
-      <c r="D31" s="1" t="s">
+      <c r="C31" s="11" t="s">
+        <v>989</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E31" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F31" s="11" t="s">
         <v>2100</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="1">
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="11">
         <v>300</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="11">
         <v>1</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="D32" s="1" t="s">
+      <c r="C32" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="D32" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E32" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="11" t="s">
         <v>2104</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="1">
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="11">
         <v>310</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="11">
         <v>1</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="11" t="s">
         <v>1660</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F33" s="11" t="s">
         <v>2106</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="1">
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="11">
         <v>320</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="11">
         <v>1</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="11" t="s">
         <v>1398</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D34" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" s="11" t="s">
         <v>2125</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="1">
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="11">
         <v>330</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="11">
         <v>1</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D35" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F35" s="11" t="s">
         <v>2108</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" s="1">
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="11">
         <v>340</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="11">
         <v>1</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" s="11" t="s">
         <v>2123</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" s="1">
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="11">
         <v>350</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="11">
         <v>1</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="F37" s="11" t="s">
         <v>2110</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="1">
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="11">
         <v>360</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="11">
         <v>1</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F38" s="11" t="s">
         <v>2114</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="1">
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="11">
         <v>370</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="11">
         <v>1</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F39" s="11" t="s">
         <v>2112</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" s="1">
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="11">
         <v>380</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="11">
         <v>1</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D40" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F40" s="11" t="s">
         <v>2116</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="1">
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="11">
         <v>390</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="11">
         <v>1</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D41" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="E41" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="F41" s="11" t="s">
         <v>2116</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="1">
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="11">
         <v>400</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="11">
         <v>1</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="11" t="s">
         <v>1732</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D42" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E42" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F42" s="11" t="s">
         <v>2118</v>
       </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" s="1">
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="11">
         <v>410</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="11">
         <v>1</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="11" t="s">
         <v>1826</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D43" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="F43" s="11" t="s">
         <v>2120</v>
       </c>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44" s="1">
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="11">
         <v>420</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="11">
         <v>1</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="11" t="s">
         <v>1811</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D44" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="E44" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" s="11" t="s">
         <v>2551</v>
       </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45" s="1">
+      <c r="G44" s="12"/>
+      <c r="H44" s="12"/>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="11">
         <v>430</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="11">
         <v>1</v>
       </c>
-      <c r="C45" s="11" t="s">
+      <c r="C45" s="13" t="s">
         <v>1902</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D45" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="E45" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="F45" s="11" t="s">
         <v>2180</v>
       </c>
-    </row>
-    <row r="46" spans="1:6">
-      <c r="A46" s="1">
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="11">
         <v>440</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="11">
         <v>1</v>
       </c>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1" t="s">
+      <c r="C46" s="11"/>
+      <c r="D46" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" s="11" t="s">
         <v>2434</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F46" s="11" t="s">
         <v>2127</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="60">
-      <c r="A47" s="1">
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+    </row>
+    <row r="47" spans="1:8" ht="60">
+      <c r="A47" s="11">
         <v>450</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="11">
         <v>1</v>
       </c>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1" t="s">
+      <c r="C47" s="11"/>
+      <c r="D47" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="E47" s="11" t="s">
         <v>2441</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="F47" s="11" t="s">
         <v>2123</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="45">
-      <c r="A48" s="1">
+      <c r="G47" s="12"/>
+      <c r="H47" s="12"/>
+    </row>
+    <row r="48" spans="1:8" ht="45">
+      <c r="A48" s="11">
         <v>460</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="11">
         <v>1</v>
       </c>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1" t="s">
+      <c r="C48" s="11"/>
+      <c r="D48" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E48" s="11" t="s">
         <v>2440</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F48" s="11" t="s">
         <v>2125</v>
       </c>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49" s="1">
+      <c r="G48" s="12"/>
+      <c r="H48" s="12"/>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="11">
         <v>470</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="11">
         <v>1</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="C49" s="12"/>
+      <c r="D49" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="12" t="s">
         <v>2435</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F49" s="11" t="s">
         <v>2123</v>
       </c>
-    </row>
-    <row r="50" spans="1:6">
-      <c r="A50" s="1">
+      <c r="G49" s="12"/>
+      <c r="H49" s="12"/>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="11">
         <v>480</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="11">
         <v>1</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="C50" s="12"/>
+      <c r="D50" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="E50" s="11" t="s">
         <v>2442</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F50" s="11" t="s">
         <v>2125</v>
       </c>
-    </row>
-    <row r="51" spans="1:6">
-      <c r="A51" s="1">
+      <c r="G50" s="12"/>
+      <c r="H50" s="12"/>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="11">
         <v>490</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B51" s="11">
         <v>1</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="C51" s="12"/>
+      <c r="D51" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" s="12" t="s">
         <v>2438</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="F51" s="11" t="s">
         <v>2123</v>
       </c>
-    </row>
-    <row r="52" spans="1:6">
-      <c r="A52" s="1">
+      <c r="G51" s="12"/>
+      <c r="H51" s="12"/>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="11">
         <v>500</v>
       </c>
-      <c r="B52" s="1">
+      <c r="B52" s="11">
         <v>1</v>
       </c>
-      <c r="C52" s="1"/>
-      <c r="D52" s="1" t="s">
+      <c r="C52" s="11"/>
+      <c r="D52" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" s="11" t="s">
         <v>2436</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="F52" s="11" t="s">
         <v>2129</v>
       </c>
-    </row>
-    <row r="53" spans="1:6">
-      <c r="A53" s="1">
+      <c r="G52" s="12"/>
+      <c r="H52" s="12"/>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" s="11">
         <v>510</v>
       </c>
-      <c r="B53" s="1">
+      <c r="B53" s="11">
         <v>1</v>
       </c>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1" t="s">
+      <c r="C53" s="11"/>
+      <c r="D53" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E53" s="12" t="s">
         <v>2443</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="F53" s="11" t="s">
         <v>2131</v>
       </c>
-    </row>
-    <row r="54" spans="1:6">
-      <c r="A54" s="1">
+      <c r="G53" s="12"/>
+      <c r="H53" s="12"/>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" s="11">
         <v>520</v>
       </c>
-      <c r="B54" s="1">
+      <c r="B54" s="11">
         <v>1</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="D54" s="1" t="s">
+      <c r="D54" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="E54" s="11" t="s">
         <v>2501</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="F54" s="11" t="s">
         <v>2086</v>
       </c>
-    </row>
-    <row r="55" spans="1:6">
-      <c r="A55" s="1">
+      <c r="G54" s="12"/>
+      <c r="H54" s="12"/>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" s="11">
         <v>530</v>
       </c>
-      <c r="B55" s="1">
+      <c r="B55" s="11">
         <v>1</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="D55" s="1" t="s">
+      <c r="D55" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" s="11" t="s">
         <v>2501</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="F55" s="11" t="s">
         <v>2086</v>
       </c>
-    </row>
-    <row r="56" spans="1:6">
-      <c r="A56" s="1">
+      <c r="G55" s="12"/>
+      <c r="H55" s="12"/>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56" s="11">
         <v>540</v>
       </c>
-      <c r="B56" s="1">
+      <c r="B56" s="11">
         <v>1</v>
       </c>
-      <c r="D56" t="s">
+      <c r="C56" s="12"/>
+      <c r="D56" s="12" t="s">
         <v>2439</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E56" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="F56" s="11" t="s">
         <v>2086</v>
       </c>
-    </row>
-    <row r="57" spans="1:6">
-      <c r="A57" s="1">
+      <c r="G56" s="12"/>
+      <c r="H56" s="12"/>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" s="11">
         <v>550</v>
       </c>
-      <c r="B57" s="1">
+      <c r="B57" s="11">
         <v>1</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="C57" s="12"/>
+      <c r="D57" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E57" s="12" t="s">
         <v>2439</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="F57" s="11" t="s">
         <v>2086</v>
       </c>
-    </row>
-    <row r="58" spans="1:6">
-      <c r="A58" s="4">
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58" s="11">
         <v>560</v>
       </c>
-      <c r="B58" s="4">
+      <c r="B58" s="11">
         <v>1</v>
       </c>
-      <c r="D58" s="1" t="s">
+      <c r="C58" s="12"/>
+      <c r="D58" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E58" s="12" t="s">
         <v>2185</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F58" s="12" t="s">
         <v>2185</v>
       </c>
-    </row>
-    <row r="59" spans="1:6">
-      <c r="A59" s="4">
+      <c r="G58" s="12"/>
+      <c r="H58" s="12"/>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59" s="11">
         <v>570</v>
       </c>
-      <c r="B59" s="5">
+      <c r="B59" s="12">
         <v>1</v>
       </c>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4" t="s">
+      <c r="C59" s="11"/>
+      <c r="D59" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="E59" s="4" t="s">
+      <c r="E59" s="11" t="s">
         <v>2444</v>
       </c>
-      <c r="F59" s="4" t="s">
+      <c r="F59" s="11" t="s">
         <v>2154</v>
       </c>
-    </row>
-    <row r="60" spans="1:6">
-      <c r="A60" s="4">
+      <c r="G59" s="12"/>
+      <c r="H59" s="12"/>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" s="11">
         <v>580</v>
       </c>
-      <c r="B60" s="5">
+      <c r="B60" s="12">
         <v>1</v>
       </c>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5" t="s">
+      <c r="C60" s="12"/>
+      <c r="D60" s="12" t="s">
         <v>2445</v>
       </c>
-      <c r="E60" s="5" t="s">
+      <c r="E60" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="F60" s="5" t="s">
+      <c r="F60" s="12" t="s">
         <v>2125</v>
       </c>
-    </row>
-    <row r="61" spans="1:6">
-      <c r="A61" s="4">
+      <c r="G60" s="12"/>
+      <c r="H60" s="12"/>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" s="11">
         <v>590</v>
       </c>
-      <c r="B61" s="5">
+      <c r="B61" s="12">
         <v>1</v>
       </c>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5" t="s">
+      <c r="C61" s="12"/>
+      <c r="D61" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="E61" s="12" t="s">
         <v>2446</v>
       </c>
-      <c r="F61" s="5" t="s">
+      <c r="F61" s="12" t="s">
         <v>2125</v>
       </c>
-    </row>
-    <row r="62" spans="1:6">
-      <c r="A62" s="4">
+      <c r="G61" s="12"/>
+      <c r="H61" s="12"/>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" s="11">
         <v>600</v>
       </c>
-      <c r="B62" s="5">
+      <c r="B62" s="12">
         <v>1</v>
       </c>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5" t="s">
+      <c r="C62" s="12"/>
+      <c r="D62" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E62" s="5" t="s">
+      <c r="E62" s="12" t="s">
         <v>2447</v>
       </c>
-      <c r="F62" s="5" t="s">
+      <c r="F62" s="12" t="s">
         <v>2123</v>
       </c>
-    </row>
-    <row r="63" spans="1:6">
-      <c r="A63" s="4">
+      <c r="G62" s="12"/>
+      <c r="H62" s="12"/>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" s="11">
         <v>610</v>
       </c>
-      <c r="B63" s="5">
+      <c r="B63" s="12">
         <v>1</v>
       </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5" t="s">
+      <c r="C63" s="12"/>
+      <c r="D63" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E63" s="5" t="s">
+      <c r="E63" s="12" t="s">
         <v>2448</v>
       </c>
-      <c r="F63" s="5" t="s">
+      <c r="F63" s="12" t="s">
         <v>2449</v>
       </c>
-    </row>
-    <row r="64" spans="1:6">
-      <c r="A64" s="4">
+      <c r="G63" s="12"/>
+      <c r="H63" s="12"/>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" s="11">
         <v>620</v>
       </c>
-      <c r="B64" s="5">
+      <c r="B64" s="12">
         <v>1</v>
       </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5" t="s">
+      <c r="C64" s="12"/>
+      <c r="D64" s="12" t="s">
         <v>2450</v>
       </c>
-      <c r="E64" s="5" t="s">
+      <c r="E64" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="F64" s="5" t="s">
+      <c r="F64" s="12" t="s">
         <v>2127</v>
       </c>
-    </row>
-    <row r="65" spans="1:6">
-      <c r="A65" s="4">
+      <c r="G64" s="12"/>
+      <c r="H64" s="12"/>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" s="11">
         <v>630</v>
       </c>
-      <c r="B65" s="5">
+      <c r="B65" s="12">
         <v>1</v>
       </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5" t="s">
+      <c r="C65" s="12"/>
+      <c r="D65" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E65" s="5" t="s">
+      <c r="E65" s="12" t="s">
         <v>2451</v>
       </c>
-      <c r="F65" s="5" t="s">
+      <c r="F65" s="12" t="s">
         <v>2127</v>
       </c>
-    </row>
-    <row r="66" spans="1:6">
-      <c r="A66" s="4">
+      <c r="G65" s="12"/>
+      <c r="H65" s="12"/>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" s="11">
         <v>640</v>
       </c>
-      <c r="B66" s="5">
+      <c r="B66" s="12">
         <v>1</v>
       </c>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5" t="s">
+      <c r="C66" s="12"/>
+      <c r="D66" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E66" s="5" t="s">
+      <c r="E66" s="12" t="s">
         <v>2452</v>
       </c>
-      <c r="F66" s="5" t="s">
+      <c r="F66" s="12" t="s">
         <v>2122</v>
       </c>
-    </row>
-    <row r="67" spans="1:6">
-      <c r="A67" s="4">
+      <c r="G66" s="12"/>
+      <c r="H66" s="12"/>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" s="11">
         <v>650</v>
       </c>
-      <c r="B67" s="5">
+      <c r="B67" s="12">
         <v>1</v>
       </c>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5" t="s">
+      <c r="C67" s="12"/>
+      <c r="D67" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E67" s="5" t="s">
+      <c r="E67" s="12" t="s">
         <v>2453</v>
       </c>
-      <c r="F67" s="5" t="s">
+      <c r="F67" s="12" t="s">
         <v>2089</v>
       </c>
-    </row>
-    <row r="68" spans="1:6">
-      <c r="A68" s="4">
+      <c r="G67" s="12"/>
+      <c r="H67" s="12"/>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" s="11">
         <v>660</v>
       </c>
-      <c r="B68" s="5">
+      <c r="B68" s="12">
         <v>1</v>
       </c>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5" t="s">
+      <c r="C68" s="12"/>
+      <c r="D68" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E68" s="5" t="s">
+      <c r="E68" s="12" t="s">
         <v>2454</v>
       </c>
-      <c r="F68" s="5" t="s">
+      <c r="F68" s="12" t="s">
         <v>2129</v>
       </c>
-    </row>
-    <row r="69" spans="1:6">
-      <c r="A69" s="4">
+      <c r="G68" s="12"/>
+      <c r="H68" s="12"/>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" s="11">
         <v>670</v>
       </c>
-      <c r="B69" s="5">
+      <c r="B69" s="12">
         <v>1</v>
       </c>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5" t="s">
+      <c r="C69" s="12"/>
+      <c r="D69" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E69" s="5" t="s">
+      <c r="E69" s="12" t="s">
         <v>2455</v>
       </c>
-      <c r="F69" s="5" t="s">
+      <c r="F69" s="12" t="s">
         <v>2098</v>
       </c>
-    </row>
-    <row r="70" spans="1:6">
-      <c r="A70" s="4">
+      <c r="G69" s="12"/>
+      <c r="H69" s="12"/>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" s="11">
         <v>680</v>
       </c>
-      <c r="B70" s="5">
+      <c r="B70" s="12">
         <v>1</v>
       </c>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5" t="s">
+      <c r="C70" s="12"/>
+      <c r="D70" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E70" s="5" t="s">
+      <c r="E70" s="12" t="s">
         <v>2456</v>
       </c>
-      <c r="F70" s="5" t="s">
+      <c r="F70" s="12" t="s">
         <v>2097</v>
       </c>
-    </row>
-    <row r="71" spans="1:6">
-      <c r="A71" s="4">
+      <c r="G70" s="12"/>
+      <c r="H70" s="12"/>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" s="11">
         <v>690</v>
       </c>
-      <c r="B71" s="5">
+      <c r="B71" s="12">
         <v>1</v>
       </c>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5" t="s">
+      <c r="C71" s="12"/>
+      <c r="D71" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E71" s="5" t="s">
+      <c r="E71" s="12" t="s">
         <v>2457</v>
       </c>
-      <c r="F71" s="5" t="s">
+      <c r="F71" s="12" t="s">
         <v>2185</v>
       </c>
-    </row>
-    <row r="72" spans="1:6">
-      <c r="A72" s="4">
+      <c r="G71" s="12"/>
+      <c r="H71" s="12"/>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" s="11">
         <v>700</v>
       </c>
-      <c r="B72" s="5">
+      <c r="B72" s="12">
         <v>1</v>
       </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5" t="s">
+      <c r="C72" s="12"/>
+      <c r="D72" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E72" s="5" t="s">
+      <c r="E72" s="12" t="s">
         <v>2458</v>
       </c>
-      <c r="F72" s="5" t="s">
+      <c r="F72" s="12" t="s">
         <v>2088</v>
       </c>
-    </row>
-    <row r="73" spans="1:6">
-      <c r="A73" s="4">
+      <c r="G72" s="12"/>
+      <c r="H72" s="12"/>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" s="11">
         <v>710</v>
       </c>
-      <c r="B73" s="5">
+      <c r="B73" s="12">
         <v>1</v>
       </c>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5" t="s">
+      <c r="C73" s="12"/>
+      <c r="D73" s="12" t="s">
         <v>2459</v>
       </c>
-      <c r="E73" s="5" t="s">
+      <c r="E73" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="F73" s="5" t="s">
+      <c r="F73" s="12" t="s">
         <v>2086</v>
       </c>
-    </row>
-    <row r="74" spans="1:6">
-      <c r="A74" s="4">
+      <c r="G73" s="12"/>
+      <c r="H73" s="12"/>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" s="11">
         <v>720</v>
       </c>
-      <c r="B74" s="5">
+      <c r="B74" s="12">
         <v>1</v>
       </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5" t="s">
+      <c r="C74" s="12"/>
+      <c r="D74" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E74" s="5" t="s">
+      <c r="E74" s="12" t="s">
         <v>2460</v>
       </c>
-      <c r="F74" s="5" t="s">
+      <c r="F74" s="12" t="s">
         <v>2086</v>
       </c>
-    </row>
-    <row r="75" spans="1:6">
-      <c r="C75" s="5"/>
-      <c r="D75" s="5" t="s">
+      <c r="G74" s="12"/>
+      <c r="H74" s="12"/>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" s="11">
+        <v>730</v>
+      </c>
+      <c r="B75" s="12">
+        <v>1</v>
+      </c>
+      <c r="C75" s="12"/>
+      <c r="D75" s="12" t="s">
         <v>2058</v>
       </c>
-      <c r="E75" s="5" t="s">
+      <c r="E75" s="12" t="s">
         <v>2461</v>
       </c>
-      <c r="F75" s="5" t="s">
+      <c r="F75" s="12" t="s">
         <v>2089</v>
       </c>
+      <c r="G75" s="12"/>
+      <c r="H75" s="12"/>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" s="12"/>
+      <c r="B76" s="12"/>
+      <c r="C76" s="12"/>
+      <c r="D76" s="12"/>
+      <c r="E76" s="12"/>
+      <c r="F76" s="12"/>
+      <c r="G76" s="12"/>
+      <c r="H76" s="12"/>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" s="12"/>
+      <c r="B77" s="12"/>
+      <c r="C77" s="12"/>
+      <c r="D77" s="12"/>
+      <c r="E77" s="12"/>
+      <c r="F77" s="12"/>
+      <c r="G77" s="12"/>
+      <c r="H77" s="12"/>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78" s="12"/>
+      <c r="B78" s="12"/>
+      <c r="C78" s="12"/>
+      <c r="D78" s="12"/>
+      <c r="E78" s="12"/>
+      <c r="F78" s="12"/>
+      <c r="G78" s="12"/>
+      <c r="H78" s="12"/>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79" s="12"/>
+      <c r="B79" s="12"/>
+      <c r="C79" s="12"/>
+      <c r="D79" s="12"/>
+      <c r="E79" s="12"/>
+      <c r="F79" s="12"/>
+      <c r="G79" s="12"/>
+      <c r="H79" s="12"/>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80" s="12"/>
+      <c r="B80" s="12"/>
+      <c r="C80" s="12"/>
+      <c r="D80" s="12"/>
+      <c r="E80" s="12"/>
+      <c r="F80" s="12"/>
+      <c r="G80" s="12"/>
+      <c r="H80" s="12"/>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81" s="12"/>
+      <c r="B81" s="12"/>
+      <c r="C81" s="12"/>
+      <c r="D81" s="12"/>
+      <c r="E81" s="12"/>
+      <c r="F81" s="12"/>
+      <c r="G81" s="12"/>
+      <c r="H81" s="12"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F44">

</xml_diff>

<commit_message>
feat: Implement amount scaling for summary values in job summary results and update related configurations
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5058" uniqueCount="2562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5074" uniqueCount="2570">
   <si>
     <t>part_used</t>
   </si>
@@ -7722,6 +7722,30 @@
   </si>
   <si>
     <t>BERGARIS|Tampilan tidak normal|KUNING</t>
+  </si>
+  <si>
+    <t>2TC24CB3IBK</t>
+  </si>
+  <si>
+    <t>2TC40AE1IAM</t>
+  </si>
+  <si>
+    <t>LC24SA4000I</t>
+  </si>
+  <si>
+    <t>LC29LE507I</t>
+  </si>
+  <si>
+    <t>LC32LE295I</t>
+  </si>
+  <si>
+    <t>LC32SA4101IWH</t>
+  </si>
+  <si>
+    <t>LC40LE185IWH</t>
+  </si>
+  <si>
+    <t>LC40SA5100I</t>
   </si>
 </sst>
 </file>
@@ -7856,7 +7880,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -7867,7 +7891,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -7893,6 +7916,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -22863,7 +22890,7 @@
       </c>
     </row>
     <row r="1835" spans="1:2">
-      <c r="A1835" s="7" t="s">
+      <c r="A1835" s="6" t="s">
         <v>2531</v>
       </c>
       <c r="B1835" s="1" t="s">
@@ -22871,15 +22898,15 @@
       </c>
     </row>
     <row r="1836" spans="1:2">
-      <c r="A1836" s="7" t="s">
+      <c r="A1836" s="6" t="s">
         <v>2532</v>
       </c>
-      <c r="B1836" s="8" t="s">
+      <c r="B1836" s="7" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="1837" spans="1:2">
-      <c r="A1837" s="7" t="s">
+      <c r="A1837" s="6" t="s">
         <v>2533</v>
       </c>
       <c r="B1837" s="1" t="s">
@@ -22894,7 +22921,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B113"/>
+  <dimension ref="A1:B121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -22910,903 +22937,968 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="17" t="s">
         <v>1942</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="17" t="s">
         <v>1944</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="17" t="s">
         <v>1945</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="17" t="s">
         <v>1946</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="17" t="s">
         <v>1947</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="17" t="s">
         <v>1948</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="17" t="s">
         <v>1949</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="17" t="s">
         <v>1950</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="17" t="s">
         <v>1951</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="17" t="s">
         <v>1952</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="17" t="s">
         <v>1953</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="17" t="s">
         <v>1954</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="17" t="s">
         <v>1955</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="17" t="s">
         <v>1956</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="17" t="s">
         <v>1957</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="17" t="s">
         <v>1956</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="17" t="s">
         <v>1958</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="17" t="s">
         <v>1956</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="17" t="s">
         <v>1959</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="17" t="s">
         <v>1956</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="17" t="s">
         <v>1960</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="17" t="s">
         <v>1962</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="17" t="s">
         <v>1963</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="17" t="s">
         <v>1964</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="17" t="s">
         <v>1965</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="17" t="s">
         <v>1966</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="17" t="s">
         <v>1967</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="17" t="s">
         <v>1968</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="17" t="s">
         <v>1969</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="17" t="s">
         <v>1970</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="17" t="s">
         <v>1971</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="1" t="s">
+      <c r="A29" s="17" t="s">
         <v>1972</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="17" t="s">
         <v>1973</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="17" t="s">
         <v>1974</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="17" t="s">
         <v>1975</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="17" t="s">
         <v>1976</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="17" t="s">
         <v>1977</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="1" t="s">
+      <c r="A35" s="17" t="s">
         <v>1978</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="17" t="s">
         <v>1979</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="1" t="s">
+      <c r="A37" s="17" t="s">
         <v>1980</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="1" t="s">
+      <c r="A38" s="17" t="s">
         <v>1981</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="1" t="s">
+      <c r="A39" s="17" t="s">
         <v>1982</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="1" t="s">
+      <c r="A40" s="17" t="s">
         <v>1983</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="1" t="s">
+      <c r="A41" s="17" t="s">
         <v>1984</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="17" t="s">
         <v>1985</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="1" t="s">
+      <c r="A43" s="17" t="s">
         <v>1986</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="1" t="s">
+      <c r="A44" s="17" t="s">
         <v>1987</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="1" t="s">
+      <c r="A45" s="17" t="s">
         <v>1988</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="1" t="s">
+      <c r="A46" s="17" t="s">
         <v>1989</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="1" t="s">
+      <c r="A47" s="17" t="s">
         <v>1990</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="17" t="s">
         <v>1991</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="1" t="s">
+      <c r="A49" s="17" t="s">
         <v>1992</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="50" spans="1:2">
-      <c r="A50" s="1" t="s">
+      <c r="A50" s="17" t="s">
         <v>1993</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="51" spans="1:2">
-      <c r="A51" s="1" t="s">
+      <c r="A51" s="17" t="s">
         <v>1994</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="52" spans="1:2">
-      <c r="A52" s="1" t="s">
+      <c r="A52" s="17" t="s">
         <v>1995</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="53" spans="1:2">
-      <c r="A53" s="1" t="s">
+      <c r="A53" s="17" t="s">
         <v>1996</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="54" spans="1:2">
-      <c r="A54" s="1" t="s">
+      <c r="A54" s="17" t="s">
         <v>1997</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="55" spans="1:2">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="17" t="s">
         <v>1998</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="56" spans="1:2">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="17" t="s">
         <v>1999</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="57" spans="1:2">
-      <c r="A57" s="1" t="s">
+      <c r="A57" s="17" t="s">
         <v>2000</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="58" spans="1:2">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="17" t="s">
         <v>2001</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="59" spans="1:2">
-      <c r="A59" s="1" t="s">
+      <c r="A59" s="17" t="s">
         <v>2002</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="60" spans="1:2">
-      <c r="A60" s="1" t="s">
+      <c r="A60" s="17" t="s">
         <v>2003</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="61" spans="1:2">
-      <c r="A61" s="1" t="s">
+      <c r="A61" s="17" t="s">
         <v>2004</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="62" spans="1:2">
-      <c r="A62" s="1" t="s">
+      <c r="A62" s="17" t="s">
         <v>2005</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="63" spans="1:2">
-      <c r="A63" s="1" t="s">
+      <c r="A63" s="17" t="s">
         <v>2006</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="64" spans="1:2">
-      <c r="A64" s="1" t="s">
+      <c r="A64" s="17" t="s">
         <v>2007</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="65" spans="1:2">
-      <c r="A65" s="1" t="s">
+      <c r="A65" s="17" t="s">
         <v>2008</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="66" spans="1:2">
-      <c r="A66" s="1" t="s">
+      <c r="A66" s="17" t="s">
         <v>2009</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="67" spans="1:2">
-      <c r="A67" s="1" t="s">
+      <c r="A67" s="17" t="s">
         <v>2010</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="68" spans="1:2">
-      <c r="A68" s="1" t="s">
+      <c r="A68" s="17" t="s">
         <v>2011</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="69" spans="1:2">
-      <c r="A69" s="1" t="s">
+      <c r="A69" s="17" t="s">
         <v>2012</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" s="17" t="s">
         <v>1961</v>
       </c>
     </row>
     <row r="70" spans="1:2">
-      <c r="A70" s="1" t="s">
+      <c r="A70" s="17" t="s">
         <v>2013</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" s="17" t="s">
         <v>2014</v>
       </c>
     </row>
     <row r="71" spans="1:2">
-      <c r="A71" s="1" t="s">
+      <c r="A71" s="17" t="s">
         <v>2015</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" s="17" t="s">
         <v>2014</v>
       </c>
     </row>
     <row r="72" spans="1:2">
-      <c r="A72" t="s">
+      <c r="A72" s="15" t="s">
         <v>2452</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="73" spans="1:2">
-      <c r="A73" t="s">
+      <c r="A73" s="15" t="s">
         <v>2453</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="74" spans="1:2">
-      <c r="A74" t="s">
+      <c r="A74" s="15" t="s">
         <v>2454</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="75" spans="1:2">
-      <c r="A75" t="s">
+      <c r="A75" s="15" t="s">
         <v>2455</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B75" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="76" spans="1:2">
-      <c r="A76" t="s">
+      <c r="A76" s="15" t="s">
         <v>2456</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="77" spans="1:2">
-      <c r="A77" t="s">
+      <c r="A77" s="15" t="s">
         <v>2457</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" s="17" t="s">
         <v>2489</v>
       </c>
     </row>
     <row r="78" spans="1:2">
-      <c r="A78" t="s">
+      <c r="A78" s="15" t="s">
         <v>2458</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B78" s="17" t="s">
         <v>2489</v>
       </c>
     </row>
     <row r="79" spans="1:2">
-      <c r="A79" t="s">
+      <c r="A79" s="15" t="s">
         <v>2459</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B79" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="80" spans="1:2">
-      <c r="A80" t="s">
+      <c r="A80" s="15" t="s">
         <v>2460</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B80" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="81" spans="1:2">
-      <c r="A81" t="s">
+      <c r="A81" s="15" t="s">
         <v>2461</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B81" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="82" spans="1:2">
-      <c r="A82" t="s">
+      <c r="A82" s="15" t="s">
         <v>2462</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B82" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="83" spans="1:2">
-      <c r="A83" t="s">
+      <c r="A83" s="15" t="s">
         <v>2463</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B83" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="84" spans="1:2">
-      <c r="A84" t="s">
+      <c r="A84" s="15" t="s">
         <v>2464</v>
       </c>
-      <c r="B84" s="1" t="s">
+      <c r="B84" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="85" spans="1:2">
-      <c r="A85" t="s">
+      <c r="A85" s="15" t="s">
         <v>2465</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B85" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="86" spans="1:2">
-      <c r="A86" t="s">
+      <c r="A86" s="15" t="s">
         <v>2466</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B86" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="87" spans="1:2">
-      <c r="A87" t="s">
+      <c r="A87" s="15" t="s">
         <v>2467</v>
       </c>
-      <c r="B87" s="1" t="s">
+      <c r="B87" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="88" spans="1:2">
-      <c r="A88" t="s">
+      <c r="A88" s="15" t="s">
         <v>2468</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B88" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="89" spans="1:2">
-      <c r="A89" t="s">
+      <c r="A89" s="15" t="s">
         <v>2469</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B89" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="90" spans="1:2">
-      <c r="A90" t="s">
+      <c r="A90" s="15" t="s">
         <v>2470</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B90" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="91" spans="1:2">
-      <c r="A91" t="s">
+      <c r="A91" s="15" t="s">
         <v>2471</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B91" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="92" spans="1:2">
-      <c r="A92" t="s">
+      <c r="A92" s="15" t="s">
         <v>2472</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="B92" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="93" spans="1:2">
-      <c r="A93" t="s">
+      <c r="A93" s="15" t="s">
         <v>2473</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B93" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="94" spans="1:2">
-      <c r="A94" t="s">
+      <c r="A94" s="15" t="s">
         <v>2474</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B94" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="95" spans="1:2">
-      <c r="A95" t="s">
+      <c r="A95" s="15" t="s">
         <v>2475</v>
       </c>
-      <c r="B95" s="1" t="s">
+      <c r="B95" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="96" spans="1:2">
-      <c r="A96" t="s">
+      <c r="A96" s="15" t="s">
         <v>2476</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B96" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="97" spans="1:2">
-      <c r="A97" t="s">
+      <c r="A97" s="15" t="s">
         <v>2477</v>
       </c>
-      <c r="B97" s="1" t="s">
+      <c r="B97" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="98" spans="1:2">
-      <c r="A98" t="s">
+      <c r="A98" s="15" t="s">
         <v>2478</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="B98" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="99" spans="1:2">
-      <c r="A99" t="s">
+      <c r="A99" s="15" t="s">
         <v>2479</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B99" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="100" spans="1:2">
-      <c r="A100" t="s">
+      <c r="A100" s="15" t="s">
         <v>2480</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B100" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="101" spans="1:2">
-      <c r="A101" t="s">
+      <c r="A101" s="15" t="s">
         <v>2481</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B101" s="17" t="s">
         <v>2489</v>
       </c>
     </row>
     <row r="102" spans="1:2">
-      <c r="A102" t="s">
+      <c r="A102" s="15" t="s">
         <v>2482</v>
       </c>
-      <c r="B102" s="1" t="s">
+      <c r="B102" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="103" spans="1:2">
-      <c r="A103" t="s">
+      <c r="A103" s="15" t="s">
         <v>2483</v>
       </c>
-      <c r="B103" s="1" t="s">
+      <c r="B103" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="104" spans="1:2">
-      <c r="A104" t="s">
+      <c r="A104" s="15" t="s">
         <v>2484</v>
       </c>
-      <c r="B104" s="1" t="s">
+      <c r="B104" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="105" spans="1:2">
-      <c r="A105" t="s">
+      <c r="A105" s="15" t="s">
         <v>2485</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B105" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="106" spans="1:2">
-      <c r="A106" t="s">
+      <c r="A106" s="15" t="s">
         <v>2486</v>
       </c>
-      <c r="B106" s="1" t="s">
+      <c r="B106" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="107" spans="1:2">
-      <c r="A107" t="s">
+      <c r="A107" s="15" t="s">
         <v>2487</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B107" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="108" spans="1:2">
-      <c r="A108" s="4" t="s">
+      <c r="A108" s="18" t="s">
         <v>2498</v>
       </c>
-      <c r="B108" s="1" t="s">
+      <c r="B108" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="109" spans="1:2">
-      <c r="A109" s="4" t="s">
+      <c r="A109" s="18" t="s">
         <v>2499</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="B109" s="17" t="s">
         <v>2488</v>
       </c>
     </row>
     <row r="110" spans="1:2">
-      <c r="A110" t="s">
+      <c r="A110" s="15" t="s">
         <v>2500</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="B110" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="111" spans="1:2">
-      <c r="A111" t="s">
+      <c r="A111" s="15" t="s">
         <v>2501</v>
       </c>
-      <c r="B111" s="1" t="s">
+      <c r="B111" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="112" spans="1:2">
-      <c r="A112" t="s">
+      <c r="A112" s="15" t="s">
         <v>2502</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="B112" s="17" t="s">
         <v>1943</v>
       </c>
     </row>
     <row r="113" spans="1:2">
-      <c r="A113" t="s">
+      <c r="A113" s="15" t="s">
         <v>2503</v>
       </c>
-      <c r="B113" s="1" t="s">
+      <c r="B113" s="17" t="s">
         <v>1943</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="12" t="s">
+        <v>2562</v>
+      </c>
+      <c r="B114" s="17" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="12" t="s">
+        <v>2563</v>
+      </c>
+      <c r="B115" s="17" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="12" t="s">
+        <v>2564</v>
+      </c>
+      <c r="B116" s="17" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="12" t="s">
+        <v>2565</v>
+      </c>
+      <c r="B117" s="17" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="12" t="s">
+        <v>2566</v>
+      </c>
+      <c r="B118" s="17" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="12" t="s">
+        <v>2567</v>
+      </c>
+      <c r="B119" s="17" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="12" t="s">
+        <v>2568</v>
+      </c>
+      <c r="B120" s="17" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="12" t="s">
+        <v>2569</v>
+      </c>
+      <c r="B121" s="17" t="s">
+        <v>1961</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -24074,7 +24166,7 @@
       <c r="A14" s="3">
         <v>770</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>214</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -24154,7 +24246,7 @@
       <c r="A18" s="3">
         <v>780</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="14" t="s">
         <v>322</v>
       </c>
       <c r="C18" s="3" t="s">
@@ -24569,7 +24661,7 @@
       <c r="C39" s="3" t="s">
         <v>2021</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="5" t="s">
         <v>2529</v>
       </c>
       <c r="E39" s="3" t="s">
@@ -24583,7 +24675,7 @@
       <c r="A40" s="3">
         <v>790</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="4" t="s">
         <v>459</v>
       </c>
       <c r="C40" s="3" t="s">
@@ -25563,7 +25655,7 @@
       <c r="A92" s="3">
         <v>460</v>
       </c>
-      <c r="B92" s="17"/>
+      <c r="B92" s="16"/>
       <c r="C92" s="3" t="s">
         <v>2021</v>
       </c>
@@ -25635,7 +25727,7 @@
       <c r="A96" s="3">
         <v>710</v>
       </c>
-      <c r="B96" s="16"/>
+      <c r="B96" s="15"/>
       <c r="C96" s="3" t="s">
         <v>2021</v>
       </c>
@@ -25653,7 +25745,7 @@
       <c r="A97" s="3">
         <v>791</v>
       </c>
-      <c r="B97" s="5"/>
+      <c r="B97" s="4"/>
       <c r="C97" s="3" t="s">
         <v>2021</v>
       </c>
@@ -25809,60 +25901,60 @@
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="9">
+      <c r="A2" s="8">
         <v>20</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>1</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9" t="s">
+      <c r="C2" s="8"/>
+      <c r="D2" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>2086</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>2087</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="9">
+      <c r="A3" s="8">
         <v>700</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>1</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="10" t="s">
+      <c r="C3" s="11"/>
+      <c r="D3" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>2448</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>2087</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="9">
+      <c r="A4" s="8">
         <v>50</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>1</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>2090</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>2091</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="1">
@@ -25881,8 +25973,8 @@
       <c r="F5" s="1" t="s">
         <v>2085</v>
       </c>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="1">
@@ -25891,7 +25983,7 @@
       <c r="B6" s="1">
         <v>1</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>1816</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -25903,1564 +25995,1564 @@
       <c r="F6" s="1" t="s">
         <v>2085</v>
       </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="9">
+      <c r="A7" s="8">
         <v>111</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>1</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>2491</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>2085</v>
       </c>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="9">
+      <c r="A8" s="8">
         <v>520</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>1</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>2491</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>2085</v>
       </c>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="9">
+      <c r="A9" s="8">
         <v>530</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <v>1</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>2491</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>2085</v>
       </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="9">
+      <c r="A10" s="8">
         <v>540</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>1</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="9" t="s">
         <v>2430</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>2085</v>
       </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="9">
+      <c r="A11" s="8">
         <v>550</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>1</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="9" t="s">
+      <c r="C11" s="9"/>
+      <c r="D11" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="9" t="s">
         <v>2430</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="8" t="s">
         <v>2085</v>
       </c>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="9">
+      <c r="A12" s="8">
         <v>710</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>1</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10" t="s">
+      <c r="C12" s="9"/>
+      <c r="D12" s="9" t="s">
         <v>2449</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="9" t="s">
         <v>2085</v>
       </c>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="9">
+      <c r="A13" s="8">
         <v>720</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>1</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10" t="s">
+      <c r="C13" s="9"/>
+      <c r="D13" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>2450</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="9" t="s">
         <v>2085</v>
       </c>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="9">
+      <c r="A14" s="8">
         <v>70</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>1</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9" t="s">
+      <c r="C14" s="8"/>
+      <c r="D14" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>2094</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>2095</v>
       </c>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="9">
+      <c r="A15" s="8">
         <v>680</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>1</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10" t="s">
+      <c r="C15" s="9"/>
+      <c r="D15" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>2446</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="9" t="s">
         <v>2095</v>
       </c>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="9">
+      <c r="A16" s="8">
         <v>260</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>1</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>2128</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>2129</v>
       </c>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="9">
+      <c r="A17" s="8">
         <v>270</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="8">
         <v>1</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>2128</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>2129</v>
       </c>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="9">
+      <c r="A18" s="8">
         <v>510</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>1</v>
       </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9" t="s">
+      <c r="C18" s="8"/>
+      <c r="D18" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="9" t="s">
         <v>2434</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>2129</v>
       </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="9">
+      <c r="A19" s="8">
         <v>250</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>1</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>2126</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="8" t="s">
         <v>2127</v>
       </c>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="9">
+      <c r="A20" s="8">
         <v>500</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>1</v>
       </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9" t="s">
+      <c r="C20" s="8"/>
+      <c r="D20" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>2427</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="8" t="s">
         <v>2127</v>
       </c>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="9">
+      <c r="A21" s="8">
         <v>660</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="9">
         <v>1</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10" t="s">
+      <c r="C21" s="9"/>
+      <c r="D21" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="9" t="s">
         <v>2445</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="9" t="s">
         <v>2127</v>
       </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="9">
+      <c r="A22" s="8">
         <v>570</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="9">
         <v>1</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9" t="s">
+      <c r="C22" s="8"/>
+      <c r="D22" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="8" t="s">
         <v>2435</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="8" t="s">
         <v>2152</v>
       </c>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
     </row>
     <row r="23" spans="1:8" ht="60">
-      <c r="A23" s="9">
+      <c r="A23" s="8">
         <v>220</v>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="8">
         <v>1</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="C23" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>2496</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="8" t="s">
         <v>2121</v>
       </c>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="9">
+      <c r="A24" s="8">
         <v>340</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>2121</v>
       </c>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
     </row>
     <row r="25" spans="1:8" ht="60">
-      <c r="A25" s="9">
+      <c r="A25" s="8">
         <v>450</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="8">
         <v>1</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9" t="s">
+      <c r="C25" s="8"/>
+      <c r="D25" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>2432</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="8" t="s">
         <v>2121</v>
       </c>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="9">
+      <c r="A26" s="8">
         <v>470</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="8">
         <v>1</v>
       </c>
-      <c r="C26" s="10"/>
-      <c r="D26" s="9" t="s">
+      <c r="C26" s="9"/>
+      <c r="D26" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="9" t="s">
         <v>2426</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>2121</v>
       </c>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="9">
+      <c r="A27" s="8">
         <v>490</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="8">
         <v>1</v>
       </c>
-      <c r="C27" s="10"/>
-      <c r="D27" s="9" t="s">
+      <c r="C27" s="9"/>
+      <c r="D27" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="9" t="s">
         <v>2429</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>2121</v>
       </c>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="9">
+      <c r="A28" s="8">
         <v>600</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="9">
         <v>1</v>
       </c>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10" t="s">
+      <c r="C28" s="9"/>
+      <c r="D28" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="9" t="s">
         <v>2438</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="9" t="s">
         <v>2121</v>
       </c>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
     </row>
     <row r="29" spans="1:8" ht="45">
-      <c r="A29" s="9">
+      <c r="A29" s="8">
         <v>230</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="8">
         <v>1</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="8" t="s">
         <v>1429</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="8" t="s">
         <v>2122</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="F29" s="8" t="s">
         <v>2123</v>
       </c>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="9">
+      <c r="A30" s="8">
         <v>320</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="8">
         <v>1</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="8" t="s">
         <v>1398</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="E30" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F30" s="9" t="s">
+      <c r="F30" s="8" t="s">
         <v>2123</v>
       </c>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
     </row>
     <row r="31" spans="1:8" ht="45">
-      <c r="A31" s="9">
+      <c r="A31" s="8">
         <v>460</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="8">
         <v>1</v>
       </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9" t="s">
+      <c r="C31" s="8"/>
+      <c r="D31" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="8" t="s">
         <v>2431</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="F31" s="8" t="s">
         <v>2123</v>
       </c>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="9">
+      <c r="A32" s="8">
         <v>480</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="8">
         <v>1</v>
       </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="9" t="s">
+      <c r="C32" s="9"/>
+      <c r="D32" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E32" s="9" t="s">
+      <c r="E32" s="8" t="s">
         <v>2433</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="F32" s="8" t="s">
         <v>2123</v>
       </c>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="9">
+      <c r="A33" s="8">
         <v>580</v>
       </c>
-      <c r="B33" s="10">
+      <c r="B33" s="9">
         <v>1</v>
       </c>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10" t="s">
+      <c r="C33" s="9"/>
+      <c r="D33" s="9" t="s">
         <v>2436</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="E33" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="F33" s="10" t="s">
+      <c r="F33" s="9" t="s">
         <v>2123</v>
       </c>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
     </row>
     <row r="34" spans="1:8">
-      <c r="A34" s="9">
+      <c r="A34" s="8">
         <v>590</v>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="9">
         <v>1</v>
       </c>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10" t="s">
+      <c r="C34" s="9"/>
+      <c r="D34" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="E34" s="9" t="s">
         <v>2437</v>
       </c>
-      <c r="F34" s="10" t="s">
+      <c r="F34" s="9" t="s">
         <v>2123</v>
       </c>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
     </row>
     <row r="35" spans="1:8">
-      <c r="A35" s="9">
+      <c r="A35" s="8">
         <v>240</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="8">
         <v>1</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>1660</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="8" t="s">
         <v>2124</v>
       </c>
-      <c r="F35" s="9" t="s">
+      <c r="F35" s="8" t="s">
         <v>2125</v>
       </c>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
     </row>
     <row r="36" spans="1:8">
-      <c r="A36" s="9">
+      <c r="A36" s="8">
         <v>440</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="8">
         <v>1</v>
       </c>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9" t="s">
+      <c r="C36" s="8"/>
+      <c r="D36" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="E36" s="8" t="s">
         <v>2425</v>
       </c>
-      <c r="F36" s="9" t="s">
+      <c r="F36" s="8" t="s">
         <v>2125</v>
       </c>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
     </row>
     <row r="37" spans="1:8">
-      <c r="A37" s="9">
+      <c r="A37" s="8">
         <v>620</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="9">
         <v>1</v>
       </c>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10" t="s">
+      <c r="C37" s="9"/>
+      <c r="D37" s="9" t="s">
         <v>2441</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="F37" s="9" t="s">
         <v>2125</v>
       </c>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="9">
+      <c r="A38" s="8">
         <v>630</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="9">
         <v>1</v>
       </c>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10" t="s">
+      <c r="C38" s="9"/>
+      <c r="D38" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="9" t="s">
         <v>2442</v>
       </c>
-      <c r="F38" s="10" t="s">
+      <c r="F38" s="9" t="s">
         <v>2125</v>
       </c>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
     </row>
     <row r="39" spans="1:8">
-      <c r="A39" s="9">
+      <c r="A39" s="8">
         <v>610</v>
       </c>
-      <c r="B39" s="10">
+      <c r="B39" s="9">
         <v>1</v>
       </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10" t="s">
+      <c r="C39" s="9"/>
+      <c r="D39" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="E39" s="9" t="s">
         <v>2439</v>
       </c>
-      <c r="F39" s="10" t="s">
+      <c r="F39" s="9" t="s">
         <v>2440</v>
       </c>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
     </row>
     <row r="40" spans="1:8">
-      <c r="A40" s="9">
+      <c r="A40" s="8">
         <v>210</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="8">
         <v>1</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="8" t="s">
         <v>1811</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="8" t="s">
         <v>2119</v>
       </c>
-      <c r="F40" s="9" t="s">
+      <c r="F40" s="8" t="s">
         <v>2120</v>
       </c>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="9">
+      <c r="A41" s="8">
         <v>640</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="9">
         <v>1</v>
       </c>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10" t="s">
+      <c r="C41" s="9"/>
+      <c r="D41" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E41" s="10" t="s">
+      <c r="E41" s="9" t="s">
         <v>2443</v>
       </c>
-      <c r="F41" s="10" t="s">
+      <c r="F41" s="9" t="s">
         <v>2120</v>
       </c>
-      <c r="G41" s="10"/>
-      <c r="H41" s="10"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
     </row>
     <row r="42" spans="1:8">
-      <c r="A42" s="9">
+      <c r="A42" s="8">
         <v>160</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="8">
         <v>1</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E42" s="8" t="s">
         <v>2111</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="F42" s="8" t="s">
         <v>2112</v>
       </c>
-      <c r="G42" s="10"/>
-      <c r="H42" s="10"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
     </row>
     <row r="43" spans="1:8">
-      <c r="A43" s="9">
+      <c r="A43" s="8">
         <v>360</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="8">
         <v>1</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F43" s="9" t="s">
+      <c r="F43" s="8" t="s">
         <v>2112</v>
       </c>
-      <c r="G43" s="10"/>
-      <c r="H43" s="10"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
     </row>
     <row r="44" spans="1:8">
-      <c r="A44" s="9">
+      <c r="A44" s="8">
         <v>150</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="8">
         <v>1</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="D44" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E44" s="8" t="s">
         <v>2109</v>
       </c>
-      <c r="F44" s="9" t="s">
+      <c r="F44" s="8" t="s">
         <v>2110</v>
       </c>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="9">
+      <c r="A45" s="8">
         <v>370</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45" s="8">
         <v>1</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="D45" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F45" s="8" t="s">
         <v>2110</v>
       </c>
-      <c r="G45" s="10"/>
-      <c r="H45" s="10"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
     </row>
     <row r="46" spans="1:8">
-      <c r="A46" s="9">
+      <c r="A46" s="8">
         <v>170</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="8">
         <v>1</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="D46" s="9" t="s">
+      <c r="D46" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E46" s="9" t="s">
+      <c r="E46" s="8" t="s">
         <v>2113</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F46" s="8" t="s">
         <v>2114</v>
       </c>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
     </row>
     <row r="47" spans="1:8">
-      <c r="A47" s="9">
+      <c r="A47" s="8">
         <v>180</v>
       </c>
-      <c r="B47" s="9">
+      <c r="B47" s="8">
         <v>1</v>
       </c>
-      <c r="C47" s="14" t="s">
+      <c r="C47" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="D47" s="9" t="s">
+      <c r="D47" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="8" t="s">
         <v>2113</v>
       </c>
-      <c r="F47" s="9" t="s">
+      <c r="F47" s="8" t="s">
         <v>2114</v>
       </c>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
     </row>
     <row r="48" spans="1:8">
-      <c r="A48" s="9">
+      <c r="A48" s="8">
         <v>380</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="8">
         <v>1</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="D48" s="9" t="s">
+      <c r="D48" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E48" s="9" t="s">
+      <c r="E48" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F48" s="9" t="s">
+      <c r="F48" s="8" t="s">
         <v>2114</v>
       </c>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
     </row>
     <row r="49" spans="1:8">
-      <c r="A49" s="9">
+      <c r="A49" s="8">
         <v>390</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B49" s="8">
         <v>1</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="8" t="s">
         <v>322</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="D49" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E49" s="9" t="s">
+      <c r="E49" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F49" s="9" t="s">
+      <c r="F49" s="8" t="s">
         <v>2114</v>
       </c>
-      <c r="G49" s="10"/>
-      <c r="H49" s="10"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
     </row>
     <row r="50" spans="1:8">
-      <c r="A50" s="9">
+      <c r="A50" s="8">
         <v>130</v>
       </c>
-      <c r="B50" s="9">
+      <c r="B50" s="8">
         <v>1</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="D50" s="9" t="s">
+      <c r="D50" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E50" s="9" t="s">
+      <c r="E50" s="8" t="s">
         <v>2105</v>
       </c>
-      <c r="F50" s="9" t="s">
+      <c r="F50" s="8" t="s">
         <v>2106</v>
       </c>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:8">
-      <c r="A51" s="9">
+      <c r="A51" s="8">
         <v>330</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="8">
         <v>1</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E51" s="9" t="s">
+      <c r="E51" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F51" s="9" t="s">
+      <c r="F51" s="8" t="s">
         <v>2106</v>
       </c>
-      <c r="G51" s="10"/>
-      <c r="H51" s="10"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:8">
-      <c r="A52" s="9">
+      <c r="A52" s="8">
         <v>140</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52" s="8">
         <v>1</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="D52" s="9" t="s">
+      <c r="D52" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E52" s="9" t="s">
+      <c r="E52" s="8" t="s">
         <v>2107</v>
       </c>
-      <c r="F52" s="9" t="s">
+      <c r="F52" s="8" t="s">
         <v>2108</v>
       </c>
-      <c r="G52" s="10"/>
-      <c r="H52" s="10"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
     </row>
     <row r="53" spans="1:8">
-      <c r="A53" s="9">
+      <c r="A53" s="8">
         <v>350</v>
       </c>
-      <c r="B53" s="9">
+      <c r="B53" s="8">
         <v>1</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="D53" s="9" t="s">
+      <c r="D53" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E53" s="9" t="s">
+      <c r="E53" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F53" s="9" t="s">
+      <c r="F53" s="8" t="s">
         <v>2108</v>
       </c>
-      <c r="G53" s="10"/>
-      <c r="H53" s="10"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
     </row>
     <row r="54" spans="1:8">
-      <c r="A54" s="9">
+      <c r="A54" s="8">
         <v>110</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54" s="8">
         <v>1</v>
       </c>
-      <c r="C54" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="D54" s="9" t="s">
+      <c r="C54" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="D54" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E54" s="9" t="s">
+      <c r="E54" s="8" t="s">
         <v>2101</v>
       </c>
-      <c r="F54" s="9" t="s">
+      <c r="F54" s="8" t="s">
         <v>2102</v>
       </c>
-      <c r="G54" s="10"/>
-      <c r="H54" s="10"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="9">
+      <c r="A55" s="8">
         <v>300</v>
       </c>
-      <c r="B55" s="9">
+      <c r="B55" s="8">
         <v>1</v>
       </c>
-      <c r="C55" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="D55" s="9" t="s">
+      <c r="C55" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="D55" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E55" s="9" t="s">
+      <c r="E55" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F55" s="9" t="s">
+      <c r="F55" s="8" t="s">
         <v>2102</v>
       </c>
-      <c r="G55" s="10"/>
-      <c r="H55" s="10"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
     </row>
     <row r="56" spans="1:8">
-      <c r="A56" s="9">
+      <c r="A56" s="8">
         <v>90</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="8">
         <v>1</v>
       </c>
-      <c r="C56" s="9" t="s">
-        <v>989</v>
-      </c>
-      <c r="D56" s="9" t="s">
+      <c r="C56" s="8" t="s">
+        <v>989</v>
+      </c>
+      <c r="D56" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E56" s="9" t="s">
+      <c r="E56" s="8" t="s">
         <v>2097</v>
       </c>
-      <c r="F56" s="9" t="s">
+      <c r="F56" s="8" t="s">
         <v>2098</v>
       </c>
-      <c r="G56" s="10"/>
-      <c r="H56" s="10"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
     </row>
     <row r="57" spans="1:8">
-      <c r="A57" s="9">
+      <c r="A57" s="8">
         <v>91</v>
       </c>
-      <c r="B57" s="9">
+      <c r="B57" s="8">
         <v>1</v>
       </c>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9" t="s">
+      <c r="C57" s="8"/>
+      <c r="D57" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E57" s="9" t="s">
+      <c r="E57" s="8" t="s">
         <v>2097</v>
       </c>
-      <c r="F57" s="9" t="s">
+      <c r="F57" s="8" t="s">
         <v>2098</v>
       </c>
-      <c r="G57" s="10"/>
-      <c r="H57" s="10"/>
+      <c r="G57" s="9"/>
+      <c r="H57" s="9"/>
     </row>
     <row r="58" spans="1:8">
-      <c r="A58" s="9">
+      <c r="A58" s="8">
         <v>290</v>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="8">
         <v>1</v>
       </c>
-      <c r="C58" s="9" t="s">
-        <v>989</v>
-      </c>
-      <c r="D58" s="9" t="s">
+      <c r="C58" s="8" t="s">
+        <v>989</v>
+      </c>
+      <c r="D58" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E58" s="9" t="s">
+      <c r="E58" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F58" s="9" t="s">
+      <c r="F58" s="8" t="s">
         <v>2098</v>
       </c>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
     </row>
     <row r="59" spans="1:8">
-      <c r="A59" s="9">
+      <c r="A59" s="8">
         <v>100</v>
       </c>
-      <c r="B59" s="9">
+      <c r="B59" s="8">
         <v>1</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="8" t="s">
         <v>1429</v>
       </c>
-      <c r="D59" s="9" t="s">
+      <c r="D59" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E59" s="9" t="s">
+      <c r="E59" s="8" t="s">
         <v>2099</v>
       </c>
-      <c r="F59" s="9" t="s">
+      <c r="F59" s="8" t="s">
         <v>2100</v>
       </c>
-      <c r="G59" s="10"/>
-      <c r="H59" s="10"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
     </row>
     <row r="60" spans="1:8">
-      <c r="A60" s="9">
+      <c r="A60" s="8">
         <v>280</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="8">
         <v>1</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="8" t="s">
         <v>1429</v>
       </c>
-      <c r="D60" s="9" t="s">
+      <c r="D60" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E60" s="9" t="s">
+      <c r="E60" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F60" s="9" t="s">
+      <c r="F60" s="8" t="s">
         <v>2100</v>
       </c>
-      <c r="G60" s="10"/>
-      <c r="H60" s="10"/>
+      <c r="G60" s="9"/>
+      <c r="H60" s="9"/>
     </row>
     <row r="61" spans="1:8">
-      <c r="A61" s="9">
+      <c r="A61" s="8">
         <v>120</v>
       </c>
-      <c r="B61" s="9">
+      <c r="B61" s="8">
         <v>1</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="8" t="s">
         <v>1660</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="D61" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E61" s="9" t="s">
+      <c r="E61" s="8" t="s">
         <v>2103</v>
       </c>
-      <c r="F61" s="9" t="s">
+      <c r="F61" s="8" t="s">
         <v>2104</v>
       </c>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
+      <c r="G61" s="9"/>
+      <c r="H61" s="9"/>
     </row>
     <row r="62" spans="1:8">
-      <c r="A62" s="9">
+      <c r="A62" s="8">
         <v>310</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62" s="8">
         <v>1</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="C62" s="8" t="s">
         <v>1660</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="D62" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E62" s="9" t="s">
+      <c r="E62" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F62" s="9" t="s">
+      <c r="F62" s="8" t="s">
         <v>2104</v>
       </c>
-      <c r="G62" s="10"/>
-      <c r="H62" s="10"/>
+      <c r="G62" s="9"/>
+      <c r="H62" s="9"/>
     </row>
     <row r="63" spans="1:8">
-      <c r="A63" s="9">
+      <c r="A63" s="8">
         <v>190</v>
       </c>
-      <c r="B63" s="9">
+      <c r="B63" s="8">
         <v>1</v>
       </c>
-      <c r="C63" s="9" t="s">
+      <c r="C63" s="8" t="s">
         <v>1732</v>
       </c>
-      <c r="D63" s="9" t="s">
+      <c r="D63" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E63" s="9" t="s">
+      <c r="E63" s="8" t="s">
         <v>2115</v>
       </c>
-      <c r="F63" s="9" t="s">
+      <c r="F63" s="8" t="s">
         <v>2116</v>
       </c>
-      <c r="G63" s="10"/>
-      <c r="H63" s="10"/>
+      <c r="G63" s="9"/>
+      <c r="H63" s="9"/>
     </row>
     <row r="64" spans="1:8">
-      <c r="A64" s="9">
+      <c r="A64" s="8">
         <v>400</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="8">
         <v>1</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="8" t="s">
         <v>1732</v>
       </c>
-      <c r="D64" s="9" t="s">
+      <c r="D64" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E64" s="9" t="s">
+      <c r="E64" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F64" s="9" t="s">
+      <c r="F64" s="8" t="s">
         <v>2116</v>
       </c>
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
+      <c r="G64" s="9"/>
+      <c r="H64" s="9"/>
     </row>
     <row r="65" spans="1:8">
-      <c r="A65" s="9">
+      <c r="A65" s="8">
         <v>420</v>
       </c>
-      <c r="B65" s="9">
+      <c r="B65" s="8">
         <v>1</v>
       </c>
-      <c r="C65" s="9" t="s">
+      <c r="C65" s="8" t="s">
         <v>1811</v>
       </c>
-      <c r="D65" s="9" t="s">
+      <c r="D65" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E65" s="9" t="s">
+      <c r="E65" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F65" s="9" t="s">
+      <c r="F65" s="8" t="s">
         <v>2534</v>
       </c>
-      <c r="G65" s="10"/>
-      <c r="H65" s="10"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
     </row>
     <row r="66" spans="1:8">
-      <c r="A66" s="9">
+      <c r="A66" s="8">
         <v>200</v>
       </c>
-      <c r="B66" s="9">
+      <c r="B66" s="8">
         <v>1</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C66" s="8" t="s">
         <v>1826</v>
       </c>
-      <c r="D66" s="9" t="s">
+      <c r="D66" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E66" s="9" t="s">
+      <c r="E66" s="8" t="s">
         <v>2117</v>
       </c>
-      <c r="F66" s="9" t="s">
+      <c r="F66" s="8" t="s">
         <v>2118</v>
       </c>
-      <c r="G66" s="10"/>
-      <c r="H66" s="10"/>
+      <c r="G66" s="9"/>
+      <c r="H66" s="9"/>
     </row>
     <row r="67" spans="1:8">
-      <c r="A67" s="9">
+      <c r="A67" s="8">
         <v>410</v>
       </c>
-      <c r="B67" s="9">
+      <c r="B67" s="8">
         <v>1</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="8" t="s">
         <v>1826</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D67" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E67" s="9" t="s">
+      <c r="E67" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F67" s="9" t="s">
+      <c r="F67" s="8" t="s">
         <v>2118</v>
       </c>
-      <c r="G67" s="10"/>
-      <c r="H67" s="10"/>
+      <c r="G67" s="9"/>
+      <c r="H67" s="9"/>
     </row>
     <row r="68" spans="1:8">
-      <c r="A68" s="9">
+      <c r="A68" s="8">
         <v>430</v>
       </c>
-      <c r="B68" s="9">
+      <c r="B68" s="8">
         <v>1</v>
       </c>
-      <c r="C68" s="13" t="s">
+      <c r="C68" s="12" t="s">
         <v>1902</v>
       </c>
-      <c r="D68" s="9" t="s">
+      <c r="D68" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E68" s="9" t="s">
+      <c r="E68" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="F68" s="9" t="s">
+      <c r="F68" s="8" t="s">
         <v>2178</v>
       </c>
-      <c r="G68" s="10"/>
-      <c r="H68" s="10"/>
+      <c r="G68" s="9"/>
+      <c r="H68" s="9"/>
     </row>
     <row r="69" spans="1:8" ht="45">
-      <c r="A69" s="9">
+      <c r="A69" s="8">
         <v>80</v>
       </c>
-      <c r="B69" s="9">
+      <c r="B69" s="8">
         <v>1</v>
       </c>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9" t="s">
+      <c r="C69" s="8"/>
+      <c r="D69" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E69" s="9" t="s">
+      <c r="E69" s="8" t="s">
         <v>2428</v>
       </c>
-      <c r="F69" s="9" t="s">
+      <c r="F69" s="8" t="s">
         <v>2096</v>
       </c>
-      <c r="G69" s="10"/>
-      <c r="H69" s="10"/>
+      <c r="G69" s="9"/>
+      <c r="H69" s="9"/>
     </row>
     <row r="70" spans="1:8">
-      <c r="A70" s="9">
+      <c r="A70" s="8">
         <v>670</v>
       </c>
-      <c r="B70" s="10">
+      <c r="B70" s="9">
         <v>1</v>
       </c>
-      <c r="C70" s="10"/>
-      <c r="D70" s="10" t="s">
+      <c r="C70" s="9"/>
+      <c r="D70" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E70" s="10" t="s">
+      <c r="E70" s="9" t="s">
         <v>2537</v>
       </c>
-      <c r="F70" s="10" t="s">
+      <c r="F70" s="9" t="s">
         <v>2096</v>
       </c>
-      <c r="G70" s="10"/>
-      <c r="H70" s="10"/>
+      <c r="G70" s="9"/>
+      <c r="H70" s="9"/>
     </row>
     <row r="71" spans="1:8">
-      <c r="A71" s="9">
+      <c r="A71" s="8">
         <v>560</v>
       </c>
-      <c r="B71" s="9">
+      <c r="B71" s="8">
         <v>1</v>
       </c>
-      <c r="C71" s="10"/>
-      <c r="D71" s="9" t="s">
+      <c r="C71" s="9"/>
+      <c r="D71" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E71" s="10" t="s">
+      <c r="E71" s="9" t="s">
         <v>2541</v>
       </c>
-      <c r="F71" s="10" t="s">
+      <c r="F71" s="9" t="s">
         <v>2183</v>
       </c>
-      <c r="G71" s="10"/>
-      <c r="H71" s="10"/>
+      <c r="G71" s="9"/>
+      <c r="H71" s="9"/>
     </row>
     <row r="72" spans="1:8">
-      <c r="A72" s="9">
+      <c r="A72" s="8">
         <v>690</v>
       </c>
-      <c r="B72" s="10">
+      <c r="B72" s="9">
         <v>1</v>
       </c>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10" t="s">
+      <c r="C72" s="9"/>
+      <c r="D72" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E72" s="10" t="s">
+      <c r="E72" s="9" t="s">
         <v>2447</v>
       </c>
-      <c r="F72" s="10" t="s">
+      <c r="F72" s="9" t="s">
         <v>2183</v>
       </c>
-      <c r="G72" s="10"/>
-      <c r="H72" s="10"/>
+      <c r="G72" s="9"/>
+      <c r="H72" s="9"/>
     </row>
     <row r="73" spans="1:8">
-      <c r="A73" s="9">
+      <c r="A73" s="8">
         <v>60</v>
       </c>
-      <c r="B73" s="9">
+      <c r="B73" s="8">
         <v>1</v>
       </c>
-      <c r="C73" s="8"/>
-      <c r="D73" s="9" t="s">
+      <c r="C73" s="7"/>
+      <c r="D73" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E73" s="9" t="s">
+      <c r="E73" s="8" t="s">
         <v>2092</v>
       </c>
-      <c r="F73" s="9" t="s">
+      <c r="F73" s="8" t="s">
         <v>2093</v>
       </c>
-      <c r="G73" s="10"/>
-      <c r="H73" s="10"/>
+      <c r="G73" s="9"/>
+      <c r="H73" s="9"/>
     </row>
     <row r="74" spans="1:8" ht="30">
-      <c r="A74" s="9">
+      <c r="A74" s="8">
         <v>30</v>
       </c>
-      <c r="B74" s="9">
+      <c r="B74" s="8">
         <v>1</v>
       </c>
-      <c r="C74" s="9"/>
-      <c r="D74" s="9" t="s">
+      <c r="C74" s="8"/>
+      <c r="D74" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E74" s="9" t="s">
+      <c r="E74" s="8" t="s">
         <v>2497</v>
       </c>
-      <c r="F74" s="9" t="s">
+      <c r="F74" s="8" t="s">
         <v>2088</v>
       </c>
-      <c r="G74" s="10"/>
-      <c r="H74" s="10"/>
+      <c r="G74" s="9"/>
+      <c r="H74" s="9"/>
     </row>
     <row r="75" spans="1:8">
-      <c r="A75" s="9">
+      <c r="A75" s="8">
         <v>650</v>
       </c>
-      <c r="B75" s="10">
+      <c r="B75" s="9">
         <v>1</v>
       </c>
-      <c r="C75" s="10"/>
-      <c r="D75" s="10" t="s">
+      <c r="C75" s="9"/>
+      <c r="D75" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E75" s="10" t="s">
+      <c r="E75" s="9" t="s">
         <v>2444</v>
       </c>
-      <c r="F75" s="10" t="s">
+      <c r="F75" s="9" t="s">
         <v>2088</v>
       </c>
-      <c r="G75" s="10"/>
-      <c r="H75" s="10"/>
+      <c r="G75" s="9"/>
+      <c r="H75" s="9"/>
     </row>
     <row r="76" spans="1:8">
-      <c r="A76" s="9">
+      <c r="A76" s="8">
         <v>730</v>
       </c>
-      <c r="B76" s="10">
+      <c r="B76" s="9">
         <v>1</v>
       </c>
-      <c r="C76" s="10"/>
-      <c r="D76" s="10" t="s">
+      <c r="C76" s="9"/>
+      <c r="D76" s="9" t="s">
         <v>2057</v>
       </c>
-      <c r="E76" s="10" t="s">
+      <c r="E76" s="9" t="s">
         <v>2451</v>
       </c>
-      <c r="F76" s="10" t="s">
+      <c r="F76" s="9" t="s">
         <v>2088</v>
       </c>
-      <c r="G76" s="10"/>
-      <c r="H76" s="10"/>
+      <c r="G76" s="9"/>
+      <c r="H76" s="9"/>
     </row>
     <row r="77" spans="1:8">
-      <c r="A77" s="9">
+      <c r="A77" s="8">
         <v>40</v>
       </c>
-      <c r="B77" s="9">
+      <c r="B77" s="8">
         <v>1</v>
       </c>
-      <c r="C77" s="9"/>
-      <c r="D77" s="9" t="s">
+      <c r="C77" s="8"/>
+      <c r="D77" s="8" t="s">
         <v>2057</v>
       </c>
-      <c r="E77" s="9" t="s">
+      <c r="E77" s="8" t="s">
         <v>2540</v>
       </c>
-      <c r="F77" s="9" t="s">
+      <c r="F77" s="8" t="s">
         <v>2089</v>
       </c>
-      <c r="G77" s="10"/>
-      <c r="H77" s="10"/>
+      <c r="G77" s="9"/>
+      <c r="H77" s="9"/>
     </row>
     <row r="78" spans="1:8">
-      <c r="A78" s="10"/>
-      <c r="B78" s="10"/>
-      <c r="C78" s="10"/>
-      <c r="D78" s="10"/>
-      <c r="E78" s="10"/>
-      <c r="F78" s="10"/>
-      <c r="G78" s="10"/>
-      <c r="H78" s="10"/>
+      <c r="A78" s="9"/>
+      <c r="B78" s="9"/>
+      <c r="C78" s="9"/>
+      <c r="D78" s="9"/>
+      <c r="E78" s="9"/>
+      <c r="F78" s="9"/>
+      <c r="G78" s="9"/>
+      <c r="H78" s="9"/>
     </row>
     <row r="79" spans="1:8">
-      <c r="A79" s="10"/>
-      <c r="B79" s="10"/>
-      <c r="C79" s="10"/>
-      <c r="D79" s="10"/>
-      <c r="E79" s="10"/>
-      <c r="F79" s="10"/>
-      <c r="G79" s="10"/>
-      <c r="H79" s="10"/>
+      <c r="A79" s="9"/>
+      <c r="B79" s="9"/>
+      <c r="C79" s="9"/>
+      <c r="D79" s="9"/>
+      <c r="E79" s="9"/>
+      <c r="F79" s="9"/>
+      <c r="G79" s="9"/>
+      <c r="H79" s="9"/>
     </row>
     <row r="80" spans="1:8">
-      <c r="A80" s="10"/>
-      <c r="B80" s="10"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="10"/>
-      <c r="E80" s="10"/>
-      <c r="F80" s="10"/>
-      <c r="G80" s="10"/>
-      <c r="H80" s="10"/>
+      <c r="A80" s="9"/>
+      <c r="B80" s="9"/>
+      <c r="C80" s="9"/>
+      <c r="D80" s="9"/>
+      <c r="E80" s="9"/>
+      <c r="F80" s="9"/>
+      <c r="G80" s="9"/>
+      <c r="H80" s="9"/>
     </row>
     <row r="81" spans="1:8">
-      <c r="A81" s="10"/>
-      <c r="B81" s="10"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="10"/>
-      <c r="E81" s="10"/>
-      <c r="F81" s="10"/>
-      <c r="G81" s="10"/>
-      <c r="H81" s="10"/>
+      <c r="A81" s="9"/>
+      <c r="B81" s="9"/>
+      <c r="C81" s="9"/>
+      <c r="D81" s="9"/>
+      <c r="E81" s="9"/>
+      <c r="F81" s="9"/>
+      <c r="G81" s="9"/>
+      <c r="H81" s="9"/>
     </row>
     <row r="82" spans="1:8">
-      <c r="A82" s="10"/>
-      <c r="B82" s="10"/>
-      <c r="C82" s="10"/>
-      <c r="D82" s="10"/>
-      <c r="E82" s="10"/>
-      <c r="F82" s="10"/>
-      <c r="G82" s="10"/>
-      <c r="H82" s="10"/>
+      <c r="A82" s="9"/>
+      <c r="B82" s="9"/>
+      <c r="C82" s="9"/>
+      <c r="D82" s="9"/>
+      <c r="E82" s="9"/>
+      <c r="F82" s="9"/>
+      <c r="G82" s="9"/>
+      <c r="H82" s="9"/>
     </row>
     <row r="83" spans="1:8">
-      <c r="A83" s="10"/>
-      <c r="B83" s="10"/>
-      <c r="C83" s="10"/>
-      <c r="D83" s="10"/>
-      <c r="E83" s="10"/>
-      <c r="F83" s="10"/>
-      <c r="G83" s="10"/>
-      <c r="H83" s="10"/>
+      <c r="A83" s="9"/>
+      <c r="B83" s="9"/>
+      <c r="C83" s="9"/>
+      <c r="D83" s="9"/>
+      <c r="E83" s="9"/>
+      <c r="F83" s="9"/>
+      <c r="G83" s="9"/>
+      <c r="H83" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F46">

</xml_diff>

<commit_message>
feat: Add combined sections configuration for static part summary and update related tests
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">branch!$A$1:$B$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">comment_synonyms!$A$1:$D$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">defect_category!$A$1:$D$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">factory!$A$1:$B$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">factory!$A$1:$C$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">panel_usage!$A$1:$B$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">part_list!$A$1:$B$1834</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">symptom!$A$1:$F$91</definedName>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5074" uniqueCount="2570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5203" uniqueCount="2578">
   <si>
     <t>part_used</t>
   </si>
@@ -7746,6 +7746,30 @@
   </si>
   <si>
     <t>LC40SA5100I</t>
+  </si>
+  <si>
+    <t>series</t>
+  </si>
+  <si>
+    <t>2TC24CB3I</t>
+  </si>
+  <si>
+    <t>2TC32BB1I</t>
+  </si>
+  <si>
+    <t>2TC32BD1I</t>
+  </si>
+  <si>
+    <t>9TAHL6500IP004</t>
+  </si>
+  <si>
+    <t>RUNTKC242WJN1</t>
+  </si>
+  <si>
+    <t>PEVA-A042VDZZ</t>
+  </si>
+  <si>
+    <t>RSNSZA025QBZZ</t>
   </si>
 </sst>
 </file>
@@ -8210,7 +8234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1837"/>
+  <dimension ref="A1:B1841"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -22913,6 +22937,38 @@
         <v>1826</v>
       </c>
     </row>
+    <row r="1838" spans="1:2">
+      <c r="A1838" t="s">
+        <v>2574</v>
+      </c>
+      <c r="B1838" s="7" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="1839" spans="1:2">
+      <c r="A1839" t="s">
+        <v>2575</v>
+      </c>
+      <c r="B1839" s="7" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="1840" spans="1:2">
+      <c r="A1840" t="s">
+        <v>2576</v>
+      </c>
+      <c r="B1840" s="7" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="1841" spans="1:2">
+      <c r="A1841" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B1841" s="7" t="s">
+        <v>964</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B1834"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22921,982 +22977,1351 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B121"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
         <v>1940</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1941</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="17" t="s">
-        <v>1942</v>
+      <c r="C1" s="2" t="s">
+        <v>2570</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="12" t="s">
+        <v>2562</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>2571</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="17" t="s">
-        <v>1944</v>
+        <v>1960</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>1960</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="17" t="s">
-        <v>1945</v>
+        <v>1962</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>1962</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="17" t="s">
-        <v>1946</v>
+        <v>1963</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="17" t="s">
-        <v>1947</v>
+        <v>1964</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="17" t="s">
-        <v>1948</v>
+        <v>1965</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="17" t="s">
-        <v>1949</v>
+        <v>1966</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" s="17" t="s">
-        <v>1950</v>
+        <v>1967</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>1967</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10" s="17" t="s">
-        <v>1951</v>
+        <v>1968</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="17" t="s">
-        <v>1952</v>
+        <v>1969</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>2572</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="17" t="s">
-        <v>1953</v>
+        <v>1970</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>2573</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="17" t="s">
-        <v>1954</v>
+        <v>1971</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>1971</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="17" t="s">
-        <v>1955</v>
+        <v>1972</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>1956</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>1972</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" s="17" t="s">
-        <v>1957</v>
+        <v>1973</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>1956</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>1973</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="17" t="s">
-        <v>1958</v>
+        <v>1974</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>1956</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>1973</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="17" t="s">
-        <v>1959</v>
+        <v>1975</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>1956</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+        <v>1961</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>1975</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="17" t="s">
-        <v>1960</v>
+        <v>1976</v>
       </c>
       <c r="B18" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="C18" s="17" t="s">
+        <v>1976</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" s="17" t="s">
-        <v>1962</v>
+        <v>1977</v>
       </c>
       <c r="B19" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="20" spans="1:2">
+      <c r="C19" s="17" t="s">
+        <v>1979</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" s="17" t="s">
-        <v>1963</v>
+        <v>1978</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="C20" s="17" t="s">
+        <v>1979</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" s="17" t="s">
-        <v>1964</v>
+        <v>1979</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="22" spans="1:2">
+      <c r="C21" s="17" t="s">
+        <v>1979</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="A22" s="17" t="s">
-        <v>1965</v>
+        <v>2013</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
+        <v>2014</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="A23" s="17" t="s">
-        <v>1966</v>
+        <v>1942</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>1944</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
       <c r="A24" s="17" t="s">
-        <v>1967</v>
+        <v>1944</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>1944</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
       <c r="A25" s="17" t="s">
-        <v>1968</v>
+        <v>1980</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="A26" s="17" t="s">
-        <v>1969</v>
+      <c r="C25" s="17" t="s">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="12" t="s">
+        <v>2563</v>
       </c>
       <c r="B26" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="27" spans="1:2">
+      <c r="C26" s="17" t="s">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" s="17" t="s">
-        <v>1970</v>
+        <v>1981</v>
       </c>
       <c r="B27" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="28" spans="1:2">
+      <c r="C27" s="17" t="s">
+        <v>1981</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
       <c r="A28" s="17" t="s">
-        <v>1971</v>
+        <v>1982</v>
       </c>
       <c r="B28" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="29" spans="1:2">
+      <c r="C28" s="17" t="s">
+        <v>1982</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
       <c r="A29" s="17" t="s">
-        <v>1972</v>
+        <v>1983</v>
       </c>
       <c r="B29" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="30" spans="1:2">
+      <c r="C29" s="17" t="s">
+        <v>1983</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
       <c r="A30" s="17" t="s">
-        <v>1973</v>
+        <v>1984</v>
       </c>
       <c r="B30" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="31" spans="1:2">
+      <c r="C30" s="17" t="s">
+        <v>1984</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
       <c r="A31" s="17" t="s">
-        <v>1974</v>
+        <v>1985</v>
       </c>
       <c r="B31" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="32" spans="1:2">
+      <c r="C31" s="17" t="s">
+        <v>1984</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
       <c r="A32" s="17" t="s">
-        <v>1975</v>
+        <v>1986</v>
       </c>
       <c r="B32" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="33" spans="1:2">
+      <c r="C32" s="17" t="s">
+        <v>1986</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33" s="17" t="s">
-        <v>1976</v>
+        <v>1987</v>
       </c>
       <c r="B33" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
+      <c r="C33" s="17" t="s">
+        <v>1987</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="A34" s="17" t="s">
-        <v>1977</v>
+        <v>1988</v>
       </c>
       <c r="B34" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="35" spans="1:2">
+      <c r="C34" s="17" t="s">
+        <v>1987</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
       <c r="A35" s="17" t="s">
-        <v>1978</v>
+        <v>1989</v>
       </c>
       <c r="B35" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="36" spans="1:2">
+      <c r="C35" s="17" t="s">
+        <v>1989</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
       <c r="A36" s="17" t="s">
-        <v>1979</v>
+        <v>1990</v>
       </c>
       <c r="B36" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="37" spans="1:2">
+      <c r="C36" s="17" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" s="17" t="s">
-        <v>1980</v>
+        <v>2015</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
+        <v>2014</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38" s="17" t="s">
-        <v>1981</v>
+        <v>1991</v>
       </c>
       <c r="B38" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="39" spans="1:2">
-      <c r="A39" s="17" t="s">
-        <v>1982</v>
+      <c r="C38" s="17" t="s">
+        <v>1991</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="15" t="s">
+        <v>2452</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="17" t="s">
-        <v>1983</v>
+        <v>2488</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>2452</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="15" t="s">
+        <v>2453</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>2453</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41" s="17" t="s">
-        <v>1984</v>
+        <v>1992</v>
       </c>
       <c r="B41" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="42" spans="1:2">
+      <c r="C41" s="17" t="s">
+        <v>1992</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
       <c r="A42" s="17" t="s">
-        <v>1985</v>
+        <v>1993</v>
       </c>
       <c r="B42" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="43" spans="1:2">
+      <c r="C42" s="17" t="s">
+        <v>1993</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
       <c r="A43" s="17" t="s">
-        <v>1986</v>
+        <v>1994</v>
       </c>
       <c r="B43" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="44" spans="1:2">
+      <c r="C43" s="17" t="s">
+        <v>1994</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44" s="17" t="s">
-        <v>1987</v>
+        <v>1995</v>
       </c>
       <c r="B44" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="45" spans="1:2">
+      <c r="C44" s="17" t="s">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
       <c r="A45" s="17" t="s">
-        <v>1988</v>
+        <v>1996</v>
       </c>
       <c r="B45" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="46" spans="1:2">
+      <c r="C45" s="17" t="s">
+        <v>1996</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
       <c r="A46" s="17" t="s">
-        <v>1989</v>
+        <v>1997</v>
       </c>
       <c r="B46" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="47" spans="1:2">
+      <c r="C46" s="17" t="s">
+        <v>1997</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
       <c r="A47" s="17" t="s">
-        <v>1990</v>
+        <v>1998</v>
       </c>
       <c r="B47" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="48" spans="1:2">
+      <c r="C47" s="17" t="s">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
       <c r="A48" s="17" t="s">
-        <v>1991</v>
+        <v>1945</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="A49" s="17" t="s">
-        <v>1992</v>
+        <v>1943</v>
+      </c>
+      <c r="C48" s="17" t="s">
+        <v>1945</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="15" t="s">
+        <v>2454</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C49" s="15" t="s">
+        <v>2454</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
       <c r="A50" s="17" t="s">
-        <v>1993</v>
+        <v>1999</v>
       </c>
       <c r="B50" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="51" spans="1:2">
+      <c r="C50" s="17" t="s">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
       <c r="A51" s="17" t="s">
-        <v>1994</v>
+        <v>2000</v>
       </c>
       <c r="B51" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="A52" s="17" t="s">
-        <v>1995</v>
+      <c r="C51" s="17" t="s">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="15" t="s">
+        <v>2455</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C52" s="15" t="s">
+        <v>2455</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
       <c r="A53" s="17" t="s">
-        <v>1996</v>
+        <v>1955</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="A54" s="17" t="s">
-        <v>1997</v>
+        <v>1956</v>
+      </c>
+      <c r="C53" s="17" t="s">
+        <v>1955</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="15" t="s">
+        <v>2456</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C54" s="15" t="s">
+        <v>2456</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
       <c r="A55" s="17" t="s">
-        <v>1998</v>
+        <v>2001</v>
       </c>
       <c r="B55" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="56" spans="1:2">
+      <c r="C55" s="17" t="s">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
       <c r="A56" s="17" t="s">
-        <v>1999</v>
+        <v>1946</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C56" s="17" t="s">
+        <v>1946</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
       <c r="A57" s="17" t="s">
-        <v>2000</v>
+        <v>1947</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" s="17" t="s">
-        <v>2001</v>
+        <v>1943</v>
+      </c>
+      <c r="C57" s="17" t="s">
+        <v>1947</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="15" t="s">
+        <v>2457</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="A59" s="17" t="s">
-        <v>2002</v>
+        <v>2489</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>2457</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="15" t="s">
+        <v>2458</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2">
+        <v>2489</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>2458</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
       <c r="A60" s="17" t="s">
-        <v>2003</v>
+        <v>1957</v>
       </c>
       <c r="B60" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2">
-      <c r="A61" s="17" t="s">
-        <v>2004</v>
+        <v>1956</v>
+      </c>
+      <c r="C60" s="17" t="s">
+        <v>1957</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="15" t="s">
+        <v>2459</v>
       </c>
       <c r="B61" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2">
-      <c r="A62" s="17" t="s">
-        <v>2005</v>
+        <v>2488</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>2459</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="15" t="s">
+        <v>2460</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2">
-      <c r="A63" s="17" t="s">
-        <v>2006</v>
+        <v>2488</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="15" t="s">
+        <v>2461</v>
       </c>
       <c r="B63" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C63" s="15" t="s">
+        <v>2461</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
       <c r="A64" s="17" t="s">
-        <v>2007</v>
+        <v>1948</v>
       </c>
       <c r="B64" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C64" s="17" t="s">
+        <v>1948</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
       <c r="A65" s="17" t="s">
-        <v>2008</v>
+        <v>1949</v>
       </c>
       <c r="B65" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C65" s="17" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
       <c r="A66" s="17" t="s">
-        <v>2009</v>
+        <v>1950</v>
       </c>
       <c r="B66" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2">
-      <c r="A67" s="17" t="s">
-        <v>2010</v>
+        <v>1943</v>
+      </c>
+      <c r="C66" s="17" t="s">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="15" t="s">
+        <v>2462</v>
       </c>
       <c r="B67" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2">
-      <c r="A68" s="17" t="s">
-        <v>2011</v>
+        <v>2488</v>
+      </c>
+      <c r="C67" s="15" t="s">
+        <v>2462</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="15" t="s">
+        <v>2463</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2">
-      <c r="A69" s="17" t="s">
-        <v>2012</v>
+        <v>2488</v>
+      </c>
+      <c r="C68" s="15" t="s">
+        <v>2463</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="15" t="s">
+        <v>2464</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2">
-      <c r="A70" s="17" t="s">
-        <v>2013</v>
+        <v>2488</v>
+      </c>
+      <c r="C69" s="15" t="s">
+        <v>2464</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="15" t="s">
+        <v>2465</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>2014</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2">
-      <c r="A71" s="17" t="s">
-        <v>2015</v>
+        <v>2488</v>
+      </c>
+      <c r="C70" s="15" t="s">
+        <v>2465</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="15" t="s">
+        <v>2466</v>
       </c>
       <c r="B71" s="17" t="s">
-        <v>2014</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C71" s="15" t="s">
+        <v>2466</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
       <c r="A72" s="15" t="s">
-        <v>2452</v>
+        <v>2467</v>
       </c>
       <c r="B72" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="73" spans="1:2">
+      <c r="C72" s="15" t="s">
+        <v>2467</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
       <c r="A73" s="15" t="s">
-        <v>2453</v>
+        <v>2468</v>
       </c>
       <c r="B73" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="74" spans="1:2">
+      <c r="C73" s="15" t="s">
+        <v>2468</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
       <c r="A74" s="15" t="s">
-        <v>2454</v>
+        <v>2469</v>
       </c>
       <c r="B74" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="75" spans="1:2">
+      <c r="C74" s="15" t="s">
+        <v>2469</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
       <c r="A75" s="15" t="s">
-        <v>2455</v>
+        <v>2470</v>
       </c>
       <c r="B75" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="76" spans="1:2">
-      <c r="A76" s="15" t="s">
-        <v>2456</v>
+      <c r="C75" s="15" t="s">
+        <v>2470</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="17" t="s">
+        <v>1958</v>
       </c>
       <c r="B76" s="17" t="s">
+        <v>1956</v>
+      </c>
+      <c r="C76" s="17" t="s">
+        <v>1958</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="15" t="s">
+        <v>2471</v>
+      </c>
+      <c r="B77" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="77" spans="1:2">
-      <c r="A77" s="15" t="s">
-        <v>2457</v>
-      </c>
-      <c r="B77" s="17" t="s">
-        <v>2489</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2">
+      <c r="C77" s="15" t="s">
+        <v>2471</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
       <c r="A78" s="15" t="s">
-        <v>2458</v>
+        <v>2472</v>
       </c>
       <c r="B78" s="17" t="s">
-        <v>2489</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>2472</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
       <c r="A79" s="15" t="s">
-        <v>2459</v>
+        <v>2473</v>
       </c>
       <c r="B79" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="80" spans="1:2">
+      <c r="C79" s="15" t="s">
+        <v>2473</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
       <c r="A80" s="15" t="s">
-        <v>2460</v>
+        <v>2474</v>
       </c>
       <c r="B80" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="81" spans="1:2">
-      <c r="A81" s="15" t="s">
-        <v>2461</v>
+      <c r="C80" s="15" t="s">
+        <v>2474</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" s="17" t="s">
+        <v>1951</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2">
-      <c r="A82" s="15" t="s">
-        <v>2462</v>
+        <v>1943</v>
+      </c>
+      <c r="C81" s="17" t="s">
+        <v>1951</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="17" t="s">
+        <v>1952</v>
       </c>
       <c r="B82" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C82" s="17" t="s">
+        <v>1952</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
       <c r="A83" s="15" t="s">
-        <v>2463</v>
+        <v>2500</v>
       </c>
       <c r="B83" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C83" s="15" t="s">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
       <c r="A84" s="15" t="s">
-        <v>2464</v>
+        <v>2501</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C84" s="15" t="s">
+        <v>2501</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
       <c r="A85" s="15" t="s">
-        <v>2465</v>
+        <v>2475</v>
       </c>
       <c r="B85" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="86" spans="1:2">
+      <c r="C85" s="15" t="s">
+        <v>2475</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
       <c r="A86" s="15" t="s">
-        <v>2466</v>
+        <v>2476</v>
       </c>
       <c r="B86" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="87" spans="1:2">
+      <c r="C86" s="15" t="s">
+        <v>2476</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
       <c r="A87" s="15" t="s">
-        <v>2467</v>
+        <v>2477</v>
       </c>
       <c r="B87" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="88" spans="1:2">
+      <c r="C87" s="15" t="s">
+        <v>2477</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
       <c r="A88" s="15" t="s">
-        <v>2468</v>
+        <v>2478</v>
       </c>
       <c r="B88" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="89" spans="1:2">
+      <c r="C88" s="15" t="s">
+        <v>2478</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
       <c r="A89" s="15" t="s">
-        <v>2469</v>
+        <v>2479</v>
       </c>
       <c r="B89" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="90" spans="1:2">
+      <c r="C89" s="15" t="s">
+        <v>2479</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
       <c r="A90" s="15" t="s">
-        <v>2470</v>
+        <v>2480</v>
       </c>
       <c r="B90" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="91" spans="1:2">
+      <c r="C90" s="15" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3">
       <c r="A91" s="15" t="s">
-        <v>2471</v>
+        <v>2481</v>
       </c>
       <c r="B91" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2">
-      <c r="A92" s="15" t="s">
-        <v>2472</v>
+        <v>2489</v>
+      </c>
+      <c r="C91" s="15" t="s">
+        <v>2481</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" s="17" t="s">
+        <v>1959</v>
       </c>
       <c r="B92" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2">
+        <v>1956</v>
+      </c>
+      <c r="C92" s="17" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3">
       <c r="A93" s="15" t="s">
-        <v>2473</v>
+        <v>2482</v>
       </c>
       <c r="B93" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="94" spans="1:2">
-      <c r="A94" s="15" t="s">
-        <v>2474</v>
+      <c r="C93" s="15" t="s">
+        <v>2482</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" s="18" t="s">
+        <v>2498</v>
       </c>
       <c r="B94" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="95" spans="1:2">
-      <c r="A95" s="15" t="s">
-        <v>2475</v>
+      <c r="C94" s="18" t="s">
+        <v>2498</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" s="17" t="s">
+        <v>1953</v>
       </c>
       <c r="B95" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C95" s="17" t="s">
+        <v>1953</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3">
       <c r="A96" s="15" t="s">
-        <v>2476</v>
+        <v>2503</v>
       </c>
       <c r="B96" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2">
-      <c r="A97" s="15" t="s">
-        <v>2477</v>
+        <v>1943</v>
+      </c>
+      <c r="C96" s="15" t="s">
+        <v>2503</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" s="17" t="s">
+        <v>1954</v>
       </c>
       <c r="B97" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C97" s="17" t="s">
+        <v>1954</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
       <c r="A98" s="15" t="s">
-        <v>2478</v>
+        <v>2502</v>
       </c>
       <c r="B98" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C98" s="15" t="s">
+        <v>2502</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
       <c r="A99" s="15" t="s">
-        <v>2479</v>
+        <v>2483</v>
       </c>
       <c r="B99" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2">
-      <c r="A100" s="15" t="s">
-        <v>2480</v>
+        <v>1943</v>
+      </c>
+      <c r="C99" s="15" t="s">
+        <v>2483</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" s="18" t="s">
+        <v>2499</v>
       </c>
       <c r="B100" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="101" spans="1:2">
+      <c r="C100" s="18" t="s">
+        <v>2499</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
       <c r="A101" s="15" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
       <c r="B101" s="17" t="s">
-        <v>2489</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2">
+        <v>1943</v>
+      </c>
+      <c r="C101" s="15" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3">
       <c r="A102" s="15" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
       <c r="B102" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="103" spans="1:2">
-      <c r="A103" s="15" t="s">
-        <v>2483</v>
+      <c r="C102" s="15" t="s">
+        <v>2485</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3">
+      <c r="A103" s="17" t="s">
+        <v>2002</v>
       </c>
       <c r="B103" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2">
-      <c r="A104" s="15" t="s">
-        <v>2484</v>
+        <v>1961</v>
+      </c>
+      <c r="C103" s="17" t="s">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3">
+      <c r="A104" s="12" t="s">
+        <v>2564</v>
       </c>
       <c r="B104" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2">
-      <c r="A105" s="15" t="s">
-        <v>2485</v>
+        <v>1961</v>
+      </c>
+      <c r="C104" s="12" t="s">
+        <v>2564</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="A105" s="17" t="s">
+        <v>2003</v>
       </c>
       <c r="B105" s="17" t="s">
+        <v>1961</v>
+      </c>
+      <c r="C105" s="17" t="s">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3">
+      <c r="A106" s="12" t="s">
+        <v>2565</v>
+      </c>
+      <c r="B106" s="17" t="s">
+        <v>1961</v>
+      </c>
+      <c r="C106" s="12" t="s">
+        <v>2565</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3">
+      <c r="A107" s="17" t="s">
+        <v>2004</v>
+      </c>
+      <c r="B107" s="17" t="s">
+        <v>1961</v>
+      </c>
+      <c r="C107" s="17" t="s">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="A108" s="17" t="s">
+        <v>2005</v>
+      </c>
+      <c r="B108" s="17" t="s">
+        <v>1961</v>
+      </c>
+      <c r="C108" s="17" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="A109" s="12" t="s">
+        <v>2566</v>
+      </c>
+      <c r="B109" s="17" t="s">
+        <v>1961</v>
+      </c>
+      <c r="C109" s="12" t="s">
+        <v>2566</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" s="15" t="s">
+        <v>2486</v>
+      </c>
+      <c r="B110" s="17" t="s">
         <v>2488</v>
       </c>
-    </row>
-    <row r="106" spans="1:2">
-      <c r="A106" s="15" t="s">
+      <c r="C110" s="15" t="s">
         <v>2486</v>
       </c>
-      <c r="B106" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2">
-      <c r="A107" s="15" t="s">
-        <v>2487</v>
-      </c>
-      <c r="B107" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2">
-      <c r="A108" s="18" t="s">
-        <v>2498</v>
-      </c>
-      <c r="B108" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2">
-      <c r="A109" s="18" t="s">
-        <v>2499</v>
-      </c>
-      <c r="B109" s="17" t="s">
-        <v>2488</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2">
-      <c r="A110" s="15" t="s">
-        <v>2500</v>
-      </c>
-      <c r="B110" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2">
-      <c r="A111" s="15" t="s">
-        <v>2501</v>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" s="17" t="s">
+        <v>2006</v>
       </c>
       <c r="B111" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2">
-      <c r="A112" s="15" t="s">
-        <v>2502</v>
+        <v>1961</v>
+      </c>
+      <c r="C111" s="17" t="s">
+        <v>2006</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" s="17" t="s">
+        <v>2007</v>
       </c>
       <c r="B112" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2">
-      <c r="A113" s="15" t="s">
-        <v>2503</v>
+        <v>1961</v>
+      </c>
+      <c r="C112" s="17" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" s="12" t="s">
+        <v>2567</v>
       </c>
       <c r="B113" s="17" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2">
-      <c r="A114" s="12" t="s">
-        <v>2562</v>
+        <v>1961</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114" s="17" t="s">
+        <v>2008</v>
       </c>
       <c r="B114" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="115" spans="1:2">
-      <c r="A115" s="12" t="s">
-        <v>2563</v>
+      <c r="C114" s="17" t="s">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" s="17" t="s">
+        <v>2009</v>
       </c>
       <c r="B115" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="116" spans="1:2">
-      <c r="A116" s="12" t="s">
-        <v>2564</v>
+      <c r="C115" s="17" t="s">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" s="17" t="s">
+        <v>2010</v>
       </c>
       <c r="B116" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="117" spans="1:2">
-      <c r="A117" s="12" t="s">
-        <v>2565</v>
+      <c r="C116" s="17" t="s">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" s="17" t="s">
+        <v>2011</v>
       </c>
       <c r="B117" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="118" spans="1:2">
+      <c r="C117" s="17" t="s">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3">
       <c r="A118" s="12" t="s">
-        <v>2566</v>
+        <v>2568</v>
       </c>
       <c r="B118" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="119" spans="1:2">
-      <c r="A119" s="12" t="s">
-        <v>2567</v>
+      <c r="C118" s="12" t="s">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" s="15" t="s">
+        <v>2487</v>
       </c>
       <c r="B119" s="17" t="s">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2">
+        <v>2488</v>
+      </c>
+      <c r="C119" s="15" t="s">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3">
       <c r="A120" s="12" t="s">
-        <v>2568</v>
+        <v>2569</v>
       </c>
       <c r="B120" s="17" t="s">
         <v>1961</v>
       </c>
-    </row>
-    <row r="121" spans="1:2">
-      <c r="A121" s="12" t="s">
+      <c r="C120" s="12" t="s">
         <v>2569</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3">
+      <c r="A121" s="17" t="s">
+        <v>2012</v>
       </c>
       <c r="B121" s="17" t="s">
         <v>1961</v>
       </c>
+      <c r="C121" s="17" t="s">
+        <v>2012</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1">
+    <sortState ref="A2:C121">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: enhance symptom matching by adding fallback source columns and update related tests
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5216" uniqueCount="2576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5225" uniqueCount="2577">
   <si>
     <t>part_used</t>
   </si>
@@ -7604,9 +7604,6 @@
     <t>DINYALAKAN|MENYALA</t>
   </si>
   <si>
-    <t>AFDA</t>
-  </si>
-  <si>
     <t>ADA</t>
   </si>
   <si>
@@ -7764,6 +7761,12 @@
   </si>
   <si>
     <t>ganti|replace|ir|sensor|LED IR</t>
+  </si>
+  <si>
+    <t>REPAIR_SHEET</t>
+  </si>
+  <si>
+    <t>AFDA|AADA</t>
   </si>
 </sst>
 </file>
@@ -22906,7 +22909,7 @@
     </row>
     <row r="1835" spans="1:2">
       <c r="A1835" s="6" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
       <c r="B1835" s="1" t="s">
         <v>459</v>
@@ -22914,7 +22917,7 @@
     </row>
     <row r="1836" spans="1:2">
       <c r="A1836" s="6" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="B1836" s="7" t="s">
         <v>459</v>
@@ -22922,7 +22925,7 @@
     </row>
     <row r="1837" spans="1:2">
       <c r="A1837" s="6" t="s">
-        <v>2530</v>
+        <v>2529</v>
       </c>
       <c r="B1837" s="1" t="s">
         <v>1826</v>
@@ -22930,7 +22933,7 @@
     </row>
     <row r="1838" spans="1:2">
       <c r="A1838" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="B1838" s="7" t="s">
         <v>1429</v>
@@ -22938,7 +22941,7 @@
     </row>
     <row r="1839" spans="1:2">
       <c r="A1839" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="B1839" s="7" t="s">
         <v>214</v>
@@ -22946,7 +22949,7 @@
     </row>
     <row r="1840" spans="1:2">
       <c r="A1840" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="B1840" s="7" t="s">
         <v>964</v>
@@ -22954,7 +22957,7 @@
     </row>
     <row r="1841" spans="1:2">
       <c r="A1841" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="B1841" s="7" t="s">
         <v>964</v>
@@ -22984,18 +22987,18 @@
         <v>1941</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="10" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>1961</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -23094,7 +23097,7 @@
         <v>1961</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -23105,7 +23108,7 @@
         <v>1961</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -23253,7 +23256,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="10" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>1961</v>
@@ -24111,13 +24114,13 @@
     </row>
     <row r="104" spans="1:3">
       <c r="A104" s="10" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
       <c r="B104" s="14" t="s">
         <v>1961</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -24133,13 +24136,13 @@
     </row>
     <row r="106" spans="1:3">
       <c r="A106" s="10" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
       <c r="B106" s="14" t="s">
         <v>1961</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -24166,13 +24169,13 @@
     </row>
     <row r="109" spans="1:3">
       <c r="A109" s="10" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
       <c r="B109" s="14" t="s">
         <v>1961</v>
       </c>
       <c r="C109" s="10" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -24210,7 +24213,7 @@
     </row>
     <row r="113" spans="1:3">
       <c r="A113" s="10" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
       <c r="B113" s="14" t="s">
         <v>1961</v>
@@ -24265,7 +24268,7 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" s="10" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
       <c r="B118" s="14" t="s">
         <v>1961</v>
@@ -24287,13 +24290,13 @@
     </row>
     <row r="120" spans="1:3">
       <c r="A120" s="10" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
       <c r="B120" s="14" t="s">
         <v>1961</v>
       </c>
       <c r="C120" s="10" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -24437,7 +24440,7 @@
         <v>2021</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>2042</v>
@@ -24455,7 +24458,7 @@
         <v>2021</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>2037</v>
@@ -24473,7 +24476,7 @@
         <v>2021</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>2539</v>
+        <v>2538</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>2041</v>
@@ -24589,7 +24592,7 @@
         <v>2021</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>2055</v>
@@ -24609,7 +24612,7 @@
         <v>2021</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>2553</v>
+        <v>2552</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>2045</v>
@@ -24822,7 +24825,7 @@
         <v>2021</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>2542</v>
+        <v>2541</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>2042</v>
@@ -24880,7 +24883,7 @@
         <v>2021</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>2037</v>
@@ -24920,7 +24923,7 @@
         <v>2021</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>2024</v>
@@ -24960,7 +24963,7 @@
         <v>2021</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>2055</v>
@@ -25078,7 +25081,7 @@
         <v>2021</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>2034</v>
@@ -25116,7 +25119,7 @@
         <v>2021</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>2525</v>
+        <v>2524</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>2515</v>
@@ -25234,7 +25237,7 @@
         <v>2021</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>2032</v>
@@ -25294,7 +25297,7 @@
         <v>2021</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>2554</v>
+        <v>2553</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>2025</v>
@@ -25391,7 +25394,7 @@
         <v>2021</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>2034</v>
@@ -25731,7 +25734,7 @@
         <v>2021</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>2525</v>
+        <v>2524</v>
       </c>
       <c r="E72" s="3" t="s">
         <v>2515</v>
@@ -25870,7 +25873,7 @@
         <v>2021</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="E80" s="3" t="s">
         <v>2042</v>
@@ -25888,7 +25891,7 @@
         <v>2021</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>2542</v>
+        <v>2541</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>2042</v>
@@ -25920,7 +25923,7 @@
         <v>2021</v>
       </c>
       <c r="D83" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>2422</v>
@@ -25953,7 +25956,7 @@
         <v>2021</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>2041</v>
@@ -25971,7 +25974,7 @@
         <v>2021</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>2041</v>
@@ -26025,7 +26028,7 @@
         <v>2021</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>2055</v>
@@ -26130,7 +26133,7 @@
         <v>2021</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
       <c r="E95" s="3" t="s">
         <v>2034</v>
@@ -26638,7 +26641,7 @@
         <v>2057</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>2537</v>
+        <v>2536</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>2089</v>
@@ -26958,7 +26961,7 @@
         <v>2057</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>2112</v>
@@ -27511,7 +27514,7 @@
         <v>2057</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>2531</v>
+        <v>2530</v>
       </c>
       <c r="G57" s="9"/>
       <c r="H57" s="9"/>
@@ -27910,7 +27913,7 @@
         <v>2057</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>2534</v>
+        <v>2533</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>2096</v>
@@ -27950,7 +27953,7 @@
         <v>2057</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>2573</v>
+        <v>2572</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>2181</v>
@@ -28049,7 +28052,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -28655,6 +28658,39 @@
         <v>964</v>
       </c>
       <c r="D43" s="1"/>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>2438</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>2575</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="6" t="s">
+        <v>2118</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>964</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D43"/>
@@ -28689,7 +28725,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2035</v>
@@ -28731,7 +28767,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>2538</v>
+        <v>2537</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>2514</v>
@@ -28799,10 +28835,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
+        <v>2576</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>2522</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>2523</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>2019</v>
@@ -28823,7 +28859,7 @@
         <v>2205</v>
       </c>
       <c r="F11" t="s">
-        <v>2535</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -28852,10 +28888,10 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
+        <v>2531</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>2532</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>2533</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>2232</v>
@@ -29100,7 +29136,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1" t="s">
-        <v>2524</v>
+        <v>2523</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>2252</v>
@@ -29254,7 +29290,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1" t="s">
-        <v>2536</v>
+        <v>2535</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>2281</v>
@@ -29573,7 +29609,7 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>2181</v>

</xml_diff>

<commit_message>
feat: update config dan master
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5288" uniqueCount="2590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5304" uniqueCount="2599">
   <si>
     <t>part_used</t>
   </si>
@@ -7806,6 +7806,33 @@
   </si>
   <si>
     <t>30446005652+</t>
+  </si>
+  <si>
+    <t>9TAHJ6000CP001</t>
+  </si>
+  <si>
+    <t>9TAHL6500CP005</t>
+  </si>
+  <si>
+    <t>9TAHL6500IP002</t>
+  </si>
+  <si>
+    <t>BQC-PWR3243G/L</t>
+  </si>
+  <si>
+    <t>BQC-PWR32GH/L</t>
+  </si>
+  <si>
+    <t>KSETLA984WJN1</t>
+  </si>
+  <si>
+    <t>KSETLB463WJZZ</t>
+  </si>
+  <si>
+    <t>KSETLB467WJZZ</t>
+  </si>
+  <si>
+    <t>IR_WIRE</t>
   </si>
 </sst>
 </file>
@@ -8267,7 +8294,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1843"/>
+  <dimension ref="A1:B1851"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -23016,6 +23043,70 @@
       </c>
       <c r="B1843" s="7" t="s">
         <v>1875</v>
+      </c>
+    </row>
+    <row r="1844" spans="1:2">
+      <c r="A1844" t="s">
+        <v>2590</v>
+      </c>
+      <c r="B1844" s="7" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="1845" spans="1:2">
+      <c r="A1845" t="s">
+        <v>2591</v>
+      </c>
+      <c r="B1845" s="1" t="s">
+        <v>1826</v>
+      </c>
+    </row>
+    <row r="1846" spans="1:2">
+      <c r="A1846" t="s">
+        <v>2592</v>
+      </c>
+      <c r="B1846" s="7" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="1847" spans="1:2">
+      <c r="A1847" t="s">
+        <v>2593</v>
+      </c>
+      <c r="B1847" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="1848" spans="1:2">
+      <c r="A1848" t="s">
+        <v>2594</v>
+      </c>
+      <c r="B1848" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="1849" spans="1:2">
+      <c r="A1849" t="s">
+        <v>2595</v>
+      </c>
+      <c r="B1849" s="7" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="1850" spans="1:2">
+      <c r="A1850" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B1850" s="7" t="s">
+        <v>2598</v>
+      </c>
+    </row>
+    <row r="1851" spans="1:2">
+      <c r="A1851" t="s">
+        <v>2597</v>
+      </c>
+      <c r="B1851" s="7" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance step priorities and add new parts signatures in monthly report recipe
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\Project Applications\tool-fcost\masters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARISAFARI\Works\FQMS - Sharp Confidential\01_MASTER\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5568" uniqueCount="2669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5587" uniqueCount="2676">
   <si>
     <t>part_used</t>
   </si>
@@ -8044,6 +8044,27 @@
   </si>
   <si>
     <t>SUBT|SUBTITUSI|SUBSTITUSI|TKR|TUKAR|PENARIKAN DAN PENGANTARAN|SUBS|SUB</t>
+  </si>
+  <si>
+    <t>30446005402MTC</t>
+  </si>
+  <si>
+    <t>30449605504MTC</t>
+  </si>
+  <si>
+    <t>513YST5461A</t>
+  </si>
+  <si>
+    <t>531A750D001</t>
+  </si>
+  <si>
+    <t>9TAHN7000CP001</t>
+  </si>
+  <si>
+    <t>2TC45BG1X</t>
+  </si>
+  <si>
+    <t>4TC80CL1X</t>
   </si>
 </sst>
 </file>
@@ -8819,7 +8840,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1889"/>
+  <dimension ref="A1:C1894"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -24033,6 +24054,46 @@
       </c>
       <c r="B1889" s="1" t="s">
         <v>459</v>
+      </c>
+    </row>
+    <row r="1890" spans="1:2">
+      <c r="A1890" t="s">
+        <v>2669</v>
+      </c>
+      <c r="B1890" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:2">
+      <c r="A1891" t="s">
+        <v>2670</v>
+      </c>
+      <c r="B1891" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="1892" spans="1:2">
+      <c r="A1892" t="s">
+        <v>2671</v>
+      </c>
+      <c r="B1892" s="1" t="s">
+        <v>1826</v>
+      </c>
+    </row>
+    <row r="1893" spans="1:2">
+      <c r="A1893" t="s">
+        <v>2672</v>
+      </c>
+      <c r="B1893" s="1" t="s">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="1894" spans="1:2">
+      <c r="A1894" t="s">
+        <v>2673</v>
+      </c>
+      <c r="B1894" s="1" t="s">
+        <v>1429</v>
       </c>
     </row>
   </sheetData>
@@ -24090,7 +24151,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C151"/>
+  <dimension ref="A1:C154"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -25757,6 +25818,39 @@
       </c>
       <c r="C151" s="16" t="s">
         <v>2666</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3">
+      <c r="A152" t="s">
+        <v>2674</v>
+      </c>
+      <c r="B152" t="s">
+        <v>2450</v>
+      </c>
+      <c r="C152" t="s">
+        <v>2674</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3">
+      <c r="A153" t="s">
+        <v>2675</v>
+      </c>
+      <c r="B153" t="s">
+        <v>2450</v>
+      </c>
+      <c r="C153" t="s">
+        <v>2675</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3">
+      <c r="A154" t="s">
+        <v>2675</v>
+      </c>
+      <c r="B154" t="s">
+        <v>2450</v>
+      </c>
+      <c r="C154" t="s">
+        <v>2675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
doc: update master table dan sample file excel
</commit_message>
<xml_diff>
--- a/masters/master_table.xlsx
+++ b/masters/master_table.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="part_list" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5587" uniqueCount="2676">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5587" uniqueCount="2677">
   <si>
     <t>part_used</t>
   </si>
@@ -7791,9 +7791,6 @@
     <t>Masuk laporan utama</t>
   </si>
   <si>
-    <t>Report_Category</t>
-  </si>
-  <si>
     <t>BQC-PWR32GH/L</t>
   </si>
   <si>
@@ -8065,6 +8062,12 @@
   </si>
   <si>
     <t>4TC80CL1X</t>
+  </si>
+  <si>
+    <t>REINSERT_LVDS</t>
+  </si>
+  <si>
+    <t>Defect Detail</t>
   </si>
 </sst>
 </file>
@@ -8555,7 +8558,7 @@
     <tableColumn id="2" name="Category" dataDxfId="4"/>
     <tableColumn id="3" name="Defect" dataDxfId="3"/>
     <tableColumn id="4" name="Code" dataDxfId="2"/>
-    <tableColumn id="5" name="Report_Category" dataDxfId="1"/>
+    <tableColumn id="5" name="Defect Detail" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12053,7 +12056,7 @@
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="B401" s="1" t="s">
         <v>459</v>
@@ -12157,7 +12160,7 @@
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="B414" s="1" t="s">
         <v>1826</v>
@@ -12229,7 +12232,7 @@
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
       <c r="B423" s="1" t="s">
         <v>1429</v>
@@ -13389,7 +13392,7 @@
     </row>
     <row r="568" spans="1:2">
       <c r="A568" t="s">
-        <v>2586</v>
+        <v>2585</v>
       </c>
       <c r="B568" s="1" t="s">
         <v>1398</v>
@@ -13405,7 +13408,7 @@
     </row>
     <row r="570" spans="1:2">
       <c r="A570" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
       <c r="B570" s="1" t="s">
         <v>1398</v>
@@ -17805,7 +17808,7 @@
     </row>
     <row r="1120" spans="1:2">
       <c r="A1120" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
       <c r="B1120" s="1" t="s">
         <v>989</v>
@@ -18181,15 +18184,15 @@
     </row>
     <row r="1167" spans="1:2">
       <c r="A1167" t="s">
+        <v>2591</v>
+      </c>
+      <c r="B1167" t="s">
         <v>2592</v>
-      </c>
-      <c r="B1167" t="s">
-        <v>2593</v>
       </c>
     </row>
     <row r="1168" spans="1:2">
       <c r="A1168" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
       <c r="B1168" s="1" t="s">
         <v>3</v>
@@ -23229,7 +23232,7 @@
     </row>
     <row r="1798" spans="1:2">
       <c r="A1798" t="s">
-        <v>2594</v>
+        <v>2593</v>
       </c>
       <c r="B1798" t="s">
         <v>214</v>
@@ -23669,293 +23672,293 @@
     </row>
     <row r="1853" spans="1:3">
       <c r="A1853" s="15" t="s">
+        <v>2602</v>
+      </c>
+      <c r="B1853" s="15" t="s">
+        <v>989</v>
+      </c>
+      <c r="C1853" t="s">
         <v>2603</v>
-      </c>
-      <c r="B1853" s="15" t="s">
-        <v>989</v>
-      </c>
-      <c r="C1853" t="s">
-        <v>2604</v>
       </c>
     </row>
     <row r="1854" spans="1:3">
       <c r="A1854" s="15" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="B1854" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1854" t="s">
-        <v>2604</v>
+        <v>2603</v>
       </c>
     </row>
     <row r="1855" spans="1:3">
       <c r="A1855" s="15" t="s">
+        <v>2605</v>
+      </c>
+      <c r="B1855" s="15" t="s">
+        <v>989</v>
+      </c>
+      <c r="C1855" t="s">
         <v>2606</v>
-      </c>
-      <c r="B1855" s="15" t="s">
-        <v>989</v>
-      </c>
-      <c r="C1855" t="s">
-        <v>2607</v>
       </c>
     </row>
     <row r="1856" spans="1:3">
       <c r="A1856" s="15" t="s">
-        <v>2608</v>
+        <v>2607</v>
       </c>
       <c r="B1856" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1856" t="s">
-        <v>2607</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="1857" spans="1:3">
       <c r="A1857" s="15" t="s">
+        <v>2608</v>
+      </c>
+      <c r="B1857" s="15" t="s">
+        <v>989</v>
+      </c>
+      <c r="C1857" t="s">
         <v>2609</v>
-      </c>
-      <c r="B1857" s="15" t="s">
-        <v>989</v>
-      </c>
-      <c r="C1857" t="s">
-        <v>2610</v>
       </c>
     </row>
     <row r="1858" spans="1:3">
       <c r="A1858" s="15" t="s">
-        <v>2611</v>
+        <v>2610</v>
       </c>
       <c r="B1858" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1858" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="1859" spans="1:3">
       <c r="A1859" s="15" t="s">
-        <v>2613</v>
+        <v>2612</v>
       </c>
       <c r="B1859" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1859" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="1860" spans="1:3">
       <c r="A1860" s="15" t="s">
-        <v>2614</v>
+        <v>2613</v>
       </c>
       <c r="B1860" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1860" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="1861" spans="1:3">
       <c r="A1861" s="15" t="s">
-        <v>2615</v>
+        <v>2614</v>
       </c>
       <c r="B1861" s="15" t="s">
         <v>1429</v>
       </c>
       <c r="C1861" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="1862" spans="1:3">
       <c r="A1862" s="15" t="s">
-        <v>2617</v>
+        <v>2616</v>
       </c>
       <c r="B1862" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1862" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="1863" spans="1:3">
       <c r="A1863" s="15" t="s">
-        <v>2618</v>
+        <v>2617</v>
       </c>
       <c r="B1863" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1863" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="1864" spans="1:3">
       <c r="A1864" s="15" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
       <c r="B1864" s="15" t="s">
         <v>1429</v>
       </c>
       <c r="C1864" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="1865" spans="1:3">
       <c r="A1865" s="15" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="B1865" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1865" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="1866" spans="1:3">
       <c r="A1866" s="15" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
       <c r="B1866" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1866" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="1867" spans="1:3">
       <c r="A1867" s="15" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="B1867" s="15" t="s">
         <v>1429</v>
       </c>
       <c r="C1867" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="1868" spans="1:3">
       <c r="A1868" s="15" t="s">
-        <v>2624</v>
+        <v>2623</v>
       </c>
       <c r="B1868" s="15" t="s">
         <v>1660</v>
       </c>
       <c r="C1868" t="s">
-        <v>2638</v>
+        <v>2637</v>
       </c>
     </row>
     <row r="1869" spans="1:3">
       <c r="A1869" t="s">
+        <v>2624</v>
+      </c>
+      <c r="B1869" s="15" t="s">
+        <v>989</v>
+      </c>
+      <c r="C1869" t="s">
         <v>2625</v>
-      </c>
-      <c r="B1869" s="15" t="s">
-        <v>989</v>
-      </c>
-      <c r="C1869" t="s">
-        <v>2626</v>
       </c>
     </row>
     <row r="1870" spans="1:3">
       <c r="A1870" t="s">
-        <v>2627</v>
+        <v>2626</v>
       </c>
       <c r="B1870" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1870" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="1871" spans="1:3">
       <c r="A1871" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
       <c r="B1871" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1871" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
     </row>
     <row r="1872" spans="1:3">
       <c r="A1872" t="s">
+        <v>2628</v>
+      </c>
+      <c r="B1872" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="C1872" t="s">
         <v>2629</v>
-      </c>
-      <c r="B1872" s="15" t="s">
-        <v>459</v>
-      </c>
-      <c r="C1872" t="s">
-        <v>2630</v>
       </c>
     </row>
     <row r="1873" spans="1:3">
       <c r="A1873" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
       <c r="B1873" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1873" t="s">
-        <v>2633</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="1874" spans="1:3">
       <c r="A1874" t="s">
+        <v>2631</v>
+      </c>
+      <c r="B1874" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="C1874" t="s">
         <v>2632</v>
-      </c>
-      <c r="B1874" s="15" t="s">
-        <v>459</v>
-      </c>
-      <c r="C1874" t="s">
-        <v>2633</v>
       </c>
     </row>
     <row r="1875" spans="1:3">
       <c r="A1875" t="s">
-        <v>2634</v>
+        <v>2633</v>
       </c>
       <c r="B1875" s="15" t="s">
         <v>1429</v>
       </c>
       <c r="C1875" t="s">
-        <v>2633</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="1876" spans="1:3">
       <c r="A1876" t="s">
-        <v>2636</v>
+        <v>2635</v>
       </c>
       <c r="B1876" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1876" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="1877" spans="1:3">
       <c r="A1877" t="s">
-        <v>2637</v>
+        <v>2636</v>
       </c>
       <c r="B1877" s="15" t="s">
         <v>459</v>
       </c>
       <c r="C1877" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="1878" spans="1:3">
       <c r="A1878" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
       <c r="B1878" s="15" t="s">
         <v>1429</v>
       </c>
       <c r="C1878" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="1879" spans="1:3">
       <c r="A1879" t="s">
-        <v>2649</v>
+        <v>2648</v>
       </c>
       <c r="B1879" s="15" t="s">
         <v>459</v>
@@ -23963,7 +23966,7 @@
     </row>
     <row r="1880" spans="1:3">
       <c r="A1880" t="s">
-        <v>2650</v>
+        <v>2649</v>
       </c>
       <c r="B1880" s="15" t="s">
         <v>989</v>
@@ -23971,29 +23974,29 @@
     </row>
     <row r="1881" spans="1:3">
       <c r="A1881" t="s">
-        <v>2651</v>
+        <v>2650</v>
       </c>
       <c r="B1881" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1881" t="s">
-        <v>2658</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="1882" spans="1:3">
       <c r="A1882" t="s">
-        <v>2652</v>
+        <v>2651</v>
       </c>
       <c r="B1882" s="15" t="s">
         <v>989</v>
       </c>
       <c r="C1882" t="s">
-        <v>2659</v>
+        <v>2658</v>
       </c>
     </row>
     <row r="1883" spans="1:3">
       <c r="A1883" t="s">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="B1883" s="1" t="s">
         <v>1398</v>
@@ -24001,10 +24004,10 @@
     </row>
     <row r="1884" spans="1:3">
       <c r="A1884" t="s">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="B1884" s="1" t="s">
-        <v>2660</v>
+        <v>2659</v>
       </c>
       <c r="C1884" t="s">
         <v>2013</v>
@@ -24012,10 +24015,10 @@
     </row>
     <row r="1885" spans="1:3">
       <c r="A1885" t="s">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="B1885" s="1" t="s">
-        <v>2660</v>
+        <v>2659</v>
       </c>
       <c r="C1885" t="s">
         <v>2013</v>
@@ -24023,7 +24026,7 @@
     </row>
     <row r="1886" spans="1:3">
       <c r="A1886" t="s">
-        <v>2656</v>
+        <v>2655</v>
       </c>
       <c r="B1886" s="1" t="s">
         <v>989</v>
@@ -24034,7 +24037,7 @@
     </row>
     <row r="1887" spans="1:3">
       <c r="A1887" t="s">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="B1887" s="1" t="s">
         <v>90</v>
@@ -24042,7 +24045,7 @@
     </row>
     <row r="1888" spans="1:3">
       <c r="A1888" t="s">
-        <v>2661</v>
+        <v>2660</v>
       </c>
       <c r="B1888" s="1" t="s">
         <v>989</v>
@@ -24050,7 +24053,7 @@
     </row>
     <row r="1889" spans="1:2">
       <c r="A1889" t="s">
-        <v>2662</v>
+        <v>2661</v>
       </c>
       <c r="B1889" s="1" t="s">
         <v>459</v>
@@ -24058,7 +24061,7 @@
     </row>
     <row r="1890" spans="1:2">
       <c r="A1890" t="s">
-        <v>2669</v>
+        <v>2668</v>
       </c>
       <c r="B1890" s="1" t="s">
         <v>90</v>
@@ -24066,7 +24069,7 @@
     </row>
     <row r="1891" spans="1:2">
       <c r="A1891" t="s">
-        <v>2670</v>
+        <v>2669</v>
       </c>
       <c r="B1891" s="1" t="s">
         <v>90</v>
@@ -24074,7 +24077,7 @@
     </row>
     <row r="1892" spans="1:2">
       <c r="A1892" t="s">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="B1892" s="1" t="s">
         <v>1826</v>
@@ -24082,7 +24085,7 @@
     </row>
     <row r="1893" spans="1:2">
       <c r="A1893" t="s">
-        <v>2672</v>
+        <v>2671</v>
       </c>
       <c r="B1893" s="1" t="s">
         <v>1655</v>
@@ -24090,7 +24093,7 @@
     </row>
     <row r="1894" spans="1:2">
       <c r="A1894" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="B1894" s="1" t="s">
         <v>1429</v>
@@ -25580,205 +25583,205 @@
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="B130" t="s">
         <v>1961</v>
       </c>
       <c r="C130" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>2596</v>
+        <v>2595</v>
       </c>
       <c r="B131" t="s">
         <v>1961</v>
       </c>
       <c r="C131" t="s">
-        <v>2596</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>2597</v>
+        <v>2596</v>
       </c>
       <c r="B132" t="s">
         <v>2450</v>
       </c>
       <c r="C132" t="s">
-        <v>2597</v>
+        <v>2596</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>2598</v>
+        <v>2597</v>
       </c>
       <c r="B133" t="s">
         <v>2450</v>
       </c>
       <c r="C133" t="s">
-        <v>2598</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="B134" t="s">
         <v>2450</v>
       </c>
       <c r="C134" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="B135" t="s">
         <v>2450</v>
       </c>
       <c r="C135" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>2601</v>
+        <v>2600</v>
       </c>
       <c r="B136" t="s">
         <v>2450</v>
       </c>
       <c r="C136" t="s">
-        <v>2601</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>2602</v>
+        <v>2601</v>
       </c>
       <c r="B137" t="s">
         <v>1961</v>
       </c>
       <c r="C137" t="s">
-        <v>2602</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>2640</v>
+        <v>2639</v>
       </c>
       <c r="B138" t="s">
         <v>2014</v>
       </c>
       <c r="C138" t="s">
-        <v>2640</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
       <c r="B139" t="s">
         <v>2014</v>
       </c>
       <c r="C139" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>2641</v>
+        <v>2640</v>
       </c>
       <c r="B140" t="s">
         <v>2014</v>
       </c>
       <c r="C140" t="s">
-        <v>2641</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>2642</v>
+        <v>2641</v>
       </c>
       <c r="B141" t="s">
         <v>2014</v>
       </c>
       <c r="C141" t="s">
-        <v>2642</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>2643</v>
+        <v>2642</v>
       </c>
       <c r="B142" t="s">
         <v>2014</v>
       </c>
       <c r="C142" t="s">
-        <v>2643</v>
+        <v>2642</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>2644</v>
+        <v>2643</v>
       </c>
       <c r="B143" t="s">
         <v>2014</v>
       </c>
       <c r="C143" t="s">
-        <v>2644</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="B144" t="s">
         <v>2014</v>
       </c>
       <c r="C144" t="s">
-        <v>2645</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>2646</v>
+        <v>2645</v>
       </c>
       <c r="B145" t="s">
         <v>2014</v>
       </c>
       <c r="C145" t="s">
-        <v>2646</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>2647</v>
+        <v>2646</v>
       </c>
       <c r="B146" t="s">
         <v>2014</v>
       </c>
       <c r="C146" t="s">
-        <v>2647</v>
+        <v>2646</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>2648</v>
+        <v>2647</v>
       </c>
       <c r="B147" t="s">
         <v>2014</v>
       </c>
       <c r="C147" t="s">
-        <v>2648</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" s="16" t="s">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="B148" t="s">
         <v>1961</v>
@@ -25789,7 +25792,7 @@
     </row>
     <row r="149" spans="1:3">
       <c r="A149" s="16" t="s">
-        <v>2664</v>
+        <v>2663</v>
       </c>
       <c r="B149" t="s">
         <v>1961</v>
@@ -25800,57 +25803,57 @@
     </row>
     <row r="150" spans="1:3">
       <c r="A150" s="16" t="s">
-        <v>2665</v>
+        <v>2664</v>
       </c>
       <c r="B150" t="s">
         <v>1961</v>
       </c>
       <c r="C150" s="16" t="s">
-        <v>2667</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" s="16" t="s">
-        <v>2666</v>
+        <v>2665</v>
       </c>
       <c r="B151" t="s">
         <v>1961</v>
       </c>
       <c r="C151" s="16" t="s">
-        <v>2666</v>
+        <v>2665</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>2674</v>
+        <v>2673</v>
       </c>
       <c r="B152" t="s">
         <v>2450</v>
       </c>
       <c r="C152" t="s">
-        <v>2674</v>
+        <v>2673</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>2675</v>
+        <v>2674</v>
       </c>
       <c r="B153" t="s">
         <v>2450</v>
       </c>
       <c r="C153" t="s">
-        <v>2675</v>
+        <v>2674</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>2675</v>
+        <v>2674</v>
       </c>
       <c r="B154" t="s">
         <v>2450</v>
       </c>
       <c r="C154" t="s">
-        <v>2675</v>
+        <v>2674</v>
       </c>
     </row>
   </sheetData>
@@ -29401,7 +29404,7 @@
         <v>2057</v>
       </c>
       <c r="E75" t="s">
-        <v>2668</v>
+        <v>2667</v>
       </c>
       <c r="F75" t="s">
         <v>2149</v>
@@ -29551,7 +29554,7 @@
         <v>2130</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>2584</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -29806,7 +29809,7 @@
         <v>60</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>964</v>
+        <v>345</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -29823,7 +29826,7 @@
         <v>61</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>964</v>
+        <v>345</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -29840,7 +29843,7 @@
         <v>62</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>964</v>
+        <v>2675</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -29976,7 +29979,7 @@
         <v>70</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>964</v>
+        <v>989</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -29993,7 +29996,7 @@
         <v>71</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>964</v>
+        <v>989</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -30078,7 +30081,7 @@
         <v>76</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>964</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -30095,7 +30098,7 @@
         <v>77</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>964</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -30248,7 +30251,7 @@
         <v>2</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>2132</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="43" spans="1:5">

</xml_diff>